<commit_message>
chore(reports): nightly refresh 2026-08-07
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -484,7 +484,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>158.46</v>
+        <v>166.92</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -642,7 +642,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -652,30 +652,30 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="G2" t="n">
-        <v>33.95</v>
+        <v>24.99</v>
       </c>
       <c r="H2" t="n">
-        <v>22.63333333333333</v>
+        <v>24.99</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.62475</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -684,14 +684,14 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -701,30 +701,30 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G3" t="n">
-        <v>23.95</v>
+        <v>12.99</v>
       </c>
       <c r="H3" t="n">
-        <v>23.95</v>
+        <v>25.98</v>
       </c>
       <c r="I3" t="n">
-        <v>0.59875</v>
+        <v>0.6495</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -764,16 +764,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>750</v>
+        <v>1500</v>
       </c>
       <c r="G4" t="n">
-        <v>18.5</v>
+        <v>40.4</v>
       </c>
       <c r="H4" t="n">
-        <v>24.66666666666667</v>
+        <v>26.93333333333333</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.6733333333333333</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -799,30 +799,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1000</v>
       </c>
       <c r="G5" t="n">
-        <v>24.99</v>
+        <v>28.5</v>
       </c>
       <c r="H5" t="n">
-        <v>24.99</v>
+        <v>28.5</v>
       </c>
       <c r="I5" t="n">
-        <v>0.62475</v>
+        <v>0.7125</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -862,32 +862,32 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="G6" t="n">
-        <v>12.95</v>
+        <v>22.02</v>
       </c>
       <c r="H6" t="n">
-        <v>25.9</v>
+        <v>29.36</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6475</v>
+        <v>0.734</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -897,30 +897,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G7" t="n">
-        <v>12.95</v>
+        <v>7.49</v>
       </c>
       <c r="H7" t="n">
-        <v>25.9</v>
+        <v>29.96</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6475</v>
+        <v>0.749</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -929,14 +929,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -946,30 +946,30 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>500</v>
       </c>
       <c r="G8" t="n">
-        <v>12.99</v>
+        <v>15.41</v>
       </c>
       <c r="H8" t="n">
-        <v>25.98</v>
+        <v>30.82</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6495</v>
+        <v>0.7705</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -978,14 +978,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -995,39 +995,39 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="G9" t="n">
-        <v>7.49</v>
+        <v>15.93</v>
       </c>
       <c r="H9" t="n">
-        <v>29.96</v>
+        <v>31.86</v>
       </c>
       <c r="I9" t="n">
-        <v>0.749</v>
+        <v>0.7965</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -1061,13 +1061,13 @@
         <v>250</v>
       </c>
       <c r="G10" t="n">
-        <v>7.5</v>
+        <v>8.93</v>
       </c>
       <c r="H10" t="n">
-        <v>30</v>
+        <v>35.72</v>
       </c>
       <c r="I10" t="n">
-        <v>0.75</v>
+        <v>0.893</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1110,13 +1110,13 @@
         <v>400</v>
       </c>
       <c r="G11" t="n">
-        <v>12.5</v>
+        <v>15.38</v>
       </c>
       <c r="H11" t="n">
-        <v>31.25</v>
+        <v>38.45</v>
       </c>
       <c r="I11" t="n">
-        <v>0.78125</v>
+        <v>0.96125</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1159,13 +1159,13 @@
         <v>1000</v>
       </c>
       <c r="G12" t="n">
-        <v>33.95</v>
+        <v>40.4</v>
       </c>
       <c r="H12" t="n">
-        <v>33.95</v>
+        <v>40.4</v>
       </c>
       <c r="I12" t="n">
-        <v>0.84875</v>
+        <v>1.01</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1208,13 +1208,13 @@
         <v>500</v>
       </c>
       <c r="G13" t="n">
-        <v>18.5</v>
+        <v>22.02</v>
       </c>
       <c r="H13" t="n">
-        <v>37</v>
+        <v>44.04</v>
       </c>
       <c r="I13" t="n">
-        <v>0.925</v>
+        <v>1.101</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - citrón limetka</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1254,32 +1254,32 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="G14" t="n">
-        <v>13.95</v>
+        <v>18.98</v>
       </c>
       <c r="H14" t="n">
-        <v>46.5</v>
+        <v>47.45</v>
       </c>
       <c r="I14" t="n">
-        <v>1.1625</v>
+        <v>1.18625</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1289,30 +1289,30 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>14.95</v>
+        <v>4.99</v>
       </c>
       <c r="H15" t="n">
-        <v>49.83333333333334</v>
+        <v>49.9</v>
       </c>
       <c r="I15" t="n">
-        <v>1.245833333333333</v>
+        <v>1.2475</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1321,14 +1321,14 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1338,46 +1338,46 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="G16" t="n">
-        <v>4.99</v>
+        <v>17.16</v>
       </c>
       <c r="H16" t="n">
-        <v>49.9</v>
+        <v>57.2</v>
       </c>
       <c r="I16" t="n">
-        <v>1.2475</v>
+        <v>1.43</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1387,30 +1387,30 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Mixed Berry 1kg</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="G17" t="n">
-        <v>74.98999999999999</v>
+        <v>17.79</v>
       </c>
       <c r="H17" t="n">
-        <v>74.98999999999999</v>
+        <v>59.3</v>
       </c>
       <c r="I17" t="n">
-        <v>1.87475</v>
+        <v>1.4825</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creapure-creatine-monohydrate/bpb-crea-0000</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 500g</t>
+          <t>Creatine Monohydrate (Creapure®️) - Mixed Berry 1kg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1450,16 +1450,16 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G18" t="n">
-        <v>39.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>79.98</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>1.9995</v>
+        <v>1.87475</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1485,37 +1485,86 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 500g</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Bulk</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>500</v>
+      </c>
+      <c r="G19" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="H19" t="n">
+        <v>79.98</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.9995</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>https://www.bulk.com/uk/products/creapure-creatine-monohydrate/bpb-crea-0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>bulk</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>creatine_monohydrate</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Creatine Monohydrate (Creapure®️) - Unflavoured 100g</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Bulk</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F20" t="n">
         <v>100</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G20" t="n">
         <v>9.99</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H20" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I20" t="n">
         <v>2.4975</v>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
         <is>
           <t>https://www.bulk.com/uk/products/creapure-creatine-monohydrate/bpb-crea-0000</t>
         </is>
@@ -1532,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P142"/>
+  <dimension ref="A1:P143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3803,13 +3852,13 @@
         <v>2000</v>
       </c>
       <c r="G46" t="n">
-        <v>104.66</v>
+        <v>87.95</v>
       </c>
       <c r="H46" t="n">
-        <v>52.33</v>
+        <v>43.975</v>
       </c>
       <c r="I46" t="n">
-        <v>1.30825</v>
+        <v>1.099375</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3852,13 +3901,13 @@
         <v>900</v>
       </c>
       <c r="G47" t="n">
-        <v>53.49</v>
+        <v>44.95</v>
       </c>
       <c r="H47" t="n">
-        <v>59.43333333333333</v>
+        <v>49.94444444444444</v>
       </c>
       <c r="I47" t="n">
-        <v>1.485833333333333</v>
+        <v>1.248611111111111</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -6922,7 +6971,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - citrón limetka</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6936,16 +6985,16 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="G110" t="n">
-        <v>33.95</v>
+        <v>18.98</v>
       </c>
       <c r="H110" t="n">
-        <v>33.95</v>
+        <v>47.45</v>
       </c>
       <c r="I110" t="n">
-        <v>0.84875</v>
+        <v>1.18625</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -6954,7 +7003,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6971,7 +7020,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6985,16 +7034,16 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="G111" t="n">
-        <v>14.95</v>
+        <v>40.4</v>
       </c>
       <c r="H111" t="n">
-        <v>49.83333333333334</v>
+        <v>40.4</v>
       </c>
       <c r="I111" t="n">
-        <v>1.245833333333333</v>
+        <v>1.01</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7020,7 +7069,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7034,16 +7083,16 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G112" t="n">
-        <v>18.5</v>
+        <v>17.79</v>
       </c>
       <c r="H112" t="n">
-        <v>37</v>
+        <v>59.3</v>
       </c>
       <c r="I112" t="n">
-        <v>0.925</v>
+        <v>1.4825</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7069,7 +7118,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7086,22 +7135,22 @@
         <v>500</v>
       </c>
       <c r="G113" t="n">
-        <v>12.95</v>
+        <v>22.02</v>
       </c>
       <c r="H113" t="n">
-        <v>25.9</v>
+        <v>44.04</v>
       </c>
       <c r="I113" t="n">
-        <v>0.6475</v>
+        <v>1.101</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7167,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7132,25 +7181,25 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G114" t="n">
-        <v>23.95</v>
+        <v>15.93</v>
       </c>
       <c r="H114" t="n">
-        <v>23.95</v>
+        <v>31.86</v>
       </c>
       <c r="I114" t="n">
-        <v>0.59875</v>
+        <v>0.7965</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7216,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7181,16 +7230,16 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="G115" t="n">
-        <v>33.95</v>
+        <v>28.5</v>
       </c>
       <c r="H115" t="n">
-        <v>22.63333333333333</v>
+        <v>28.5</v>
       </c>
       <c r="I115" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.7125</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7216,7 +7265,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7230,16 +7279,16 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>250</v>
+        <v>1500</v>
       </c>
       <c r="G116" t="n">
-        <v>7.5</v>
+        <v>40.4</v>
       </c>
       <c r="H116" t="n">
-        <v>30</v>
+        <v>26.93333333333333</v>
       </c>
       <c r="I116" t="n">
-        <v>0.75</v>
+        <v>0.6733333333333333</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -7265,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7279,16 +7328,16 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G117" t="n">
-        <v>12.95</v>
+        <v>8.93</v>
       </c>
       <c r="H117" t="n">
-        <v>25.9</v>
+        <v>35.72</v>
       </c>
       <c r="I117" t="n">
-        <v>0.6475</v>
+        <v>0.893</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7314,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7328,16 +7377,16 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="G118" t="n">
-        <v>18.5</v>
+        <v>15.41</v>
       </c>
       <c r="H118" t="n">
-        <v>24.66666666666667</v>
+        <v>30.82</v>
       </c>
       <c r="I118" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.7705</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7363,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7377,25 +7426,25 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="G119" t="n">
-        <v>13.95</v>
+        <v>22.02</v>
       </c>
       <c r="H119" t="n">
-        <v>46.5</v>
+        <v>29.36</v>
       </c>
       <c r="I119" t="n">
-        <v>1.1625</v>
+        <v>0.734</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7412,7 +7461,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7426,16 +7475,16 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G120" t="n">
-        <v>12.5</v>
+        <v>17.16</v>
       </c>
       <c r="H120" t="n">
-        <v>31.25</v>
+        <v>57.2</v>
       </c>
       <c r="I120" t="n">
-        <v>0.78125</v>
+        <v>1.43</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -7444,56 +7493,56 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>protein_works</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>The Protein Works</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="G121" t="n">
-        <v>34.99</v>
+        <v>15.38</v>
       </c>
       <c r="H121" t="n">
-        <v>69.98</v>
+        <v>38.45</v>
       </c>
       <c r="I121" t="n">
-        <v>1.7495</v>
+        <v>0.96125</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
@@ -7524,16 +7573,16 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G122" t="n">
-        <v>61.49</v>
+        <v>34.99</v>
       </c>
       <c r="H122" t="n">
-        <v>61.49</v>
+        <v>69.98</v>
       </c>
       <c r="I122" t="n">
-        <v>1.53725</v>
+        <v>1.7495</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -7573,16 +7622,16 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G123" t="n">
-        <v>111.49</v>
+        <v>61.49</v>
       </c>
       <c r="H123" t="n">
-        <v>55.745</v>
+        <v>61.49</v>
       </c>
       <c r="I123" t="n">
-        <v>1.393625</v>
+        <v>1.53725</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -7622,20 +7671,20 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="G124" t="n">
-        <v>214.99</v>
+        <v>111.49</v>
       </c>
       <c r="H124" t="n">
-        <v>53.7475</v>
+        <v>55.745</v>
       </c>
       <c r="I124" t="n">
-        <v>1.3436875</v>
+        <v>1.393625</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -7657,7 +7706,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -7671,25 +7720,25 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>500</v>
+        <v>4000</v>
       </c>
       <c r="G125" t="n">
-        <v>23.99</v>
+        <v>214.99</v>
       </c>
       <c r="H125" t="n">
-        <v>47.98</v>
+        <v>53.7475</v>
       </c>
       <c r="I125" t="n">
-        <v>1.1995</v>
+        <v>1.3436875</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7720,16 +7769,16 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G126" t="n">
-        <v>44.99</v>
+        <v>23.99</v>
       </c>
       <c r="H126" t="n">
-        <v>44.99</v>
+        <v>47.98</v>
       </c>
       <c r="I126" t="n">
-        <v>1.12475</v>
+        <v>1.1995</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7755,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7769,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="G127" t="n">
-        <v>15.99</v>
+        <v>44.99</v>
       </c>
       <c r="H127" t="n">
-        <v>26.65</v>
+        <v>44.99</v>
       </c>
       <c r="I127" t="n">
-        <v>0.66625</v>
+        <v>1.12475</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7787,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7818,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="G128" t="n">
-        <v>26.99</v>
+        <v>15.99</v>
       </c>
       <c r="H128" t="n">
-        <v>22.49166666666667</v>
+        <v>26.65</v>
       </c>
       <c r="I128" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.66625</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7867,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>2400</v>
+        <v>1200</v>
       </c>
       <c r="G129" t="n">
-        <v>46.99</v>
+        <v>26.99</v>
       </c>
       <c r="H129" t="n">
-        <v>19.57916666666667</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I129" t="n">
-        <v>0.4894791666666667</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7916,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>4800</v>
+        <v>2400</v>
       </c>
       <c r="G130" t="n">
-        <v>89.98999999999999</v>
+        <v>46.99</v>
       </c>
       <c r="H130" t="n">
-        <v>18.74791666666667</v>
+        <v>19.57916666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.4686979166666667</v>
+        <v>0.4894791666666667</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7965,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>600</v>
+        <v>4800</v>
       </c>
       <c r="G131" t="n">
-        <v>16.99</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="H131" t="n">
-        <v>28.31666666666667</v>
+        <v>18.74791666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.4686979166666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -7983,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8014,16 +8063,16 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="G132" t="n">
-        <v>28.99</v>
+        <v>16.99</v>
       </c>
       <c r="H132" t="n">
-        <v>24.15833333333333</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I132" t="n">
-        <v>0.6039583333333334</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8063,16 +8112,16 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>2400</v>
+        <v>1200</v>
       </c>
       <c r="G133" t="n">
-        <v>46.99</v>
+        <v>28.99</v>
       </c>
       <c r="H133" t="n">
-        <v>19.57916666666667</v>
+        <v>24.15833333333333</v>
       </c>
       <c r="I133" t="n">
-        <v>0.4894791666666667</v>
+        <v>0.6039583333333334</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8112,16 +8161,16 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>4800</v>
+        <v>2400</v>
       </c>
       <c r="G134" t="n">
-        <v>89.98999999999999</v>
+        <v>46.99</v>
       </c>
       <c r="H134" t="n">
-        <v>18.74791666666667</v>
+        <v>19.57916666666667</v>
       </c>
       <c r="I134" t="n">
-        <v>0.4686979166666667</v>
+        <v>0.4894791666666667</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8147,7 +8196,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8161,16 +8210,16 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>500</v>
+        <v>4800</v>
       </c>
       <c r="G135" t="n">
-        <v>20.99</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="H135" t="n">
-        <v>41.98</v>
+        <v>18.74791666666667</v>
       </c>
       <c r="I135" t="n">
-        <v>1.0495</v>
+        <v>0.4686979166666667</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8179,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8210,16 +8259,16 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G136" t="n">
-        <v>36.99</v>
+        <v>20.99</v>
       </c>
       <c r="H136" t="n">
-        <v>36.99</v>
+        <v>41.98</v>
       </c>
       <c r="I136" t="n">
-        <v>0.92475</v>
+        <v>1.0495</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8259,16 +8308,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G137" t="n">
-        <v>70.98999999999999</v>
+        <v>36.99</v>
       </c>
       <c r="H137" t="n">
-        <v>35.495</v>
+        <v>36.99</v>
       </c>
       <c r="I137" t="n">
-        <v>0.887375</v>
+        <v>0.92475</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8308,16 +8357,16 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="G138" t="n">
-        <v>135.99</v>
+        <v>70.98999999999999</v>
       </c>
       <c r="H138" t="n">
-        <v>33.9975</v>
+        <v>35.495</v>
       </c>
       <c r="I138" t="n">
-        <v>0.8499375</v>
+        <v>0.887375</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8343,7 +8392,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Whey Protein 360 - Vanilla</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8357,16 +8406,16 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>600</v>
+        <v>4000</v>
       </c>
       <c r="G139" t="n">
-        <v>12.99</v>
+        <v>135.99</v>
       </c>
       <c r="H139" t="n">
-        <v>21.65</v>
+        <v>33.9975</v>
       </c>
       <c r="I139" t="n">
-        <v>0.54125</v>
+        <v>0.8499375</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8375,7 +8424,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8406,16 +8455,16 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="G140" t="n">
-        <v>22.99</v>
+        <v>12.99</v>
       </c>
       <c r="H140" t="n">
-        <v>19.15833333333333</v>
+        <v>21.65</v>
       </c>
       <c r="I140" t="n">
-        <v>0.4789583333333333</v>
+        <v>0.54125</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8455,16 +8504,16 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>2400</v>
+        <v>1200</v>
       </c>
       <c r="G141" t="n">
-        <v>39.99</v>
+        <v>22.99</v>
       </c>
       <c r="H141" t="n">
-        <v>16.6625</v>
+        <v>19.15833333333333</v>
       </c>
       <c r="I141" t="n">
-        <v>0.4165625</v>
+        <v>0.4789583333333333</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8504,23 +8553,72 @@
         </is>
       </c>
       <c r="F142" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G142" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="H142" t="n">
+        <v>16.6625</v>
+      </c>
+      <c r="I142" t="n">
+        <v>0.4165625</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>protein_works</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>whey_protein</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Whey Protein 360 - Vanilla</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>The Protein Works</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
         <v>4800</v>
       </c>
-      <c r="G142" t="n">
+      <c r="G143" t="n">
         <v>76.98999999999999</v>
       </c>
-      <c r="H142" t="n">
+      <c r="H143" t="n">
         <v>16.03958333333333</v>
       </c>
-      <c r="I142" t="n">
+      <c r="I143" t="n">
         <v>0.4009895833333333</v>
       </c>
-      <c r="O142" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P142" t="inlineStr">
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
         <is>
           <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-08
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -461,7 +461,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>136.42</v>
+        <v>143.48</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>166.92</v>
+        <v>158.46</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -652,30 +652,30 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G2" t="n">
-        <v>24.99</v>
+        <v>33.95</v>
       </c>
       <c r="H2" t="n">
-        <v>24.99</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I2" t="n">
-        <v>0.62475</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -684,14 +684,14 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -701,30 +701,30 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G3" t="n">
-        <v>12.99</v>
+        <v>23.95</v>
       </c>
       <c r="H3" t="n">
-        <v>25.98</v>
+        <v>23.95</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6495</v>
+        <v>0.59875</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -764,16 +764,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="G4" t="n">
-        <v>40.4</v>
+        <v>18.5</v>
       </c>
       <c r="H4" t="n">
-        <v>26.93333333333333</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -799,30 +799,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1000</v>
       </c>
       <c r="G5" t="n">
-        <v>28.5</v>
+        <v>24.99</v>
       </c>
       <c r="H5" t="n">
-        <v>28.5</v>
+        <v>24.99</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7125</v>
+        <v>0.62475</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -862,32 +862,32 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="G6" t="n">
-        <v>22.02</v>
+        <v>12.95</v>
       </c>
       <c r="H6" t="n">
-        <v>29.36</v>
+        <v>25.9</v>
       </c>
       <c r="I6" t="n">
-        <v>0.734</v>
+        <v>0.6475</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -897,30 +897,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="G7" t="n">
-        <v>7.49</v>
+        <v>12.95</v>
       </c>
       <c r="H7" t="n">
-        <v>29.96</v>
+        <v>25.9</v>
       </c>
       <c r="I7" t="n">
-        <v>0.749</v>
+        <v>0.6475</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -929,14 +929,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -946,30 +946,30 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>500</v>
       </c>
       <c r="G8" t="n">
-        <v>15.41</v>
+        <v>12.99</v>
       </c>
       <c r="H8" t="n">
-        <v>30.82</v>
+        <v>25.98</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7705</v>
+        <v>0.6495</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -978,14 +978,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -995,39 +995,39 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G9" t="n">
-        <v>15.93</v>
+        <v>7.49</v>
       </c>
       <c r="H9" t="n">
-        <v>31.86</v>
+        <v>29.96</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7965</v>
+        <v>0.749</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -1061,13 +1061,13 @@
         <v>250</v>
       </c>
       <c r="G10" t="n">
-        <v>8.93</v>
+        <v>7.5</v>
       </c>
       <c r="H10" t="n">
-        <v>35.72</v>
+        <v>30</v>
       </c>
       <c r="I10" t="n">
-        <v>0.893</v>
+        <v>0.75</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1110,13 +1110,13 @@
         <v>400</v>
       </c>
       <c r="G11" t="n">
-        <v>15.38</v>
+        <v>12.5</v>
       </c>
       <c r="H11" t="n">
-        <v>38.45</v>
+        <v>31.25</v>
       </c>
       <c r="I11" t="n">
-        <v>0.96125</v>
+        <v>0.78125</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1159,13 +1159,13 @@
         <v>1000</v>
       </c>
       <c r="G12" t="n">
-        <v>40.4</v>
+        <v>33.95</v>
       </c>
       <c r="H12" t="n">
-        <v>40.4</v>
+        <v>33.95</v>
       </c>
       <c r="I12" t="n">
-        <v>1.01</v>
+        <v>0.84875</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1208,13 +1208,13 @@
         <v>500</v>
       </c>
       <c r="G13" t="n">
-        <v>22.02</v>
+        <v>18.5</v>
       </c>
       <c r="H13" t="n">
-        <v>44.04</v>
+        <v>37</v>
       </c>
       <c r="I13" t="n">
-        <v>1.101</v>
+        <v>0.925</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1257,13 +1257,13 @@
         <v>400</v>
       </c>
       <c r="G14" t="n">
-        <v>18.98</v>
+        <v>15.95</v>
       </c>
       <c r="H14" t="n">
-        <v>47.45</v>
+        <v>39.875</v>
       </c>
       <c r="I14" t="n">
-        <v>1.18625</v>
+        <v>0.996875</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1279,7 +1279,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1289,39 +1289,39 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="G15" t="n">
-        <v>4.99</v>
+        <v>13.95</v>
       </c>
       <c r="H15" t="n">
-        <v>49.9</v>
+        <v>46.5</v>
       </c>
       <c r="I15" t="n">
-        <v>1.2475</v>
+        <v>1.1625</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1355,29 +1355,29 @@
         <v>300</v>
       </c>
       <c r="G16" t="n">
-        <v>17.16</v>
+        <v>14.95</v>
       </c>
       <c r="H16" t="n">
-        <v>57.2</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I16" t="n">
-        <v>1.43</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1387,30 +1387,30 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>17.79</v>
+        <v>4.99</v>
       </c>
       <c r="H17" t="n">
-        <v>59.3</v>
+        <v>49.9</v>
       </c>
       <c r="I17" t="n">
-        <v>1.4825</v>
+        <v>1.2475</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Mixed Berry 1kg</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1696,13 +1696,13 @@
         <v>1000</v>
       </c>
       <c r="G2" t="n">
-        <v>27.99</v>
+        <v>29.99</v>
       </c>
       <c r="H2" t="n">
-        <v>27.99</v>
+        <v>29.99</v>
       </c>
       <c r="I2" t="n">
-        <v>0.69975</v>
+        <v>0.74975</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -1745,13 +1745,13 @@
         <v>2500</v>
       </c>
       <c r="G3" t="n">
-        <v>67.98999999999999</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>27.196</v>
+        <v>27.996</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6798999999999999</v>
+        <v>0.6999</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -1794,13 +1794,13 @@
         <v>5000</v>
       </c>
       <c r="G4" t="n">
-        <v>129.99</v>
+        <v>134.99</v>
       </c>
       <c r="H4" t="n">
-        <v>25.998</v>
+        <v>26.998</v>
       </c>
       <c r="I4" t="n">
-        <v>0.64995</v>
+        <v>0.67495</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -1843,13 +1843,13 @@
         <v>500</v>
       </c>
       <c r="G5" t="n">
-        <v>15.99</v>
+        <v>16.99</v>
       </c>
       <c r="H5" t="n">
-        <v>31.98</v>
+        <v>33.98</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7995</v>
+        <v>0.8495</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1892,13 +1892,13 @@
         <v>1000</v>
       </c>
       <c r="G6" t="n">
-        <v>41.99</v>
+        <v>44.99</v>
       </c>
       <c r="H6" t="n">
-        <v>41.99</v>
+        <v>44.99</v>
       </c>
       <c r="I6" t="n">
-        <v>1.04975</v>
+        <v>1.12475</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1941,13 +1941,13 @@
         <v>2500</v>
       </c>
       <c r="G7" t="n">
-        <v>94.98999999999999</v>
+        <v>104.99</v>
       </c>
       <c r="H7" t="n">
-        <v>37.996</v>
+        <v>41.996</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9499</v>
+        <v>1.0499</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1990,13 +1990,13 @@
         <v>5000</v>
       </c>
       <c r="G8" t="n">
-        <v>184.99</v>
+        <v>199.99</v>
       </c>
       <c r="H8" t="n">
-        <v>36.998</v>
+        <v>39.998</v>
       </c>
       <c r="I8" t="n">
-        <v>0.92495</v>
+        <v>0.99995</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -2039,13 +2039,13 @@
         <v>500</v>
       </c>
       <c r="G9" t="n">
-        <v>23.99</v>
+        <v>24.99</v>
       </c>
       <c r="H9" t="n">
-        <v>47.98</v>
+        <v>49.98</v>
       </c>
       <c r="I9" t="n">
-        <v>1.1995</v>
+        <v>1.2495</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2085,16 +2085,16 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2270</v>
+        <v>500</v>
       </c>
       <c r="G10" t="n">
-        <v>79.98999999999999</v>
+        <v>16.99</v>
       </c>
       <c r="H10" t="n">
-        <v>35.23788546255506</v>
+        <v>33.98</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8809471365638767</v>
+        <v>0.8495</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2134,16 +2134,16 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G11" t="n">
-        <v>16.99</v>
+        <v>31.99</v>
       </c>
       <c r="H11" t="n">
-        <v>33.98</v>
+        <v>31.99</v>
       </c>
       <c r="I11" t="n">
-        <v>0.8495</v>
+        <v>0.79975</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2183,16 +2183,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G12" t="n">
-        <v>31.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>31.99</v>
+        <v>29.996</v>
       </c>
       <c r="I12" t="n">
-        <v>0.79975</v>
+        <v>0.7499</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2232,16 +2232,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="G13" t="n">
-        <v>74.98999999999999</v>
+        <v>139.99</v>
       </c>
       <c r="H13" t="n">
-        <v>29.996</v>
+        <v>27.998</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7499</v>
+        <v>0.69995</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>5000</v>
+        <v>2270</v>
       </c>
       <c r="G14" t="n">
-        <v>139.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>27.998</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I14" t="n">
-        <v>0.69995</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -2676,13 +2676,13 @@
         <v>500</v>
       </c>
       <c r="G22" t="n">
-        <v>15.99</v>
+        <v>16.99</v>
       </c>
       <c r="H22" t="n">
-        <v>31.98</v>
+        <v>33.98</v>
       </c>
       <c r="I22" t="n">
-        <v>0.7995</v>
+        <v>0.8495</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -3117,13 +3117,13 @@
         <v>1250</v>
       </c>
       <c r="G31" t="n">
-        <v>16.99</v>
+        <v>18.99</v>
       </c>
       <c r="H31" t="n">
-        <v>13.592</v>
+        <v>15.192</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3398</v>
+        <v>0.3798</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3166,13 +3166,13 @@
         <v>2500</v>
       </c>
       <c r="G32" t="n">
-        <v>32.99</v>
+        <v>35.99</v>
       </c>
       <c r="H32" t="n">
-        <v>13.196</v>
+        <v>14.396</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3299</v>
+        <v>0.3599</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Mixed Berry 1kg</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -6988,13 +6988,13 @@
         <v>400</v>
       </c>
       <c r="G110" t="n">
-        <v>18.98</v>
+        <v>15.95</v>
       </c>
       <c r="H110" t="n">
-        <v>47.45</v>
+        <v>39.875</v>
       </c>
       <c r="I110" t="n">
-        <v>1.18625</v>
+        <v>0.996875</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7037,13 +7037,13 @@
         <v>1000</v>
       </c>
       <c r="G111" t="n">
-        <v>40.4</v>
+        <v>33.95</v>
       </c>
       <c r="H111" t="n">
-        <v>40.4</v>
+        <v>33.95</v>
       </c>
       <c r="I111" t="n">
-        <v>1.01</v>
+        <v>0.84875</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7086,13 +7086,13 @@
         <v>300</v>
       </c>
       <c r="G112" t="n">
-        <v>17.79</v>
+        <v>14.95</v>
       </c>
       <c r="H112" t="n">
-        <v>59.3</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I112" t="n">
-        <v>1.4825</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7135,13 +7135,13 @@
         <v>500</v>
       </c>
       <c r="G113" t="n">
-        <v>22.02</v>
+        <v>18.5</v>
       </c>
       <c r="H113" t="n">
-        <v>44.04</v>
+        <v>37</v>
       </c>
       <c r="I113" t="n">
-        <v>1.101</v>
+        <v>0.925</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7184,13 +7184,13 @@
         <v>500</v>
       </c>
       <c r="G114" t="n">
-        <v>15.93</v>
+        <v>12.95</v>
       </c>
       <c r="H114" t="n">
-        <v>31.86</v>
+        <v>25.9</v>
       </c>
       <c r="I114" t="n">
-        <v>0.7965</v>
+        <v>0.6475</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7233,13 +7233,13 @@
         <v>1000</v>
       </c>
       <c r="G115" t="n">
-        <v>28.5</v>
+        <v>23.95</v>
       </c>
       <c r="H115" t="n">
-        <v>28.5</v>
+        <v>23.95</v>
       </c>
       <c r="I115" t="n">
-        <v>0.7125</v>
+        <v>0.59875</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7282,13 +7282,13 @@
         <v>1500</v>
       </c>
       <c r="G116" t="n">
-        <v>40.4</v>
+        <v>33.95</v>
       </c>
       <c r="H116" t="n">
-        <v>26.93333333333333</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I116" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -7331,13 +7331,13 @@
         <v>250</v>
       </c>
       <c r="G117" t="n">
-        <v>8.93</v>
+        <v>7.5</v>
       </c>
       <c r="H117" t="n">
-        <v>35.72</v>
+        <v>30</v>
       </c>
       <c r="I117" t="n">
-        <v>0.893</v>
+        <v>0.75</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7380,13 +7380,13 @@
         <v>500</v>
       </c>
       <c r="G118" t="n">
-        <v>15.41</v>
+        <v>12.95</v>
       </c>
       <c r="H118" t="n">
-        <v>30.82</v>
+        <v>25.9</v>
       </c>
       <c r="I118" t="n">
-        <v>0.7705</v>
+        <v>0.6475</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7429,13 +7429,13 @@
         <v>750</v>
       </c>
       <c r="G119" t="n">
-        <v>22.02</v>
+        <v>18.5</v>
       </c>
       <c r="H119" t="n">
-        <v>29.36</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I119" t="n">
-        <v>0.734</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7478,13 +7478,13 @@
         <v>300</v>
       </c>
       <c r="G120" t="n">
-        <v>17.16</v>
+        <v>13.95</v>
       </c>
       <c r="H120" t="n">
-        <v>57.2</v>
+        <v>46.5</v>
       </c>
       <c r="I120" t="n">
-        <v>1.43</v>
+        <v>1.1625</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -7527,13 +7527,13 @@
         <v>400</v>
       </c>
       <c r="G121" t="n">
-        <v>15.38</v>
+        <v>12.5</v>
       </c>
       <c r="H121" t="n">
-        <v>38.45</v>
+        <v>31.25</v>
       </c>
       <c r="I121" t="n">
-        <v>0.96125</v>
+        <v>0.78125</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-09
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2085,16 +2085,16 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>500</v>
+        <v>2270</v>
       </c>
       <c r="G10" t="n">
-        <v>16.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>33.98</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8495</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2134,16 +2134,16 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G11" t="n">
-        <v>31.99</v>
+        <v>16.99</v>
       </c>
       <c r="H11" t="n">
-        <v>31.99</v>
+        <v>33.98</v>
       </c>
       <c r="I11" t="n">
-        <v>0.79975</v>
+        <v>0.8495</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2183,16 +2183,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G12" t="n">
-        <v>74.98999999999999</v>
+        <v>31.99</v>
       </c>
       <c r="H12" t="n">
-        <v>29.996</v>
+        <v>31.99</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7499</v>
+        <v>0.79975</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2232,16 +2232,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="G13" t="n">
-        <v>139.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>27.998</v>
+        <v>29.996</v>
       </c>
       <c r="I13" t="n">
-        <v>0.69995</v>
+        <v>0.7499</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2270</v>
+        <v>5000</v>
       </c>
       <c r="G14" t="n">
-        <v>79.98999999999999</v>
+        <v>139.99</v>
       </c>
       <c r="H14" t="n">
-        <v>35.23788546255506</v>
+        <v>27.998</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8809471365638767</v>
+        <v>0.69995</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-10
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7769,16 +7769,16 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="G126" t="n">
-        <v>23.99</v>
+        <v>15.99</v>
       </c>
       <c r="H126" t="n">
-        <v>47.98</v>
+        <v>26.65</v>
       </c>
       <c r="I126" t="n">
-        <v>1.1995</v>
+        <v>0.66625</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7818,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="G127" t="n">
-        <v>44.99</v>
+        <v>26.99</v>
       </c>
       <c r="H127" t="n">
-        <v>44.99</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I127" t="n">
-        <v>1.12475</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>600</v>
+        <v>2400</v>
       </c>
       <c r="G128" t="n">
-        <v>15.99</v>
+        <v>46.99</v>
       </c>
       <c r="H128" t="n">
-        <v>26.65</v>
+        <v>19.57916666666667</v>
       </c>
       <c r="I128" t="n">
-        <v>0.66625</v>
+        <v>0.4894791666666667</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>1200</v>
+        <v>4800</v>
       </c>
       <c r="G129" t="n">
-        <v>26.99</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="H129" t="n">
-        <v>22.49166666666667</v>
+        <v>18.74791666666667</v>
       </c>
       <c r="I129" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.4686979166666667</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>2400</v>
+        <v>500</v>
       </c>
       <c r="G130" t="n">
-        <v>46.99</v>
+        <v>23.99</v>
       </c>
       <c r="H130" t="n">
-        <v>19.57916666666667</v>
+        <v>47.98</v>
       </c>
       <c r="I130" t="n">
-        <v>0.4894791666666667</v>
+        <v>1.1995</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8000,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>4800</v>
+        <v>1000</v>
       </c>
       <c r="G131" t="n">
-        <v>89.98999999999999</v>
+        <v>44.99</v>
       </c>
       <c r="H131" t="n">
-        <v>18.74791666666667</v>
+        <v>44.99</v>
       </c>
       <c r="I131" t="n">
-        <v>0.4686979166666667</v>
+        <v>1.12475</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-11
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2085,16 +2085,16 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2270</v>
+        <v>500</v>
       </c>
       <c r="G10" t="n">
-        <v>79.98999999999999</v>
+        <v>16.99</v>
       </c>
       <c r="H10" t="n">
-        <v>35.23788546255506</v>
+        <v>33.98</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8809471365638767</v>
+        <v>0.8495</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2134,16 +2134,16 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G11" t="n">
-        <v>16.99</v>
+        <v>31.99</v>
       </c>
       <c r="H11" t="n">
-        <v>33.98</v>
+        <v>31.99</v>
       </c>
       <c r="I11" t="n">
-        <v>0.8495</v>
+        <v>0.79975</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2183,16 +2183,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G12" t="n">
-        <v>31.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>31.99</v>
+        <v>29.996</v>
       </c>
       <c r="I12" t="n">
-        <v>0.79975</v>
+        <v>0.7499</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2232,16 +2232,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="G13" t="n">
-        <v>74.98999999999999</v>
+        <v>139.99</v>
       </c>
       <c r="H13" t="n">
-        <v>29.996</v>
+        <v>27.998</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7499</v>
+        <v>0.69995</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>5000</v>
+        <v>2270</v>
       </c>
       <c r="G14" t="n">
-        <v>139.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>27.998</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I14" t="n">
-        <v>0.69995</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3016,16 +3016,16 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G29" t="n">
-        <v>19.99</v>
+        <v>18.99</v>
       </c>
       <c r="H29" t="n">
-        <v>39.98</v>
+        <v>15.192</v>
       </c>
       <c r="I29" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.3798</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G30" t="n">
-        <v>37.99</v>
+        <v>35.99</v>
       </c>
       <c r="H30" t="n">
-        <v>37.99</v>
+        <v>14.396</v>
       </c>
       <c r="I30" t="n">
-        <v>0.94975</v>
+        <v>0.3599</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,16 +3114,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G31" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="H31" t="n">
-        <v>15.192</v>
+        <v>39.98</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3798</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G32" t="n">
-        <v>35.99</v>
+        <v>37.99</v>
       </c>
       <c r="H32" t="n">
-        <v>14.396</v>
+        <v>37.99</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3599</v>
+        <v>0.94975</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -7772,13 +7772,13 @@
         <v>600</v>
       </c>
       <c r="G126" t="n">
-        <v>15.99</v>
+        <v>16.99</v>
       </c>
       <c r="H126" t="n">
-        <v>26.65</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I126" t="n">
-        <v>0.66625</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7821,13 +7821,13 @@
         <v>1200</v>
       </c>
       <c r="G127" t="n">
-        <v>26.99</v>
+        <v>28.99</v>
       </c>
       <c r="H127" t="n">
-        <v>22.49166666666667</v>
+        <v>24.15833333333333</v>
       </c>
       <c r="I127" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.6039583333333334</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7870,13 +7870,13 @@
         <v>2400</v>
       </c>
       <c r="G128" t="n">
-        <v>46.99</v>
+        <v>48.99</v>
       </c>
       <c r="H128" t="n">
-        <v>19.57916666666667</v>
+        <v>20.4125</v>
       </c>
       <c r="I128" t="n">
-        <v>0.4894791666666667</v>
+        <v>0.5103124999999999</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7919,13 +7919,13 @@
         <v>4800</v>
       </c>
       <c r="G129" t="n">
-        <v>89.98999999999999</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="H129" t="n">
-        <v>18.74791666666667</v>
+        <v>19.58125</v>
       </c>
       <c r="I129" t="n">
-        <v>0.4686979166666667</v>
+        <v>0.48953125</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -8066,13 +8066,13 @@
         <v>600</v>
       </c>
       <c r="G132" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="H132" t="n">
-        <v>28.31666666666667</v>
+        <v>29.98333333333333</v>
       </c>
       <c r="I132" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.7495833333333334</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8115,13 +8115,13 @@
         <v>1200</v>
       </c>
       <c r="G133" t="n">
-        <v>28.99</v>
+        <v>30.99</v>
       </c>
       <c r="H133" t="n">
-        <v>24.15833333333333</v>
+        <v>25.825</v>
       </c>
       <c r="I133" t="n">
-        <v>0.6039583333333334</v>
+        <v>0.645625</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8164,13 +8164,13 @@
         <v>2400</v>
       </c>
       <c r="G134" t="n">
-        <v>46.99</v>
+        <v>48.99</v>
       </c>
       <c r="H134" t="n">
-        <v>19.57916666666667</v>
+        <v>20.4125</v>
       </c>
       <c r="I134" t="n">
-        <v>0.4894791666666667</v>
+        <v>0.5103124999999999</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8213,13 +8213,13 @@
         <v>4800</v>
       </c>
       <c r="G135" t="n">
-        <v>89.98999999999999</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="H135" t="n">
-        <v>18.74791666666667</v>
+        <v>19.58125</v>
       </c>
       <c r="I135" t="n">
-        <v>0.4686979166666667</v>
+        <v>0.48953125</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8262,13 +8262,13 @@
         <v>500</v>
       </c>
       <c r="G136" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="H136" t="n">
-        <v>41.98</v>
+        <v>43.98</v>
       </c>
       <c r="I136" t="n">
-        <v>1.0495</v>
+        <v>1.0995</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8311,13 +8311,13 @@
         <v>1000</v>
       </c>
       <c r="G137" t="n">
-        <v>36.99</v>
+        <v>38.99</v>
       </c>
       <c r="H137" t="n">
-        <v>36.99</v>
+        <v>38.99</v>
       </c>
       <c r="I137" t="n">
-        <v>0.92475</v>
+        <v>0.97475</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8360,13 +8360,13 @@
         <v>2000</v>
       </c>
       <c r="G138" t="n">
-        <v>70.98999999999999</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="H138" t="n">
-        <v>35.495</v>
+        <v>36.495</v>
       </c>
       <c r="I138" t="n">
-        <v>0.887375</v>
+        <v>0.912375</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8409,13 +8409,13 @@
         <v>4000</v>
       </c>
       <c r="G139" t="n">
-        <v>135.99</v>
+        <v>141.99</v>
       </c>
       <c r="H139" t="n">
-        <v>33.9975</v>
+        <v>35.4975</v>
       </c>
       <c r="I139" t="n">
-        <v>0.8499375</v>
+        <v>0.8874375</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8458,13 +8458,13 @@
         <v>600</v>
       </c>
       <c r="G140" t="n">
-        <v>12.99</v>
+        <v>13.99</v>
       </c>
       <c r="H140" t="n">
-        <v>21.65</v>
+        <v>23.31666666666667</v>
       </c>
       <c r="I140" t="n">
-        <v>0.54125</v>
+        <v>0.5829166666666666</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8507,13 +8507,13 @@
         <v>1200</v>
       </c>
       <c r="G141" t="n">
-        <v>22.99</v>
+        <v>23.99</v>
       </c>
       <c r="H141" t="n">
-        <v>19.15833333333333</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I141" t="n">
-        <v>0.4789583333333333</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8556,13 +8556,13 @@
         <v>2400</v>
       </c>
       <c r="G142" t="n">
-        <v>39.99</v>
+        <v>41.99</v>
       </c>
       <c r="H142" t="n">
-        <v>16.6625</v>
+        <v>17.49583333333333</v>
       </c>
       <c r="I142" t="n">
-        <v>0.4165625</v>
+        <v>0.4373958333333333</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8605,13 +8605,13 @@
         <v>4800</v>
       </c>
       <c r="G143" t="n">
-        <v>76.98999999999999</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H143" t="n">
-        <v>16.03958333333333</v>
+        <v>16.66458333333333</v>
       </c>
       <c r="I143" t="n">
-        <v>0.4009895833333333</v>
+        <v>0.4166145833333333</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-12
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2333,13 +2333,13 @@
         <v>500</v>
       </c>
       <c r="G15" t="n">
-        <v>23.99</v>
+        <v>24.99</v>
       </c>
       <c r="H15" t="n">
-        <v>47.98</v>
+        <v>49.98</v>
       </c>
       <c r="I15" t="n">
-        <v>1.1995</v>
+        <v>1.2495</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -2382,13 +2382,13 @@
         <v>1000</v>
       </c>
       <c r="G16" t="n">
-        <v>41.99</v>
+        <v>44.99</v>
       </c>
       <c r="H16" t="n">
-        <v>41.99</v>
+        <v>44.99</v>
       </c>
       <c r="I16" t="n">
-        <v>1.04975</v>
+        <v>1.12475</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -2431,13 +2431,13 @@
         <v>2500</v>
       </c>
       <c r="G17" t="n">
-        <v>94.98999999999999</v>
+        <v>104.99</v>
       </c>
       <c r="H17" t="n">
-        <v>37.996</v>
+        <v>41.996</v>
       </c>
       <c r="I17" t="n">
-        <v>0.9499</v>
+        <v>1.0499</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2480,13 +2480,13 @@
         <v>5000</v>
       </c>
       <c r="G18" t="n">
-        <v>184.99</v>
+        <v>199.99</v>
       </c>
       <c r="H18" t="n">
-        <v>36.998</v>
+        <v>39.998</v>
       </c>
       <c r="I18" t="n">
-        <v>0.92495</v>
+        <v>0.99995</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7769,16 +7769,16 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="G126" t="n">
-        <v>16.99</v>
+        <v>23.99</v>
       </c>
       <c r="H126" t="n">
-        <v>28.31666666666667</v>
+        <v>47.98</v>
       </c>
       <c r="I126" t="n">
-        <v>0.7079166666666666</v>
+        <v>1.1995</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7818,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="G127" t="n">
-        <v>28.99</v>
+        <v>44.99</v>
       </c>
       <c r="H127" t="n">
-        <v>24.15833333333333</v>
+        <v>44.99</v>
       </c>
       <c r="I127" t="n">
-        <v>0.6039583333333334</v>
+        <v>1.12475</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>2400</v>
+        <v>600</v>
       </c>
       <c r="G128" t="n">
-        <v>48.99</v>
+        <v>17.99</v>
       </c>
       <c r="H128" t="n">
-        <v>20.4125</v>
+        <v>29.98333333333333</v>
       </c>
       <c r="I128" t="n">
-        <v>0.5103124999999999</v>
+        <v>0.7495833333333334</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>4800</v>
+        <v>1200</v>
       </c>
       <c r="G129" t="n">
-        <v>93.98999999999999</v>
+        <v>30.99</v>
       </c>
       <c r="H129" t="n">
-        <v>19.58125</v>
+        <v>25.825</v>
       </c>
       <c r="I129" t="n">
-        <v>0.48953125</v>
+        <v>0.645625</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>500</v>
+        <v>2400</v>
       </c>
       <c r="G130" t="n">
-        <v>23.99</v>
+        <v>48.99</v>
       </c>
       <c r="H130" t="n">
-        <v>47.98</v>
+        <v>20.4125</v>
       </c>
       <c r="I130" t="n">
-        <v>1.1995</v>
+        <v>0.5103124999999999</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8000,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>1000</v>
+        <v>4800</v>
       </c>
       <c r="G131" t="n">
-        <v>44.99</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="H131" t="n">
-        <v>44.99</v>
+        <v>19.58125</v>
       </c>
       <c r="I131" t="n">
-        <v>1.12475</v>
+        <v>0.48953125</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8066,13 +8066,13 @@
         <v>600</v>
       </c>
       <c r="G132" t="n">
-        <v>17.99</v>
+        <v>16.99</v>
       </c>
       <c r="H132" t="n">
-        <v>29.98333333333333</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I132" t="n">
-        <v>0.7495833333333334</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8115,13 +8115,13 @@
         <v>1200</v>
       </c>
       <c r="G133" t="n">
-        <v>30.99</v>
+        <v>28.99</v>
       </c>
       <c r="H133" t="n">
-        <v>25.825</v>
+        <v>24.15833333333333</v>
       </c>
       <c r="I133" t="n">
-        <v>0.645625</v>
+        <v>0.6039583333333334</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8458,13 +8458,13 @@
         <v>600</v>
       </c>
       <c r="G140" t="n">
-        <v>13.99</v>
+        <v>14.99</v>
       </c>
       <c r="H140" t="n">
-        <v>23.31666666666667</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I140" t="n">
-        <v>0.5829166666666666</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8507,13 +8507,13 @@
         <v>1200</v>
       </c>
       <c r="G141" t="n">
-        <v>23.99</v>
+        <v>25.99</v>
       </c>
       <c r="H141" t="n">
-        <v>19.99166666666667</v>
+        <v>21.65833333333333</v>
       </c>
       <c r="I141" t="n">
-        <v>0.4997916666666667</v>
+        <v>0.5414583333333334</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8556,13 +8556,13 @@
         <v>2400</v>
       </c>
       <c r="G142" t="n">
-        <v>41.99</v>
+        <v>43.99</v>
       </c>
       <c r="H142" t="n">
-        <v>17.49583333333333</v>
+        <v>18.32916666666667</v>
       </c>
       <c r="I142" t="n">
-        <v>0.4373958333333333</v>
+        <v>0.4582291666666667</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8605,13 +8605,13 @@
         <v>4800</v>
       </c>
       <c r="G143" t="n">
-        <v>79.98999999999999</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="H143" t="n">
-        <v>16.66458333333333</v>
+        <v>17.70625</v>
       </c>
       <c r="I143" t="n">
-        <v>0.4166145833333333</v>
+        <v>0.44265625</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-13
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2931,7 +2931,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3016,16 +3016,16 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G29" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="H29" t="n">
-        <v>15.192</v>
+        <v>39.98</v>
       </c>
       <c r="I29" t="n">
-        <v>0.3798</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G30" t="n">
-        <v>35.99</v>
+        <v>37.99</v>
       </c>
       <c r="H30" t="n">
-        <v>14.396</v>
+        <v>37.99</v>
       </c>
       <c r="I30" t="n">
-        <v>0.3599</v>
+        <v>0.94975</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,16 +3114,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G31" t="n">
-        <v>19.99</v>
+        <v>18.99</v>
       </c>
       <c r="H31" t="n">
-        <v>39.98</v>
+        <v>15.192</v>
       </c>
       <c r="I31" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.3798</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G32" t="n">
-        <v>37.99</v>
+        <v>35.99</v>
       </c>
       <c r="H32" t="n">
-        <v>37.99</v>
+        <v>14.396</v>
       </c>
       <c r="I32" t="n">
-        <v>0.94975</v>
+        <v>0.3599</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-14
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1240,7 +1240,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - citrón limetka</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - citrón limetka</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-15
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1892,13 +1892,13 @@
         <v>1000</v>
       </c>
       <c r="G6" t="n">
-        <v>44.99</v>
+        <v>49.99</v>
       </c>
       <c r="H6" t="n">
-        <v>44.99</v>
+        <v>49.99</v>
       </c>
       <c r="I6" t="n">
-        <v>1.12475</v>
+        <v>1.24975</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1941,13 +1941,13 @@
         <v>2500</v>
       </c>
       <c r="G7" t="n">
-        <v>104.99</v>
+        <v>111.99</v>
       </c>
       <c r="H7" t="n">
-        <v>41.996</v>
+        <v>44.796</v>
       </c>
       <c r="I7" t="n">
-        <v>1.0499</v>
+        <v>1.1199</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1990,13 +1990,13 @@
         <v>5000</v>
       </c>
       <c r="G8" t="n">
-        <v>199.99</v>
+        <v>209.99</v>
       </c>
       <c r="H8" t="n">
-        <v>39.998</v>
+        <v>41.998</v>
       </c>
       <c r="I8" t="n">
-        <v>0.99995</v>
+        <v>1.04995</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -2039,13 +2039,13 @@
         <v>500</v>
       </c>
       <c r="G9" t="n">
-        <v>24.99</v>
+        <v>25.99</v>
       </c>
       <c r="H9" t="n">
-        <v>49.98</v>
+        <v>51.98</v>
       </c>
       <c r="I9" t="n">
-        <v>1.2495</v>
+        <v>1.2995</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -2333,13 +2333,13 @@
         <v>500</v>
       </c>
       <c r="G15" t="n">
-        <v>24.99</v>
+        <v>25.99</v>
       </c>
       <c r="H15" t="n">
-        <v>49.98</v>
+        <v>51.98</v>
       </c>
       <c r="I15" t="n">
-        <v>1.2495</v>
+        <v>1.2995</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -2382,13 +2382,13 @@
         <v>1000</v>
       </c>
       <c r="G16" t="n">
-        <v>44.99</v>
+        <v>49.99</v>
       </c>
       <c r="H16" t="n">
-        <v>44.99</v>
+        <v>49.99</v>
       </c>
       <c r="I16" t="n">
-        <v>1.12475</v>
+        <v>1.24975</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -2431,13 +2431,13 @@
         <v>2500</v>
       </c>
       <c r="G17" t="n">
-        <v>104.99</v>
+        <v>111.99</v>
       </c>
       <c r="H17" t="n">
-        <v>41.996</v>
+        <v>44.796</v>
       </c>
       <c r="I17" t="n">
-        <v>1.0499</v>
+        <v>1.1199</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2480,13 +2480,13 @@
         <v>5000</v>
       </c>
       <c r="G18" t="n">
-        <v>199.99</v>
+        <v>209.99</v>
       </c>
       <c r="H18" t="n">
-        <v>39.998</v>
+        <v>41.998</v>
       </c>
       <c r="I18" t="n">
-        <v>0.99995</v>
+        <v>1.04995</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3016,25 +3016,25 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G29" t="n">
-        <v>19.99</v>
+        <v>18.99</v>
       </c>
       <c r="H29" t="n">
-        <v>39.98</v>
+        <v>15.192</v>
       </c>
       <c r="I29" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.3798</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G30" t="n">
-        <v>37.99</v>
+        <v>35.99</v>
       </c>
       <c r="H30" t="n">
-        <v>37.99</v>
+        <v>14.396</v>
       </c>
       <c r="I30" t="n">
-        <v>0.94975</v>
+        <v>0.3599</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,16 +3114,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G31" t="n">
-        <v>18.99</v>
+        <v>21.99</v>
       </c>
       <c r="H31" t="n">
-        <v>15.192</v>
+        <v>43.98</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3798</v>
+        <v>1.0995</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G32" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H32" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-16
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2085,16 +2085,16 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>500</v>
+        <v>2270</v>
       </c>
       <c r="G10" t="n">
-        <v>16.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>33.98</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8495</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2134,16 +2134,16 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G11" t="n">
-        <v>31.99</v>
+        <v>16.99</v>
       </c>
       <c r="H11" t="n">
-        <v>31.99</v>
+        <v>33.98</v>
       </c>
       <c r="I11" t="n">
-        <v>0.79975</v>
+        <v>0.8495</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2183,16 +2183,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G12" t="n">
-        <v>74.98999999999999</v>
+        <v>31.99</v>
       </c>
       <c r="H12" t="n">
-        <v>29.996</v>
+        <v>31.99</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7499</v>
+        <v>0.79975</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2232,16 +2232,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="G13" t="n">
-        <v>139.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>27.998</v>
+        <v>29.996</v>
       </c>
       <c r="I13" t="n">
-        <v>0.69995</v>
+        <v>0.7499</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2270</v>
+        <v>5000</v>
       </c>
       <c r="G14" t="n">
-        <v>79.98999999999999</v>
+        <v>139.99</v>
       </c>
       <c r="H14" t="n">
-        <v>35.23788546255506</v>
+        <v>27.998</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8809471365638767</v>
+        <v>0.69995</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3016,25 +3016,25 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G29" t="n">
-        <v>18.99</v>
+        <v>21.99</v>
       </c>
       <c r="H29" t="n">
-        <v>15.192</v>
+        <v>43.98</v>
       </c>
       <c r="I29" t="n">
-        <v>0.3798</v>
+        <v>1.0995</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G30" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H30" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I30" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,16 +3114,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G31" t="n">
-        <v>21.99</v>
+        <v>18.99</v>
       </c>
       <c r="H31" t="n">
-        <v>43.98</v>
+        <v>15.192</v>
       </c>
       <c r="I31" t="n">
-        <v>1.0995</v>
+        <v>0.3798</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G32" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H32" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I32" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-18
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2085,16 +2085,16 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2270</v>
+        <v>500</v>
       </c>
       <c r="G10" t="n">
-        <v>79.98999999999999</v>
+        <v>16.99</v>
       </c>
       <c r="H10" t="n">
-        <v>35.23788546255506</v>
+        <v>33.98</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8809471365638767</v>
+        <v>0.8495</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2134,16 +2134,16 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G11" t="n">
-        <v>16.99</v>
+        <v>31.99</v>
       </c>
       <c r="H11" t="n">
-        <v>33.98</v>
+        <v>31.99</v>
       </c>
       <c r="I11" t="n">
-        <v>0.8495</v>
+        <v>0.79975</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2183,16 +2183,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G12" t="n">
-        <v>31.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>31.99</v>
+        <v>29.996</v>
       </c>
       <c r="I12" t="n">
-        <v>0.79975</v>
+        <v>0.7499</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2232,16 +2232,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="G13" t="n">
-        <v>74.98999999999999</v>
+        <v>139.99</v>
       </c>
       <c r="H13" t="n">
-        <v>29.996</v>
+        <v>27.998</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7499</v>
+        <v>0.69995</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>5000</v>
+        <v>2270</v>
       </c>
       <c r="G14" t="n">
-        <v>139.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>27.998</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I14" t="n">
-        <v>0.69995</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3016,16 +3016,16 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G29" t="n">
-        <v>21.99</v>
+        <v>18.99</v>
       </c>
       <c r="H29" t="n">
-        <v>43.98</v>
+        <v>15.192</v>
       </c>
       <c r="I29" t="n">
-        <v>1.0995</v>
+        <v>0.3798</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G30" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H30" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I30" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,16 +3114,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G31" t="n">
-        <v>18.99</v>
+        <v>21.99</v>
       </c>
       <c r="H31" t="n">
-        <v>15.192</v>
+        <v>43.98</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3798</v>
+        <v>1.0995</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G32" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H32" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-19
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P143"/>
+  <dimension ref="A1:P141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Organic Pure Whey Protein™ - Unflavoured 500g</t>
+          <t>Pure Whey Protein + - Chocolate 450g</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2526,25 +2526,25 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="G19" t="n">
-        <v>23.49</v>
+        <v>14.99</v>
       </c>
       <c r="H19" t="n">
-        <v>46.98</v>
+        <v>33.31111111111111</v>
       </c>
       <c r="I19" t="n">
-        <v>1.1745</v>
+        <v>0.8327777777777777</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/organic-pure-whey-protein/bpb-owpc</t>
+          <t>https://www.bulk.com/uk/products/pure-whey-protein-plus/bpb-pwpp</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Organic Pure Whey Protein™ - Unflavoured 1kg</t>
+          <t>Organic Pure Whey Protein™ - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2575,16 +2575,16 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G20" t="n">
-        <v>39.99</v>
+        <v>23.49</v>
       </c>
       <c r="H20" t="n">
-        <v>39.99</v>
+        <v>46.98</v>
       </c>
       <c r="I20" t="n">
-        <v>0.99975</v>
+        <v>1.1745</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Organic Pure Whey Protein™ - Unflavoured 2.5kg</t>
+          <t>Organic Pure Whey Protein™ - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2624,16 +2624,16 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G21" t="n">
-        <v>91.98999999999999</v>
+        <v>39.99</v>
       </c>
       <c r="H21" t="n">
-        <v>36.796</v>
+        <v>39.99</v>
       </c>
       <c r="I21" t="n">
-        <v>0.9199000000000001</v>
+        <v>0.99975</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pure Whey Protein™ - Lemon &amp; Coconut 500g </t>
+          <t>Organic Pure Whey Protein™ - Unflavoured 2.5kg</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2673,16 +2673,16 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="G22" t="n">
-        <v>16.99</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>33.98</v>
+        <v>36.796</v>
       </c>
       <c r="I22" t="n">
-        <v>0.8495</v>
+        <v>0.9199000000000001</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/pure-whey-protein-lemon-coconut-500/bpb-wpc8-lcoc-0500</t>
+          <t>https://www.bulk.com/uk/products/organic-pure-whey-protein/bpb-owpc</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Clear Whey Isolate - Apple &amp; Blackcurrant 500g</t>
+          <t xml:space="preserve">Pure Whey Protein™ - Lemon &amp; Coconut 500g </t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2725,22 +2725,22 @@
         <v>500</v>
       </c>
       <c r="G23" t="n">
-        <v>25.99</v>
+        <v>16.99</v>
       </c>
       <c r="H23" t="n">
-        <v>51.98</v>
+        <v>33.98</v>
       </c>
       <c r="I23" t="n">
-        <v>1.2995</v>
+        <v>0.8495</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/clear-whey-isolate/bpb-cwhe</t>
+          <t>https://www.bulk.com/uk/products/pure-whey-protein-lemon-coconut-500/bpb-wpc8-lcoc-0500</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Clear Whey Isolate - Strawberry &amp; Watermelon 1kg</t>
+          <t>Clear Whey Isolate - Apple &amp; Blackcurrant 500g</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2771,16 +2771,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G24" t="n">
-        <v>49.99</v>
+        <v>25.99</v>
       </c>
       <c r="H24" t="n">
-        <v>49.99</v>
+        <v>51.98</v>
       </c>
       <c r="I24" t="n">
-        <v>1.24975</v>
+        <v>1.2995</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Clear Whey Isolate - Peach Iced Tea 2kg</t>
+          <t>Clear Whey Isolate - Strawberry &amp; Watermelon 1kg</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2820,16 +2820,16 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G25" t="n">
-        <v>94.98999999999999</v>
+        <v>49.99</v>
       </c>
       <c r="H25" t="n">
-        <v>47.495</v>
+        <v>49.99</v>
       </c>
       <c r="I25" t="n">
-        <v>1.187375</v>
+        <v>1.24975</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hydrolysed Whey Protein Isolate - Unflavoured 500g</t>
+          <t>Clear Whey Isolate - Peach Iced Tea 2kg</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2869,16 +2869,16 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G26" t="n">
-        <v>27.99</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="H26" t="n">
-        <v>55.98</v>
+        <v>47.495</v>
       </c>
       <c r="I26" t="n">
-        <v>1.3995</v>
+        <v>1.187375</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/hydrolysed-whey-protein-isolate/bpb-hwpi-0000</t>
+          <t>https://www.bulk.com/uk/products/clear-whey-isolate/bpb-cwhe</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hydrolysed Whey Protein Isolate - Unflavoured 1kg</t>
+          <t>Hydrolysed Whey Protein Isolate - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2918,16 +2918,16 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G27" t="n">
-        <v>49.99</v>
+        <v>27.99</v>
       </c>
       <c r="H27" t="n">
-        <v>49.99</v>
+        <v>55.98</v>
       </c>
       <c r="I27" t="n">
-        <v>1.24975</v>
+        <v>1.3995</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hydrolysed Whey Protein Isolate - Unflavoured 2.5kg</t>
+          <t>Hydrolysed Whey Protein Isolate - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2967,20 +2967,20 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G28" t="n">
-        <v>119.99</v>
+        <v>49.99</v>
       </c>
       <c r="H28" t="n">
-        <v>47.996</v>
+        <v>49.99</v>
       </c>
       <c r="I28" t="n">
-        <v>1.1999</v>
+        <v>1.24975</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Hydrolysed Whey Protein Isolate - Unflavoured 2.5kg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3016,25 +3016,25 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1250</v>
+        <v>2500</v>
       </c>
       <c r="G29" t="n">
-        <v>18.99</v>
+        <v>119.99</v>
       </c>
       <c r="H29" t="n">
-        <v>15.192</v>
+        <v>47.996</v>
       </c>
       <c r="I29" t="n">
-        <v>0.3798</v>
+        <v>1.1999</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/hydrolysed-whey-protein-isolate/bpb-hwpi-0000</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="G30" t="n">
-        <v>35.99</v>
+        <v>21.99</v>
       </c>
       <c r="H30" t="n">
-        <v>14.396</v>
+        <v>43.98</v>
       </c>
       <c r="I30" t="n">
-        <v>0.3599</v>
+        <v>1.0995</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,16 +3114,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G31" t="n">
-        <v>21.99</v>
+        <v>39.99</v>
       </c>
       <c r="H31" t="n">
-        <v>43.98</v>
+        <v>39.99</v>
       </c>
       <c r="I31" t="n">
-        <v>1.0995</v>
+        <v>0.99975</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1000</v>
+        <v>1250</v>
       </c>
       <c r="G32" t="n">
-        <v>39.99</v>
+        <v>18.99</v>
       </c>
       <c r="H32" t="n">
-        <v>39.99</v>
+        <v>15.192</v>
       </c>
       <c r="I32" t="n">
-        <v>0.99975</v>
+        <v>0.3798</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Whey Protein Coffee - Iced Caramel Latte 500g</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3212,16 +3212,16 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="G33" t="n">
-        <v>17.99</v>
+        <v>35.99</v>
       </c>
       <c r="H33" t="n">
-        <v>35.98</v>
+        <v>14.396</v>
       </c>
       <c r="I33" t="n">
-        <v>0.8995</v>
+        <v>0.3599</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3230,7 +3230,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/whey-protein-coffee/bpb-pico</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Whey Protein Coffee - Iced Latte 1kg</t>
+          <t>Whey Protein Coffee - Iced Caramel Latte 500g</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G34" t="n">
-        <v>33.99</v>
+        <v>17.99</v>
       </c>
       <c r="H34" t="n">
-        <v>33.99</v>
+        <v>35.98</v>
       </c>
       <c r="I34" t="n">
-        <v>0.84975</v>
+        <v>0.8995</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Clear Whey All In One - Apple &amp; Blackcurrant 500g</t>
+          <t>Whey Protein Coffee - Iced Latte 1kg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3310,16 +3310,16 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G35" t="n">
-        <v>22.49</v>
+        <v>33.99</v>
       </c>
       <c r="H35" t="n">
-        <v>44.98</v>
+        <v>33.99</v>
       </c>
       <c r="I35" t="n">
-        <v>1.1245</v>
+        <v>0.84975</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/clear-all-in-one/bble-cwa1</t>
+          <t>https://www.bulk.com/uk/products/whey-protein-coffee/bpb-pico</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Clear Whey All In One - Apple &amp; Blackcurrant 1kg</t>
+          <t>Clear Whey All In One - Apple &amp; Blackcurrant 500g</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3359,16 +3359,16 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G36" t="n">
-        <v>38.99</v>
+        <v>22.49</v>
       </c>
       <c r="H36" t="n">
-        <v>38.99</v>
+        <v>44.98</v>
       </c>
       <c r="I36" t="n">
-        <v>0.97475</v>
+        <v>1.1245</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3389,12 +3389,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
+          <t>Clear Whey All In One - Apple &amp; Blackcurrant 1kg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3408,16 +3408,16 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="G37" t="n">
-        <v>4.99</v>
+        <v>38.99</v>
       </c>
       <c r="H37" t="n">
-        <v>49.9</v>
+        <v>38.99</v>
       </c>
       <c r="I37" t="n">
-        <v>1.2475</v>
+        <v>0.97475</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://www.bulk.com/uk/products/clear-all-in-one/bble-cwa1</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3457,16 +3457,16 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>12.99</v>
+        <v>4.99</v>
       </c>
       <c r="H38" t="n">
-        <v>25.98</v>
+        <v>49.9</v>
       </c>
       <c r="I38" t="n">
-        <v>0.6495</v>
+        <v>1.2475</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3506,16 +3506,16 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G39" t="n">
-        <v>24.99</v>
+        <v>12.99</v>
       </c>
       <c r="H39" t="n">
-        <v>24.99</v>
+        <v>25.98</v>
       </c>
       <c r="I39" t="n">
-        <v>0.62475</v>
+        <v>0.6495</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3555,16 +3555,16 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="G40" t="n">
-        <v>7.49</v>
+        <v>24.99</v>
       </c>
       <c r="H40" t="n">
-        <v>29.96</v>
+        <v>24.99</v>
       </c>
       <c r="I40" t="n">
-        <v>0.749</v>
+        <v>0.62475</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 100g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3604,16 +3604,16 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="G41" t="n">
-        <v>9.99</v>
+        <v>7.49</v>
       </c>
       <c r="H41" t="n">
-        <v>99.90000000000001</v>
+        <v>29.96</v>
       </c>
       <c r="I41" t="n">
-        <v>2.4975</v>
+        <v>0.749</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creapure-creatine-monohydrate/bpb-crea-0000</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 500g</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 100g</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3653,16 +3653,16 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>39.99</v>
+        <v>9.99</v>
       </c>
       <c r="H42" t="n">
-        <v>79.98</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="I42" t="n">
-        <v>1.9995</v>
+        <v>2.4975</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 1kg</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3702,16 +3702,16 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G43" t="n">
-        <v>74.98999999999999</v>
+        <v>39.99</v>
       </c>
       <c r="H43" t="n">
-        <v>74.98999999999999</v>
+        <v>79.98</v>
       </c>
       <c r="I43" t="n">
-        <v>1.87475</v>
+        <v>1.9995</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -3727,40 +3727,40 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>True Whey - GymBeam 1000 g - bez príchute - 01</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>1000</v>
       </c>
       <c r="G44" t="n">
-        <v>33.95</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H44" t="n">
-        <v>33.95</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="I44" t="n">
-        <v>0.84875</v>
+        <v>1.87475</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/true-whey-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creapure-creatine-monohydrate/bpb-crea-0000</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>True Whey - GymBeam 2500 g - bez príchute - 01</t>
+          <t>True Whey - GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3800,16 +3800,16 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G45" t="n">
-        <v>79.95</v>
+        <v>33.95</v>
       </c>
       <c r="H45" t="n">
-        <v>31.98</v>
+        <v>33.95</v>
       </c>
       <c r="I45" t="n">
-        <v>0.7995</v>
+        <v>0.84875</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ASAP True Whey - GymBeam 2000 g - banán</t>
+          <t>True Whey - GymBeam 2500 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3849,16 +3849,16 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="G46" t="n">
-        <v>87.95</v>
+        <v>79.95</v>
       </c>
       <c r="H46" t="n">
-        <v>43.975</v>
+        <v>31.98</v>
       </c>
       <c r="I46" t="n">
-        <v>1.099375</v>
+        <v>0.7995</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/asap-true-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/true-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ASAP True Whey - GymBeam 900 g - banán</t>
+          <t>ASAP True Whey - GymBeam 2000 g - banán</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3898,16 +3898,16 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="G47" t="n">
-        <v>44.95</v>
+        <v>87.95</v>
       </c>
       <c r="H47" t="n">
-        <v>49.94444444444444</v>
+        <v>43.975</v>
       </c>
       <c r="I47" t="n">
-        <v>1.248611111111111</v>
+        <v>1.099375</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Pure IsoWhey - GymBeam 1000 g - bez príchute - 01</t>
+          <t>ASAP True Whey - GymBeam 900 g - banán</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3947,16 +3947,16 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="G48" t="n">
-        <v>39.95</v>
+        <v>44.95</v>
       </c>
       <c r="H48" t="n">
-        <v>39.95</v>
+        <v>49.94444444444444</v>
       </c>
       <c r="I48" t="n">
-        <v>0.99875</v>
+        <v>1.248611111111111</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/pure-isowhey-gymbeam.html</t>
+          <t>https://gymbeam.sk/asap-true-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Pure IsoWhey - GymBeam 2500 g - bez príchute - 01</t>
+          <t>Pure IsoWhey - GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3996,20 +3996,20 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G49" t="n">
-        <v>87.95</v>
+        <v>39.95</v>
       </c>
       <c r="H49" t="n">
-        <v>35.18</v>
+        <v>39.95</v>
       </c>
       <c r="I49" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.99875</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>100% Whey - Nutrend 2250 g - banán</t>
+          <t>Pure IsoWhey - GymBeam 2500 g - čokoláda - 00</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4045,25 +4045,25 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>2250</v>
+        <v>2500</v>
       </c>
       <c r="G50" t="n">
-        <v>67.95</v>
+        <v>87.95</v>
       </c>
       <c r="H50" t="n">
-        <v>30.2</v>
+        <v>35.18</v>
       </c>
       <c r="I50" t="n">
-        <v>0.755</v>
+        <v>0.8794999999999999</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/614-protein-whey-core-100-nutrend.html</t>
+          <t>https://gymbeam.sk/pure-isowhey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -4080,7 +4080,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Whey Protein 100 - Bodylab 1000 g - banán</t>
+          <t>100% Whey - Nutrend 2250 g - banán</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4094,16 +4094,16 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1000</v>
+        <v>2250</v>
       </c>
       <c r="G51" t="n">
-        <v>19.5</v>
+        <v>67.95</v>
       </c>
       <c r="H51" t="n">
-        <v>19.5</v>
+        <v>30.2</v>
       </c>
       <c r="I51" t="n">
-        <v>0.4875</v>
+        <v>0.755</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-whey100-bodylab.html</t>
+          <t>https://gymbeam.sk/614-protein-whey-core-100-nutrend.html</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>100% Whey - Stacker2 2000 g - čokoláda</t>
+          <t>Whey Protein 100 - Bodylab 1000 g - banán</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4143,16 +4143,16 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G52" t="n">
-        <v>61.95</v>
+        <v>19.5</v>
       </c>
       <c r="H52" t="n">
-        <v>30.975</v>
+        <v>19.5</v>
       </c>
       <c r="I52" t="n">
-        <v>0.774375</v>
+        <v>0.4875</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-100-whey-stacker2.html</t>
+          <t>https://gymbeam.sk/protein-whey100-bodylab.html</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 1850 g - čokoláda</t>
+          <t>100% Whey - Stacker2 2000 g - čokoláda</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4192,16 +4192,16 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1850</v>
+        <v>2000</v>
       </c>
       <c r="G53" t="n">
-        <v>34.95</v>
+        <v>61.95</v>
       </c>
       <c r="H53" t="n">
-        <v>18.89189189189189</v>
+        <v>30.975</v>
       </c>
       <c r="I53" t="n">
-        <v>0.4722972972972973</v>
+        <v>0.774375</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/510-protein-100-whey-2350-g-scitec-nutrition-3.html</t>
+          <t>https://gymbeam.sk/protein-100-whey-stacker2.html</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 920 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 1850 g - čokoláda</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4241,16 +4241,16 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>920</v>
+        <v>1850</v>
       </c>
       <c r="G54" t="n">
-        <v>23.95</v>
+        <v>34.95</v>
       </c>
       <c r="H54" t="n">
-        <v>26.03260869565218</v>
+        <v>18.89189189189189</v>
       </c>
       <c r="I54" t="n">
-        <v>0.6508152173913043</v>
+        <v>0.4722972972972973</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 2350 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 920 g - čokoláda</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4290,16 +4290,16 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>2350</v>
+        <v>920</v>
       </c>
       <c r="G55" t="n">
-        <v>45.95</v>
+        <v>23.95</v>
       </c>
       <c r="H55" t="n">
-        <v>19.5531914893617</v>
+        <v>26.03260869565218</v>
       </c>
       <c r="I55" t="n">
-        <v>0.4888297872340426</v>
+        <v>0.6508152173913043</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 5000 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 2350 g - čokoláda</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4339,16 +4339,16 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>5000</v>
+        <v>2350</v>
       </c>
       <c r="G56" t="n">
-        <v>95.95</v>
+        <v>45.95</v>
       </c>
       <c r="H56" t="n">
-        <v>19.19</v>
+        <v>19.5531914893617</v>
       </c>
       <c r="I56" t="n">
-        <v>0.47975</v>
+        <v>0.4888297872340426</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>100% Whey Premium - ActivLab 2000 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 5000 g - čokoláda</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4388,16 +4388,16 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="G57" t="n">
-        <v>50.95</v>
+        <v>95.95</v>
       </c>
       <c r="H57" t="n">
-        <v>25.475</v>
+        <v>19.19</v>
       </c>
       <c r="I57" t="n">
-        <v>0.636875</v>
+        <v>0.47975</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-whey-premium-activlab.html</t>
+          <t>https://gymbeam.sk/510-protein-100-whey-2350-g-scitec-nutrition-3.html</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Proteín Combat 100% Whey - MusclePharm 2270 g - čokoláda</t>
+          <t>100% Whey Premium - ActivLab 2000 g - čokoláda</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4437,16 +4437,16 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>2270</v>
+        <v>2000</v>
       </c>
       <c r="G58" t="n">
-        <v>43.95</v>
+        <v>50.95</v>
       </c>
       <c r="H58" t="n">
-        <v>19.36123348017621</v>
+        <v>25.475</v>
       </c>
       <c r="I58" t="n">
-        <v>0.4840308370044053</v>
+        <v>0.636875</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-combat-100-whey-musclepharm.html</t>
+          <t>https://gymbeam.sk/100-whey-premium-activlab.html</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 1110 g - chocolate</t>
+          <t>Proteín Combat 100% Whey - MusclePharm 2270 g - čokoláda</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4486,16 +4486,16 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>1110</v>
+        <v>2270</v>
       </c>
       <c r="G59" t="n">
-        <v>23.95</v>
+        <v>43.95</v>
       </c>
       <c r="H59" t="n">
-        <v>21.57657657657658</v>
+        <v>19.36123348017621</v>
       </c>
       <c r="I59" t="n">
-        <v>0.5394144144144144</v>
+        <v>0.4840308370044053</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/10-protein-100-whey-professional-2350-g-scitec-nutrition.html</t>
+          <t>https://gymbeam.sk/protein-combat-100-whey-musclepharm.html</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 2820 g - čokoláda</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 1110 g - chocolate</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4535,16 +4535,16 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>2820</v>
+        <v>1110</v>
       </c>
       <c r="G60" t="n">
-        <v>45.95</v>
+        <v>23.95</v>
       </c>
       <c r="H60" t="n">
-        <v>16.29432624113475</v>
+        <v>21.57657657657658</v>
       </c>
       <c r="I60" t="n">
-        <v>0.4073581560283688</v>
+        <v>0.5394144144144144</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition - 500 g - chocolate</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 2820 g - čokoláda</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4584,16 +4584,16 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>500</v>
+        <v>2820</v>
       </c>
       <c r="G61" t="n">
-        <v>21.95</v>
+        <v>45.95</v>
       </c>
       <c r="H61" t="n">
-        <v>43.9</v>
+        <v>16.29432624113475</v>
       </c>
       <c r="I61" t="n">
-        <v>1.0975</v>
+        <v>0.4073581560283688</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 750 g - banán</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition - 500 g - chocolate</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4633,16 +4633,16 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="G62" t="n">
-        <v>20.95</v>
+        <v>21.95</v>
       </c>
       <c r="H62" t="n">
-        <v>27.93333333333333</v>
+        <v>43.9</v>
       </c>
       <c r="I62" t="n">
-        <v>0.6983333333333334</v>
+        <v>1.0975</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 920 g - čokoláda</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 750 g - banán</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4682,16 +4682,16 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>920</v>
+        <v>750</v>
       </c>
       <c r="G63" t="n">
-        <v>21.95</v>
+        <v>20.95</v>
       </c>
       <c r="H63" t="n">
-        <v>23.85869565217391</v>
+        <v>27.93333333333333</v>
       </c>
       <c r="I63" t="n">
-        <v>0.5964673913043478</v>
+        <v>0.6983333333333334</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 2350 g - banán</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 920 g - čokoláda</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4731,16 +4731,16 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>2350</v>
+        <v>920</v>
       </c>
       <c r="G64" t="n">
-        <v>45.95</v>
+        <v>21.95</v>
       </c>
       <c r="H64" t="n">
-        <v>19.5531914893617</v>
+        <v>23.85869565217391</v>
       </c>
       <c r="I64" t="n">
-        <v>0.4888297872340426</v>
+        <v>0.5964673913043478</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 5000 g - banán</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 2350 g - banán</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4780,16 +4780,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>5000</v>
+        <v>2350</v>
       </c>
       <c r="G65" t="n">
-        <v>99.95</v>
+        <v>45.95</v>
       </c>
       <c r="H65" t="n">
-        <v>19.99</v>
+        <v>19.5531914893617</v>
       </c>
       <c r="I65" t="n">
-        <v>0.49975</v>
+        <v>0.4888297872340426</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Isolate - Scitec Nutrition 2000 g - banán</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 5000 g - banán</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4829,16 +4829,16 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="G66" t="n">
-        <v>59.95</v>
+        <v>99.95</v>
       </c>
       <c r="H66" t="n">
-        <v>29.975</v>
+        <v>19.99</v>
       </c>
       <c r="I66" t="n">
-        <v>0.749375</v>
+        <v>0.49975</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -4847,7 +4847,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/12-protein-100-whey-isolate-20-kg.html</t>
+          <t>https://gymbeam.sk/10-protein-100-whey-professional-2350-g-scitec-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Isolate - Scitec Nutrition 4000 g - čokoláda</t>
+          <t>Protein 100% Whey Isolate - Scitec Nutrition 2000 g - banán</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4878,16 +4878,16 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="G67" t="n">
-        <v>87.95</v>
+        <v>59.95</v>
       </c>
       <c r="H67" t="n">
-        <v>21.9875</v>
+        <v>29.975</v>
       </c>
       <c r="I67" t="n">
-        <v>0.5496875</v>
+        <v>0.749375</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Isolate - Scitec Nutrition 700 g - banán</t>
+          <t>Protein 100% Whey Isolate - Scitec Nutrition 4000 g - čokoláda</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4927,16 +4927,16 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>700</v>
+        <v>4000</v>
       </c>
       <c r="G68" t="n">
-        <v>25.95</v>
+        <v>87.95</v>
       </c>
       <c r="H68" t="n">
-        <v>37.07142857142857</v>
+        <v>21.9875</v>
       </c>
       <c r="I68" t="n">
-        <v>0.9267857142857143</v>
+        <v>0.5496875</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -4962,7 +4962,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey Protein - MuscleTech  2270 g - trojitá čokoláda</t>
+          <t>Protein 100% Whey Isolate - Scitec Nutrition 700 g - banán</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4976,16 +4976,16 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>2270</v>
+        <v>700</v>
       </c>
       <c r="G69" t="n">
-        <v>33.95</v>
+        <v>25.95</v>
       </c>
       <c r="H69" t="n">
-        <v>14.95594713656388</v>
+        <v>37.07142857142857</v>
       </c>
       <c r="I69" t="n">
-        <v>0.3738986784140969</v>
+        <v>0.9267857142857143</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-premium-whey-protein-plus-muscletech.html</t>
+          <t>https://gymbeam.sk/12-protein-100-whey-isolate-20-kg.html</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Animal 100 % Whey Proteín - Universal Nutrition 1000 g - čokoláda</t>
+          <t>Proteín 100% Whey Protein - MuscleTech  2270 g - trojitá čokoláda</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -5025,16 +5025,16 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>1000</v>
+        <v>2270</v>
       </c>
       <c r="G70" t="n">
-        <v>31.95</v>
+        <v>33.95</v>
       </c>
       <c r="H70" t="n">
-        <v>31.95</v>
+        <v>14.95594713656388</v>
       </c>
       <c r="I70" t="n">
-        <v>0.79875</v>
+        <v>0.3738986784140969</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/animal-100-whey-protein-universal-nutrition.html</t>
+          <t>https://gymbeam.sk/100-premium-whey-protein-plus-muscletech.html</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 2250 g - banánový krém</t>
+          <t>Animal 100 % Whey Proteín - Universal Nutrition 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -5074,16 +5074,16 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>2250</v>
+        <v>1000</v>
       </c>
       <c r="G71" t="n">
-        <v>70.95</v>
+        <v>31.95</v>
       </c>
       <c r="H71" t="n">
-        <v>31.53333333333333</v>
+        <v>31.95</v>
       </c>
       <c r="I71" t="n">
-        <v>0.7883333333333333</v>
+        <v>0.79875</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-whey-gold-standard-optimum-nutrition.html</t>
+          <t>https://gymbeam.sk/animal-100-whey-protein-universal-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 450 g - dvojitá bohatá čokoláda</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 2250 g - vanilková zmrzlina</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -5123,20 +5123,20 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>450</v>
+        <v>2250</v>
       </c>
       <c r="G72" t="n">
-        <v>22.95</v>
+        <v>70.95</v>
       </c>
       <c r="H72" t="n">
-        <v>51</v>
+        <v>31.53333333333333</v>
       </c>
       <c r="I72" t="n">
-        <v>1.275</v>
+        <v>0.7883333333333333</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 4540 g - dvojitá bohatá čokoláda</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 450 g - dvojitá bohatá čokoláda</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -5172,16 +5172,16 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>4540</v>
+        <v>450</v>
       </c>
       <c r="G73" t="n">
-        <v>169.95</v>
+        <v>22.95</v>
       </c>
       <c r="H73" t="n">
-        <v>37.43392070484582</v>
+        <v>51</v>
       </c>
       <c r="I73" t="n">
-        <v>0.9358480176211453</v>
+        <v>1.275</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 896 g - banánový krém</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 4540 g - dvojitá bohatá čokoláda</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -5221,20 +5221,20 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>896</v>
+        <v>4540</v>
       </c>
       <c r="G74" t="n">
-        <v>32.95</v>
+        <v>169.95</v>
       </c>
       <c r="H74" t="n">
-        <v>36.77455357142857</v>
+        <v>37.43392070484582</v>
       </c>
       <c r="I74" t="n">
-        <v>0.9193638392857143</v>
+        <v>0.9358480176211453</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Proteín 100% Premium Whey Protein Plus - MuscleTech 2270 g - trojitá čokoláda</t>
+          <t>Proteín 100% Premium Whey Protein Plus - MuscleTech 2720 g - deluxe čokoláda</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5368,16 +5368,16 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>2270</v>
+        <v>2720</v>
       </c>
       <c r="G77" t="n">
-        <v>45.95</v>
+        <v>39.95</v>
       </c>
       <c r="H77" t="n">
-        <v>20.24229074889868</v>
+        <v>14.6875</v>
       </c>
       <c r="I77" t="n">
-        <v>0.5060572687224669</v>
+        <v>0.3671875</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -5403,7 +5403,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Proteín 100% Premium Whey Protein Plus - MuscleTech 2720 g - deluxe čokoláda</t>
+          <t>Proteín 100% Premium Whey Isolate Plus 1360 g - MuscleTech deluxe čokoláda</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5417,16 +5417,16 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>2720</v>
+        <v>1360</v>
       </c>
       <c r="G78" t="n">
-        <v>39.95</v>
+        <v>29.95</v>
       </c>
       <c r="H78" t="n">
-        <v>14.6875</v>
+        <v>22.02205882352941</v>
       </c>
       <c r="I78" t="n">
-        <v>0.3671875</v>
+        <v>0.5505514705882353</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -5435,7 +5435,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-premium-whey-protein-plus-muscletech-2.html</t>
+          <t>https://gymbeam.sk/protein-100-premium-whey-isolate-plus-1380-g-muscletech.html</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Proteín 100% Premium Whey Isolate Plus 1360 g - MuscleTech deluxe čokoláda</t>
+          <t>Clear Whey - Ghost 640 g - modrá malina</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5466,16 +5466,16 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>1360</v>
+        <v>640</v>
       </c>
       <c r="G79" t="n">
-        <v>29.95</v>
+        <v>46.95</v>
       </c>
       <c r="H79" t="n">
-        <v>22.02205882352941</v>
+        <v>73.359375</v>
       </c>
       <c r="I79" t="n">
-        <v>0.5505514705882353</v>
+        <v>1.833984375</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-100-premium-whey-isolate-plus-1380-g-muscletech.html</t>
+          <t>https://gymbeam.sk/clear-whey-ghost.html</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Clear Whey - Ghost 640 g - modrá malina</t>
+          <t>Protein Gold Whey - Weider 500 g - jahoda</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5515,16 +5515,16 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>640</v>
+        <v>500</v>
       </c>
       <c r="G80" t="n">
-        <v>46.95</v>
+        <v>19.95</v>
       </c>
       <c r="H80" t="n">
-        <v>73.359375</v>
+        <v>39.9</v>
       </c>
       <c r="I80" t="n">
-        <v>1.833984375</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-ghost.html</t>
+          <t>https://gymbeam.sk/protein-gold-whey-weider.html</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Protein Gold Whey - Weider 2000 g - čokoláda</t>
+          <t>BIO Whey Protein - GymBeam 900 g - kakao</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5564,25 +5564,25 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>2000</v>
+        <v>900</v>
       </c>
       <c r="G81" t="n">
-        <v>54.95</v>
+        <v>45.95</v>
       </c>
       <c r="H81" t="n">
-        <v>27.475</v>
+        <v>51.05555555555556</v>
       </c>
       <c r="I81" t="n">
-        <v>0.686875</v>
+        <v>1.276388888888889</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-gold-whey-weider.html</t>
+          <t>https://gymbeam.sk/bio-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Protein Gold Whey - Weider 500 g - banana split</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5613,25 +5613,25 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G82" t="n">
-        <v>19.95</v>
+        <v>37.95</v>
       </c>
       <c r="H82" t="n">
-        <v>39.9</v>
+        <v>37.95</v>
       </c>
       <c r="I82" t="n">
-        <v>0.9975000000000001</v>
+        <v>0.94875</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-gold-whey-weider.html</t>
+          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>BIO Whey Protein - GymBeam 900 g - kakao</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5662,16 +5662,16 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="G83" t="n">
-        <v>45.95</v>
+        <v>67.95</v>
       </c>
       <c r="H83" t="n">
-        <v>51.05555555555556</v>
+        <v>33.975</v>
       </c>
       <c r="I83" t="n">
-        <v>1.276388888888889</v>
+        <v>0.849375</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -5680,7 +5680,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/bio-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5711,16 +5711,16 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G84" t="n">
-        <v>37.95</v>
+        <v>24.95</v>
       </c>
       <c r="H84" t="n">
-        <v>37.95</v>
+        <v>49.9</v>
       </c>
       <c r="I84" t="n">
-        <v>0.94875</v>
+        <v>1.2475</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -5746,7 +5746,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
+          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5760,16 +5760,16 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G85" t="n">
-        <v>67.95</v>
+        <v>37.95</v>
       </c>
       <c r="H85" t="n">
-        <v>33.975</v>
+        <v>37.95</v>
       </c>
       <c r="I85" t="n">
-        <v>0.849375</v>
+        <v>0.94875</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
         </is>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
+          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
+          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5861,13 +5861,13 @@
         <v>1000</v>
       </c>
       <c r="G87" t="n">
-        <v>37.95</v>
+        <v>31.95</v>
       </c>
       <c r="H87" t="n">
-        <v>37.95</v>
+        <v>31.95</v>
       </c>
       <c r="I87" t="n">
-        <v>0.94875</v>
+        <v>0.79875</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
+          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
+          <t>Whey Proteín - Mammut Nutrition 3000 g - vanilka</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5907,16 +5907,16 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G88" t="n">
-        <v>24.95</v>
+        <v>93.95</v>
       </c>
       <c r="H88" t="n">
-        <v>49.9</v>
+        <v>31.31666666666667</v>
       </c>
       <c r="I88" t="n">
-        <v>1.2475</v>
+        <v>0.7829166666666667</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
+          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
+          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5956,25 +5956,25 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G89" t="n">
-        <v>31.95</v>
+        <v>21.95</v>
       </c>
       <c r="H89" t="n">
-        <v>31.95</v>
+        <v>43.9</v>
       </c>
       <c r="I89" t="n">
-        <v>0.79875</v>
+        <v>1.0975</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
+          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 3000 g - čokoláda</t>
+          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6005,25 +6005,25 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="G90" t="n">
-        <v>93.95</v>
+        <v>34.95</v>
       </c>
       <c r="H90" t="n">
-        <v>31.31666666666667</v>
+        <v>34.95</v>
       </c>
       <c r="I90" t="n">
-        <v>0.7829166666666667</v>
+        <v>0.87375</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
+          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6054,16 +6054,16 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G91" t="n">
-        <v>21.95</v>
+        <v>62.95</v>
       </c>
       <c r="H91" t="n">
-        <v>43.9</v>
+        <v>31.475</v>
       </c>
       <c r="I91" t="n">
-        <v>1.0975</v>
+        <v>0.786875</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -6072,7 +6072,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
+          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6103,16 +6103,16 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G92" t="n">
-        <v>34.95</v>
+        <v>19.5</v>
       </c>
       <c r="H92" t="n">
-        <v>34.95</v>
+        <v>39</v>
       </c>
       <c r="I92" t="n">
-        <v>0.87375</v>
+        <v>0.975</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
+          <t>Whey Protein - Bodylab24 1000 g - banán</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6152,16 +6152,16 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G93" t="n">
-        <v>62.95</v>
+        <v>39.95</v>
       </c>
       <c r="H93" t="n">
-        <v>31.475</v>
+        <v>39.95</v>
       </c>
       <c r="I93" t="n">
-        <v>0.786875</v>
+        <v>0.99875</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -6170,7 +6170,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
+          <t>Whey Protein - Bodylab24 2000 g - banán</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6201,16 +6201,16 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G94" t="n">
-        <v>19.5</v>
+        <v>64.95</v>
       </c>
       <c r="H94" t="n">
-        <v>39</v>
+        <v>32.475</v>
       </c>
       <c r="I94" t="n">
-        <v>0.975</v>
+        <v>0.811875</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 1000 g - banán</t>
+          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6250,16 +6250,16 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="G95" t="n">
-        <v>39.95</v>
+        <v>42.95</v>
       </c>
       <c r="H95" t="n">
-        <v>39.95</v>
+        <v>107.375</v>
       </c>
       <c r="I95" t="n">
-        <v>0.99875</v>
+        <v>2.684375</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
+          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
         </is>
       </c>
     </row>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 2000 g - banán</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6299,16 +6299,16 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="G96" t="n">
-        <v>64.95</v>
+        <v>34.95</v>
       </c>
       <c r="H96" t="n">
-        <v>32.475</v>
+        <v>29.125</v>
       </c>
       <c r="I96" t="n">
-        <v>0.811875</v>
+        <v>0.728125</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6317,7 +6317,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
+          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6348,16 +6348,16 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>400</v>
+        <v>2400</v>
       </c>
       <c r="G97" t="n">
-        <v>42.95</v>
+        <v>62.95</v>
       </c>
       <c r="H97" t="n">
-        <v>107.375</v>
+        <v>26.22916666666667</v>
       </c>
       <c r="I97" t="n">
-        <v>2.684375</v>
+        <v>0.6557291666666667</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
+          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
+          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6397,16 +6397,16 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="G98" t="n">
-        <v>34.95</v>
+        <v>19.5</v>
       </c>
       <c r="H98" t="n">
-        <v>29.125</v>
+        <v>32.5</v>
       </c>
       <c r="I98" t="n">
-        <v>0.728125</v>
+        <v>0.8125</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6446,16 +6446,16 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>2400</v>
+        <v>1000</v>
       </c>
       <c r="G99" t="n">
-        <v>62.95</v>
+        <v>16.5</v>
       </c>
       <c r="H99" t="n">
-        <v>26.22916666666667</v>
+        <v>16.5</v>
       </c>
       <c r="I99" t="n">
-        <v>0.6557291666666667</v>
+        <v>0.4125</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6495,16 +6495,16 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>600</v>
+        <v>2500</v>
       </c>
       <c r="G100" t="n">
-        <v>19.5</v>
+        <v>31.95</v>
       </c>
       <c r="H100" t="n">
-        <v>32.5</v>
+        <v>12.78</v>
       </c>
       <c r="I100" t="n">
-        <v>0.8125</v>
+        <v>0.3195</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6513,7 +6513,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6544,16 +6544,16 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G101" t="n">
-        <v>16.5</v>
+        <v>11.95</v>
       </c>
       <c r="H101" t="n">
-        <v>16.5</v>
+        <v>23.9</v>
       </c>
       <c r="I101" t="n">
-        <v>0.4125</v>
+        <v>0.5975</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6593,25 +6593,25 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>2500</v>
+        <v>1450</v>
       </c>
       <c r="G102" t="n">
-        <v>31.95</v>
+        <v>39.95</v>
       </c>
       <c r="H102" t="n">
-        <v>12.78</v>
+        <v>27.55172413793104</v>
       </c>
       <c r="I102" t="n">
-        <v>0.3195</v>
+        <v>0.6887931034482758</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>Whey + Isolate proteín s enzýmami DigeZyme® – GymBeam 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6642,25 +6642,25 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G103" t="n">
-        <v>11.95</v>
+        <v>37.95</v>
       </c>
       <c r="H103" t="n">
-        <v>23.9</v>
+        <v>37.95</v>
       </c>
       <c r="I103" t="n">
-        <v>0.5975</v>
+        <v>0.94875</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/whey-isolate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6677,7 +6677,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
+          <t>Whey Protein Isolate 90 - GoNutrition banán - 1000 g</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6691,25 +6691,25 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>1450</v>
+        <v>1000</v>
       </c>
       <c r="G104" t="n">
-        <v>39.95</v>
+        <v>22.95</v>
       </c>
       <c r="H104" t="n">
-        <v>27.55172413793104</v>
+        <v>22.95</v>
       </c>
       <c r="I104" t="n">
-        <v>0.6887931034482758</v>
+        <v>0.57375</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-isolate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Whey + Isolate proteín s enzýmami DigeZyme® – GymBeam 1000 g - čokoláda</t>
+          <t>Whey Protein Isolate 90 - GoNutrition trojitá čokoláda - 2500 g</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,25 +6740,25 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G105" t="n">
-        <v>37.95</v>
+        <v>45.95</v>
       </c>
       <c r="H105" t="n">
-        <v>37.95</v>
+        <v>18.38</v>
       </c>
       <c r="I105" t="n">
-        <v>0.94875</v>
+        <v>0.4595</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-isolate-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-isolate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Whey Protein Isolate 90 - GoNutrition banán - 1000 g</t>
+          <t>Anabolic Whey - GymBeam + darček 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6792,22 +6792,22 @@
         <v>1000</v>
       </c>
       <c r="G106" t="n">
-        <v>22.95</v>
+        <v>27.95</v>
       </c>
       <c r="H106" t="n">
-        <v>22.95</v>
+        <v>27.95</v>
       </c>
       <c r="I106" t="n">
-        <v>0.57375</v>
+        <v>0.69875</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-isolate-gonutrition.html</t>
+          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein Isolate 90 - GoNutrition trojitá čokoláda - 2500 g</t>
+          <t>Anabolic Whey - GymBeam + darček 2500 g - čokoláda</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6841,22 +6841,22 @@
         <v>2500</v>
       </c>
       <c r="G107" t="n">
-        <v>45.95</v>
+        <v>59.95</v>
       </c>
       <c r="H107" t="n">
-        <v>18.38</v>
+        <v>23.98</v>
       </c>
       <c r="I107" t="n">
-        <v>0.4595</v>
+        <v>0.5995</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-isolate-gonutrition.html</t>
+          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6868,12 +6868,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Anabolic Whey - GymBeam + darček 1000 g - čokoláda</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="G108" t="n">
-        <v>27.95</v>
+        <v>15.95</v>
       </c>
       <c r="H108" t="n">
-        <v>27.95</v>
+        <v>39.875</v>
       </c>
       <c r="I108" t="n">
-        <v>0.69875</v>
+        <v>0.996875</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6917,12 +6917,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Anabolic Whey - GymBeam + darček 2500 g - čokoláda</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6936,16 +6936,16 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G109" t="n">
-        <v>59.95</v>
+        <v>33.95</v>
       </c>
       <c r="H109" t="n">
-        <v>23.98</v>
+        <v>33.95</v>
       </c>
       <c r="I109" t="n">
-        <v>0.5995</v>
+        <v>0.84875</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -6971,7 +6971,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6985,16 +6985,16 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G110" t="n">
-        <v>15.95</v>
+        <v>14.95</v>
       </c>
       <c r="H110" t="n">
-        <v>39.875</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I110" t="n">
-        <v>0.996875</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7034,16 +7034,16 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G111" t="n">
-        <v>33.95</v>
+        <v>18.5</v>
       </c>
       <c r="H111" t="n">
-        <v>33.95</v>
+        <v>37</v>
       </c>
       <c r="I111" t="n">
-        <v>0.84875</v>
+        <v>0.925</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7083,25 +7083,25 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G112" t="n">
-        <v>14.95</v>
+        <v>12.95</v>
       </c>
       <c r="H112" t="n">
-        <v>49.83333333333334</v>
+        <v>25.9</v>
       </c>
       <c r="I112" t="n">
-        <v>1.245833333333333</v>
+        <v>0.6475</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7132,16 +7132,16 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G113" t="n">
-        <v>18.5</v>
+        <v>23.95</v>
       </c>
       <c r="H113" t="n">
-        <v>37</v>
+        <v>23.95</v>
       </c>
       <c r="I113" t="n">
-        <v>0.925</v>
+        <v>0.59875</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7150,7 +7150,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7181,25 +7181,25 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G114" t="n">
-        <v>12.95</v>
+        <v>33.95</v>
       </c>
       <c r="H114" t="n">
-        <v>25.9</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I114" t="n">
-        <v>0.6475</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7230,16 +7230,16 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="G115" t="n">
-        <v>23.95</v>
+        <v>7.5</v>
       </c>
       <c r="H115" t="n">
-        <v>23.95</v>
+        <v>30</v>
       </c>
       <c r="I115" t="n">
-        <v>0.59875</v>
+        <v>0.75</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7279,16 +7279,16 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="G116" t="n">
-        <v>33.95</v>
+        <v>12.95</v>
       </c>
       <c r="H116" t="n">
-        <v>22.63333333333333</v>
+        <v>25.9</v>
       </c>
       <c r="I116" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.6475</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7328,16 +7328,16 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="G117" t="n">
-        <v>7.5</v>
+        <v>18.5</v>
       </c>
       <c r="H117" t="n">
-        <v>30</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I117" t="n">
-        <v>0.75</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7377,25 +7377,25 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G118" t="n">
-        <v>12.95</v>
+        <v>13.95</v>
       </c>
       <c r="H118" t="n">
-        <v>25.9</v>
+        <v>46.5</v>
       </c>
       <c r="I118" t="n">
-        <v>0.6475</v>
+        <v>1.1625</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7426,123 +7426,123 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>750</v>
+        <v>400</v>
       </c>
       <c r="G119" t="n">
-        <v>18.5</v>
+        <v>12.5</v>
       </c>
       <c r="H119" t="n">
-        <v>24.66666666666667</v>
+        <v>31.25</v>
       </c>
       <c r="I119" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.78125</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>protein_works</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>The Protein Works</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G120" t="n">
-        <v>13.95</v>
+        <v>34.99</v>
       </c>
       <c r="H120" t="n">
-        <v>46.5</v>
+        <v>69.98</v>
       </c>
       <c r="I120" t="n">
-        <v>1.1625</v>
+        <v>1.7495</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>protein_works</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>The Protein Works</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="G121" t="n">
-        <v>12.5</v>
+        <v>61.49</v>
       </c>
       <c r="H121" t="n">
-        <v>31.25</v>
+        <v>61.49</v>
       </c>
       <c r="I121" t="n">
-        <v>0.78125</v>
+        <v>1.53725</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7573,16 +7573,16 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G122" t="n">
-        <v>34.99</v>
+        <v>111.49</v>
       </c>
       <c r="H122" t="n">
-        <v>69.98</v>
+        <v>55.745</v>
       </c>
       <c r="I122" t="n">
-        <v>1.7495</v>
+        <v>1.393625</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -7622,20 +7622,20 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="G123" t="n">
-        <v>61.49</v>
+        <v>214.99</v>
       </c>
       <c r="H123" t="n">
-        <v>61.49</v>
+        <v>53.7475</v>
       </c>
       <c r="I123" t="n">
-        <v>1.53725</v>
+        <v>1.3436875</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7671,16 +7671,16 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G124" t="n">
-        <v>111.49</v>
+        <v>23.99</v>
       </c>
       <c r="H124" t="n">
-        <v>55.745</v>
+        <v>47.98</v>
       </c>
       <c r="I124" t="n">
-        <v>1.393625</v>
+        <v>1.1995</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7689,7 +7689,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -7720,25 +7720,25 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="G125" t="n">
-        <v>214.99</v>
+        <v>44.99</v>
       </c>
       <c r="H125" t="n">
-        <v>53.7475</v>
+        <v>44.99</v>
       </c>
       <c r="I125" t="n">
-        <v>1.3436875</v>
+        <v>1.12475</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7769,16 +7769,16 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="G126" t="n">
-        <v>23.99</v>
+        <v>17.99</v>
       </c>
       <c r="H126" t="n">
-        <v>47.98</v>
+        <v>29.98333333333333</v>
       </c>
       <c r="I126" t="n">
-        <v>1.1995</v>
+        <v>0.7495833333333334</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7818,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="G127" t="n">
-        <v>44.99</v>
+        <v>30.99</v>
       </c>
       <c r="H127" t="n">
-        <v>44.99</v>
+        <v>25.825</v>
       </c>
       <c r="I127" t="n">
-        <v>1.12475</v>
+        <v>0.645625</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>600</v>
+        <v>2400</v>
       </c>
       <c r="G128" t="n">
-        <v>17.99</v>
+        <v>48.99</v>
       </c>
       <c r="H128" t="n">
-        <v>29.98333333333333</v>
+        <v>20.4125</v>
       </c>
       <c r="I128" t="n">
-        <v>0.7495833333333334</v>
+        <v>0.5103124999999999</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>1200</v>
+        <v>4800</v>
       </c>
       <c r="G129" t="n">
-        <v>30.99</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="H129" t="n">
-        <v>25.825</v>
+        <v>19.58125</v>
       </c>
       <c r="I129" t="n">
-        <v>0.645625</v>
+        <v>0.48953125</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>2400</v>
+        <v>600</v>
       </c>
       <c r="G130" t="n">
-        <v>48.99</v>
+        <v>16.99</v>
       </c>
       <c r="H130" t="n">
-        <v>20.4125</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.5103124999999999</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>4800</v>
+        <v>1200</v>
       </c>
       <c r="G131" t="n">
-        <v>93.98999999999999</v>
+        <v>28.99</v>
       </c>
       <c r="H131" t="n">
-        <v>19.58125</v>
+        <v>24.15833333333333</v>
       </c>
       <c r="I131" t="n">
-        <v>0.48953125</v>
+        <v>0.6039583333333334</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8063,16 +8063,16 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>600</v>
+        <v>2400</v>
       </c>
       <c r="G132" t="n">
-        <v>16.99</v>
+        <v>48.99</v>
       </c>
       <c r="H132" t="n">
-        <v>28.31666666666667</v>
+        <v>20.4125</v>
       </c>
       <c r="I132" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.5103124999999999</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8112,16 +8112,16 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>1200</v>
+        <v>4800</v>
       </c>
       <c r="G133" t="n">
-        <v>28.99</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="H133" t="n">
-        <v>24.15833333333333</v>
+        <v>19.58125</v>
       </c>
       <c r="I133" t="n">
-        <v>0.6039583333333334</v>
+        <v>0.48953125</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8147,7 +8147,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -8161,16 +8161,16 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>2400</v>
+        <v>500</v>
       </c>
       <c r="G134" t="n">
-        <v>48.99</v>
+        <v>21.99</v>
       </c>
       <c r="H134" t="n">
-        <v>20.4125</v>
+        <v>43.98</v>
       </c>
       <c r="I134" t="n">
-        <v>0.5103124999999999</v>
+        <v>1.0995</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8196,7 +8196,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8210,16 +8210,16 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>4800</v>
+        <v>1000</v>
       </c>
       <c r="G135" t="n">
-        <v>93.98999999999999</v>
+        <v>38.99</v>
       </c>
       <c r="H135" t="n">
-        <v>19.58125</v>
+        <v>38.99</v>
       </c>
       <c r="I135" t="n">
-        <v>0.48953125</v>
+        <v>0.97475</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8259,16 +8259,16 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G136" t="n">
-        <v>21.99</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="H136" t="n">
-        <v>43.98</v>
+        <v>36.495</v>
       </c>
       <c r="I136" t="n">
-        <v>1.0995</v>
+        <v>0.912375</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8308,16 +8308,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="G137" t="n">
-        <v>38.99</v>
+        <v>141.99</v>
       </c>
       <c r="H137" t="n">
-        <v>38.99</v>
+        <v>35.4975</v>
       </c>
       <c r="I137" t="n">
-        <v>0.97475</v>
+        <v>0.8874375</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360 - Vanilla</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8357,16 +8357,16 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>2000</v>
+        <v>600</v>
       </c>
       <c r="G138" t="n">
-        <v>72.98999999999999</v>
+        <v>14.99</v>
       </c>
       <c r="H138" t="n">
-        <v>36.495</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I138" t="n">
-        <v>0.912375</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360 - Vanilla</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8406,16 +8406,16 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
       <c r="G139" t="n">
-        <v>141.99</v>
+        <v>25.99</v>
       </c>
       <c r="H139" t="n">
-        <v>35.4975</v>
+        <v>21.65833333333333</v>
       </c>
       <c r="I139" t="n">
-        <v>0.8874375</v>
+        <v>0.5414583333333334</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>
       </c>
     </row>
@@ -8455,16 +8455,16 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>600</v>
+        <v>2400</v>
       </c>
       <c r="G140" t="n">
-        <v>14.99</v>
+        <v>43.99</v>
       </c>
       <c r="H140" t="n">
-        <v>24.98333333333333</v>
+        <v>18.32916666666667</v>
       </c>
       <c r="I140" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.4582291666666667</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8504,16 +8504,16 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>1200</v>
+        <v>4800</v>
       </c>
       <c r="G141" t="n">
-        <v>25.99</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="H141" t="n">
-        <v>21.65833333333333</v>
+        <v>17.70625</v>
       </c>
       <c r="I141" t="n">
-        <v>0.5414583333333334</v>
+        <v>0.44265625</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8521,104 +8521,6 @@
         </is>
       </c>
       <c r="P141" t="inlineStr">
-        <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>protein_works</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>whey_protein</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Whey Protein 360 - Vanilla</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>The Protein Works</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="F142" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G142" t="n">
-        <v>43.99</v>
-      </c>
-      <c r="H142" t="n">
-        <v>18.32916666666667</v>
-      </c>
-      <c r="I142" t="n">
-        <v>0.4582291666666667</v>
-      </c>
-      <c r="O142" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P142" t="inlineStr">
-        <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>protein_works</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>whey_protein</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>Whey Protein 360 - Vanilla</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>The Protein Works</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="F143" t="n">
-        <v>4800</v>
-      </c>
-      <c r="G143" t="n">
-        <v>84.98999999999999</v>
-      </c>
-      <c r="H143" t="n">
-        <v>17.70625</v>
-      </c>
-      <c r="I143" t="n">
-        <v>0.44265625</v>
-      </c>
-      <c r="O143" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P143" t="inlineStr">
         <is>
           <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-20
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2085,16 +2085,16 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>500</v>
+        <v>2270</v>
       </c>
       <c r="G10" t="n">
-        <v>16.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>33.98</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8495</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2134,16 +2134,16 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G11" t="n">
-        <v>31.99</v>
+        <v>16.99</v>
       </c>
       <c r="H11" t="n">
-        <v>31.99</v>
+        <v>33.98</v>
       </c>
       <c r="I11" t="n">
-        <v>0.79975</v>
+        <v>0.8495</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2183,16 +2183,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G12" t="n">
-        <v>74.98999999999999</v>
+        <v>31.99</v>
       </c>
       <c r="H12" t="n">
-        <v>29.996</v>
+        <v>31.99</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7499</v>
+        <v>0.79975</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2232,16 +2232,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="G13" t="n">
-        <v>139.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>27.998</v>
+        <v>29.996</v>
       </c>
       <c r="I13" t="n">
-        <v>0.69995</v>
+        <v>0.7499</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2270</v>
+        <v>5000</v>
       </c>
       <c r="G14" t="n">
-        <v>79.98999999999999</v>
+        <v>139.99</v>
       </c>
       <c r="H14" t="n">
-        <v>35.23788546255506</v>
+        <v>27.998</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8809471365638767</v>
+        <v>0.69995</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pure Whey Protein + - Chocolate 450g</t>
+          <t>Pure Whey Protein+ - Chocolate 450g</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5479,7 +5479,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -7772,13 +7772,13 @@
         <v>600</v>
       </c>
       <c r="G126" t="n">
-        <v>17.99</v>
+        <v>16.99</v>
       </c>
       <c r="H126" t="n">
-        <v>29.98333333333333</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I126" t="n">
-        <v>0.7495833333333334</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7821,13 +7821,13 @@
         <v>1200</v>
       </c>
       <c r="G127" t="n">
-        <v>30.99</v>
+        <v>28.99</v>
       </c>
       <c r="H127" t="n">
-        <v>25.825</v>
+        <v>24.15833333333333</v>
       </c>
       <c r="I127" t="n">
-        <v>0.645625</v>
+        <v>0.6039583333333334</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7968,13 +7968,13 @@
         <v>600</v>
       </c>
       <c r="G130" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="H130" t="n">
-        <v>28.31666666666667</v>
+        <v>29.98333333333333</v>
       </c>
       <c r="I130" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.7495833333333334</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8017,13 +8017,13 @@
         <v>1200</v>
       </c>
       <c r="G131" t="n">
-        <v>28.99</v>
+        <v>30.99</v>
       </c>
       <c r="H131" t="n">
-        <v>24.15833333333333</v>
+        <v>25.825</v>
       </c>
       <c r="I131" t="n">
-        <v>0.6039583333333334</v>
+        <v>0.645625</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-21
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -5599,7 +5599,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam + darček 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam + darček 2000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam + darček 500 g - banán - 01</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -6606,7 +6606,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
@@ -7674,13 +7674,13 @@
         <v>500</v>
       </c>
       <c r="G124" t="n">
-        <v>23.99</v>
+        <v>19.99</v>
       </c>
       <c r="H124" t="n">
-        <v>47.98</v>
+        <v>39.98</v>
       </c>
       <c r="I124" t="n">
-        <v>1.1995</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7772,13 +7772,13 @@
         <v>600</v>
       </c>
       <c r="G126" t="n">
-        <v>16.99</v>
+        <v>17.49</v>
       </c>
       <c r="H126" t="n">
-        <v>28.31666666666667</v>
+        <v>29.15</v>
       </c>
       <c r="I126" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.72875</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7821,13 +7821,13 @@
         <v>1200</v>
       </c>
       <c r="G127" t="n">
-        <v>28.99</v>
+        <v>27.99</v>
       </c>
       <c r="H127" t="n">
-        <v>24.15833333333333</v>
+        <v>23.325</v>
       </c>
       <c r="I127" t="n">
-        <v>0.6039583333333334</v>
+        <v>0.583125</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7870,13 +7870,13 @@
         <v>2400</v>
       </c>
       <c r="G128" t="n">
-        <v>48.99</v>
+        <v>51.29</v>
       </c>
       <c r="H128" t="n">
-        <v>20.4125</v>
+        <v>21.37083333333333</v>
       </c>
       <c r="I128" t="n">
-        <v>0.5103124999999999</v>
+        <v>0.5342708333333334</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7919,13 +7919,13 @@
         <v>4800</v>
       </c>
       <c r="G129" t="n">
-        <v>93.98999999999999</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="H129" t="n">
-        <v>19.58125</v>
+        <v>20.47708333333333</v>
       </c>
       <c r="I129" t="n">
-        <v>0.48953125</v>
+        <v>0.5119270833333334</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7968,13 +7968,13 @@
         <v>600</v>
       </c>
       <c r="G130" t="n">
-        <v>17.99</v>
+        <v>19.29</v>
       </c>
       <c r="H130" t="n">
-        <v>29.98333333333333</v>
+        <v>32.15</v>
       </c>
       <c r="I130" t="n">
-        <v>0.7495833333333334</v>
+        <v>0.80375</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -8017,13 +8017,13 @@
         <v>1200</v>
       </c>
       <c r="G131" t="n">
-        <v>30.99</v>
+        <v>30.89</v>
       </c>
       <c r="H131" t="n">
-        <v>25.825</v>
+        <v>25.74166666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.645625</v>
+        <v>0.6435416666666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8066,13 +8066,13 @@
         <v>2400</v>
       </c>
       <c r="G132" t="n">
-        <v>48.99</v>
+        <v>56.69</v>
       </c>
       <c r="H132" t="n">
-        <v>20.4125</v>
+        <v>23.62083333333333</v>
       </c>
       <c r="I132" t="n">
-        <v>0.5103124999999999</v>
+        <v>0.5905208333333334</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8115,13 +8115,13 @@
         <v>4800</v>
       </c>
       <c r="G133" t="n">
-        <v>93.98999999999999</v>
+        <v>108.69</v>
       </c>
       <c r="H133" t="n">
-        <v>19.58125</v>
+        <v>22.64375</v>
       </c>
       <c r="I133" t="n">
-        <v>0.48953125</v>
+        <v>0.56609375</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8164,13 +8164,13 @@
         <v>500</v>
       </c>
       <c r="G134" t="n">
-        <v>21.99</v>
+        <v>17.99</v>
       </c>
       <c r="H134" t="n">
-        <v>43.98</v>
+        <v>35.98</v>
       </c>
       <c r="I134" t="n">
-        <v>1.0995</v>
+        <v>0.8995</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8213,13 +8213,13 @@
         <v>1000</v>
       </c>
       <c r="G135" t="n">
-        <v>38.99</v>
+        <v>31.99</v>
       </c>
       <c r="H135" t="n">
-        <v>38.99</v>
+        <v>31.99</v>
       </c>
       <c r="I135" t="n">
-        <v>0.97475</v>
+        <v>0.79975</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8262,13 +8262,13 @@
         <v>2000</v>
       </c>
       <c r="G136" t="n">
-        <v>72.98999999999999</v>
+        <v>58.99</v>
       </c>
       <c r="H136" t="n">
-        <v>36.495</v>
+        <v>29.495</v>
       </c>
       <c r="I136" t="n">
-        <v>0.912375</v>
+        <v>0.737375</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8311,13 +8311,13 @@
         <v>4000</v>
       </c>
       <c r="G137" t="n">
-        <v>141.99</v>
+        <v>114.99</v>
       </c>
       <c r="H137" t="n">
-        <v>35.4975</v>
+        <v>28.7475</v>
       </c>
       <c r="I137" t="n">
-        <v>0.8874375</v>
+        <v>0.7186875</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8360,13 +8360,13 @@
         <v>600</v>
       </c>
       <c r="G138" t="n">
-        <v>14.99</v>
+        <v>12.29</v>
       </c>
       <c r="H138" t="n">
-        <v>24.98333333333333</v>
+        <v>20.48333333333333</v>
       </c>
       <c r="I138" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.5120833333333333</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8409,13 +8409,13 @@
         <v>1200</v>
       </c>
       <c r="G139" t="n">
-        <v>25.99</v>
+        <v>22.49</v>
       </c>
       <c r="H139" t="n">
-        <v>21.65833333333333</v>
+        <v>18.74166666666667</v>
       </c>
       <c r="I139" t="n">
-        <v>0.5414583333333334</v>
+        <v>0.4685416666666667</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8458,13 +8458,13 @@
         <v>2400</v>
       </c>
       <c r="G140" t="n">
-        <v>43.99</v>
+        <v>42.49</v>
       </c>
       <c r="H140" t="n">
-        <v>18.32916666666667</v>
+        <v>17.70416666666667</v>
       </c>
       <c r="I140" t="n">
-        <v>0.4582291666666667</v>
+        <v>0.4426041666666667</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8507,13 +8507,13 @@
         <v>4800</v>
       </c>
       <c r="G141" t="n">
-        <v>84.98999999999999</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="H141" t="n">
-        <v>17.70625</v>
+        <v>17.28958333333333</v>
       </c>
       <c r="I141" t="n">
-        <v>0.44265625</v>
+        <v>0.4322395833333333</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-22
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2049,7 +2049,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3068,13 +3068,13 @@
         <v>500</v>
       </c>
       <c r="G30" t="n">
-        <v>21.99</v>
+        <v>15.99</v>
       </c>
       <c r="H30" t="n">
-        <v>43.98</v>
+        <v>31.98</v>
       </c>
       <c r="I30" t="n">
-        <v>1.0995</v>
+        <v>0.7995</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam + darček 1000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam + darček 2000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam + darček 500 g - banán - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-24
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -461,7 +461,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>143.48</v>
+        <v>148.16</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G30" t="n">
-        <v>15.99</v>
+        <v>18.99</v>
       </c>
       <c r="H30" t="n">
-        <v>31.98</v>
+        <v>15.192</v>
       </c>
       <c r="I30" t="n">
-        <v>0.7995</v>
+        <v>0.3798</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,25 +3114,25 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G31" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H31" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I31" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G32" t="n">
-        <v>18.99</v>
+        <v>15.99</v>
       </c>
       <c r="H32" t="n">
-        <v>15.192</v>
+        <v>31.98</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3798</v>
+        <v>0.7995</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3212,16 +3212,16 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G33" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H33" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I33" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3230,7 +3230,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -7772,13 +7772,13 @@
         <v>600</v>
       </c>
       <c r="G126" t="n">
-        <v>17.49</v>
+        <v>19.29</v>
       </c>
       <c r="H126" t="n">
-        <v>29.15</v>
+        <v>32.15</v>
       </c>
       <c r="I126" t="n">
-        <v>0.72875</v>
+        <v>0.80375</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7821,13 +7821,13 @@
         <v>1200</v>
       </c>
       <c r="G127" t="n">
-        <v>27.99</v>
+        <v>30.89</v>
       </c>
       <c r="H127" t="n">
-        <v>23.325</v>
+        <v>25.74166666666667</v>
       </c>
       <c r="I127" t="n">
-        <v>0.583125</v>
+        <v>0.6435416666666667</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7870,13 +7870,13 @@
         <v>2400</v>
       </c>
       <c r="G128" t="n">
-        <v>51.29</v>
+        <v>56.69</v>
       </c>
       <c r="H128" t="n">
-        <v>21.37083333333333</v>
+        <v>23.62083333333333</v>
       </c>
       <c r="I128" t="n">
-        <v>0.5342708333333334</v>
+        <v>0.5905208333333334</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7919,13 +7919,13 @@
         <v>4800</v>
       </c>
       <c r="G129" t="n">
-        <v>98.29000000000001</v>
+        <v>108.69</v>
       </c>
       <c r="H129" t="n">
-        <v>20.47708333333333</v>
+        <v>22.64375</v>
       </c>
       <c r="I129" t="n">
-        <v>0.5119270833333334</v>
+        <v>0.56609375</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7968,13 +7968,13 @@
         <v>600</v>
       </c>
       <c r="G130" t="n">
-        <v>19.29</v>
+        <v>17.49</v>
       </c>
       <c r="H130" t="n">
-        <v>32.15</v>
+        <v>29.15</v>
       </c>
       <c r="I130" t="n">
-        <v>0.80375</v>
+        <v>0.72875</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8017,13 +8017,13 @@
         <v>1200</v>
       </c>
       <c r="G131" t="n">
-        <v>30.89</v>
+        <v>27.99</v>
       </c>
       <c r="H131" t="n">
-        <v>25.74166666666667</v>
+        <v>23.325</v>
       </c>
       <c r="I131" t="n">
-        <v>0.6435416666666667</v>
+        <v>0.583125</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8066,13 +8066,13 @@
         <v>2400</v>
       </c>
       <c r="G132" t="n">
-        <v>56.69</v>
+        <v>51.29</v>
       </c>
       <c r="H132" t="n">
-        <v>23.62083333333333</v>
+        <v>21.37083333333333</v>
       </c>
       <c r="I132" t="n">
-        <v>0.5905208333333334</v>
+        <v>0.5342708333333334</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8115,13 +8115,13 @@
         <v>4800</v>
       </c>
       <c r="G133" t="n">
-        <v>108.69</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="H133" t="n">
-        <v>22.64375</v>
+        <v>20.47708333333333</v>
       </c>
       <c r="I133" t="n">
-        <v>0.56609375</v>
+        <v>0.5119270833333334</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-25
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2490,7 +2490,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G30" t="n">
-        <v>18.99</v>
+        <v>15.99</v>
       </c>
       <c r="H30" t="n">
-        <v>15.192</v>
+        <v>31.98</v>
       </c>
       <c r="I30" t="n">
-        <v>0.3798</v>
+        <v>0.7995</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,25 +3114,25 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G31" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H31" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G32" t="n">
-        <v>15.99</v>
+        <v>18.99</v>
       </c>
       <c r="H32" t="n">
-        <v>31.98</v>
+        <v>15.192</v>
       </c>
       <c r="I32" t="n">
-        <v>0.7995</v>
+        <v>0.3798</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3212,25 +3212,25 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G33" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H33" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I33" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
+          <t>Protein Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
+          <t>Protein Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7674,13 +7674,13 @@
         <v>500</v>
       </c>
       <c r="G124" t="n">
-        <v>19.99</v>
+        <v>23.99</v>
       </c>
       <c r="H124" t="n">
-        <v>39.98</v>
+        <v>47.98</v>
       </c>
       <c r="I124" t="n">
-        <v>0.9995000000000001</v>
+        <v>1.1995</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7772,13 +7772,13 @@
         <v>600</v>
       </c>
       <c r="G126" t="n">
-        <v>19.29</v>
+        <v>17.49</v>
       </c>
       <c r="H126" t="n">
-        <v>32.15</v>
+        <v>29.15</v>
       </c>
       <c r="I126" t="n">
-        <v>0.80375</v>
+        <v>0.72875</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7821,13 +7821,13 @@
         <v>1200</v>
       </c>
       <c r="G127" t="n">
-        <v>30.89</v>
+        <v>27.99</v>
       </c>
       <c r="H127" t="n">
-        <v>25.74166666666667</v>
+        <v>23.325</v>
       </c>
       <c r="I127" t="n">
-        <v>0.6435416666666667</v>
+        <v>0.583125</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7870,13 +7870,13 @@
         <v>2400</v>
       </c>
       <c r="G128" t="n">
-        <v>56.69</v>
+        <v>51.29</v>
       </c>
       <c r="H128" t="n">
-        <v>23.62083333333333</v>
+        <v>21.37083333333333</v>
       </c>
       <c r="I128" t="n">
-        <v>0.5905208333333334</v>
+        <v>0.5342708333333334</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7919,13 +7919,13 @@
         <v>4800</v>
       </c>
       <c r="G129" t="n">
-        <v>108.69</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="H129" t="n">
-        <v>22.64375</v>
+        <v>20.47708333333333</v>
       </c>
       <c r="I129" t="n">
-        <v>0.56609375</v>
+        <v>0.5119270833333334</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7968,13 +7968,13 @@
         <v>600</v>
       </c>
       <c r="G130" t="n">
-        <v>17.49</v>
+        <v>19.29</v>
       </c>
       <c r="H130" t="n">
-        <v>29.15</v>
+        <v>32.15</v>
       </c>
       <c r="I130" t="n">
-        <v>0.72875</v>
+        <v>0.80375</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8017,13 +8017,13 @@
         <v>1200</v>
       </c>
       <c r="G131" t="n">
-        <v>27.99</v>
+        <v>30.89</v>
       </c>
       <c r="H131" t="n">
-        <v>23.325</v>
+        <v>25.74166666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.583125</v>
+        <v>0.6435416666666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8066,13 +8066,13 @@
         <v>2400</v>
       </c>
       <c r="G132" t="n">
-        <v>51.29</v>
+        <v>56.69</v>
       </c>
       <c r="H132" t="n">
-        <v>21.37083333333333</v>
+        <v>23.62083333333333</v>
       </c>
       <c r="I132" t="n">
-        <v>0.5342708333333334</v>
+        <v>0.5905208333333334</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8115,13 +8115,13 @@
         <v>4800</v>
       </c>
       <c r="G133" t="n">
-        <v>98.29000000000001</v>
+        <v>108.69</v>
       </c>
       <c r="H133" t="n">
-        <v>20.47708333333333</v>
+        <v>22.64375</v>
       </c>
       <c r="I133" t="n">
-        <v>0.5119270833333334</v>
+        <v>0.56609375</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-27
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P145"/>
+  <dimension ref="A1:P143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2270</v>
+        <v>500</v>
       </c>
       <c r="G14" t="n">
-        <v>79.98999999999999</v>
+        <v>16.99</v>
       </c>
       <c r="H14" t="n">
-        <v>35.23788546255506</v>
+        <v>33.98</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8809471365638767</v>
+        <v>0.8495</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 500g</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2330,16 +2330,16 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G15" t="n">
-        <v>16.99</v>
+        <v>31.99</v>
       </c>
       <c r="H15" t="n">
-        <v>33.98</v>
+        <v>31.99</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8495</v>
+        <v>0.79975</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2379,16 +2379,16 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G16" t="n">
-        <v>31.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>31.99</v>
+        <v>29.996</v>
       </c>
       <c r="I16" t="n">
-        <v>0.79975</v>
+        <v>0.7499</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2428,16 +2428,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="G17" t="n">
-        <v>74.98999999999999</v>
+        <v>139.99</v>
       </c>
       <c r="H17" t="n">
-        <v>29.996</v>
+        <v>27.998</v>
       </c>
       <c r="I17" t="n">
-        <v>0.7499</v>
+        <v>0.69995</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Protein™ - Chocolate 5kg</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2477,16 +2477,16 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>5000</v>
+        <v>2270</v>
       </c>
       <c r="G18" t="n">
-        <v>139.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>27.998</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I18" t="n">
-        <v>0.69995</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-protein/bpb-npwp-0000</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>True Whey - GymBeam 1000 g - bez príchute - 01</t>
+          <t>Proteín True Whey - GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>True Whey - GymBeam 2500 g - bez príchute - 01</t>
+          <t>Proteín True Whey - GymBeam 2500 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ASAP True Whey - GymBeam 2000 g - banán</t>
+          <t>Proteín ASAP True Whey - GymBeam 2000 g - banán</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ASAP True Whey - GymBeam 900 g - banán</t>
+          <t>Proteín ASAP True Whey - GymBeam 900 g - banán</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Pure IsoWhey - GymBeam 1000 g - bez príchute - 01</t>
+          <t>Proteín Pure IsoWhey - GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Pure IsoWhey - GymBeam 2500 g - čokoláda - 00</t>
+          <t>Proteín Pure IsoWhey - GymBeam 2500 g - čokoláda - 00</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Protein Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Protein Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6040,7 +6040,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
+          <t>Proteín Anabolic Whey - GymBeam 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6057,13 +6057,13 @@
         <v>1000</v>
       </c>
       <c r="G91" t="n">
-        <v>31.95</v>
+        <v>27.95</v>
       </c>
       <c r="H91" t="n">
-        <v>31.95</v>
+        <v>27.95</v>
       </c>
       <c r="I91" t="n">
-        <v>0.79875</v>
+        <v>0.69875</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -6072,7 +6072,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
+          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 3000 g - vanilka</t>
+          <t>Proteín Anabolic Whey - GymBeam 2500 g - čokoláda</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6103,16 +6103,16 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="G92" t="n">
-        <v>93.95</v>
+        <v>59.95</v>
       </c>
       <c r="H92" t="n">
-        <v>31.31666666666667</v>
+        <v>23.98</v>
       </c>
       <c r="I92" t="n">
-        <v>0.7829166666666667</v>
+        <v>0.5995</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -6121,7 +6121,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
+          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
+          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6152,25 +6152,25 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G93" t="n">
-        <v>21.95</v>
+        <v>31.95</v>
       </c>
       <c r="H93" t="n">
-        <v>43.9</v>
+        <v>31.95</v>
       </c>
       <c r="I93" t="n">
-        <v>1.0975</v>
+        <v>0.79875</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
+          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
+          <t>Whey Proteín - Mammut Nutrition 3000 g - vanilka</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6201,25 +6201,25 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="G94" t="n">
-        <v>34.95</v>
+        <v>93.95</v>
       </c>
       <c r="H94" t="n">
-        <v>34.95</v>
+        <v>31.31666666666667</v>
       </c>
       <c r="I94" t="n">
-        <v>0.87375</v>
+        <v>0.7829166666666667</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
+          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6250,16 +6250,16 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G95" t="n">
-        <v>62.95</v>
+        <v>21.95</v>
       </c>
       <c r="H95" t="n">
-        <v>31.475</v>
+        <v>43.9</v>
       </c>
       <c r="I95" t="n">
-        <v>0.786875</v>
+        <v>1.0975</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
         </is>
       </c>
     </row>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
+          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6299,16 +6299,16 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G96" t="n">
-        <v>19.5</v>
+        <v>34.95</v>
       </c>
       <c r="H96" t="n">
-        <v>39</v>
+        <v>34.95</v>
       </c>
       <c r="I96" t="n">
-        <v>0.975</v>
+        <v>0.87375</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 1000 g - banán</t>
+          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6348,16 +6348,16 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G97" t="n">
-        <v>39.95</v>
+        <v>62.95</v>
       </c>
       <c r="H97" t="n">
-        <v>39.95</v>
+        <v>31.475</v>
       </c>
       <c r="I97" t="n">
-        <v>0.99875</v>
+        <v>0.786875</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 2000 g - banán</t>
+          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6397,16 +6397,16 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G98" t="n">
-        <v>64.95</v>
+        <v>19.5</v>
       </c>
       <c r="H98" t="n">
-        <v>32.475</v>
+        <v>39</v>
       </c>
       <c r="I98" t="n">
-        <v>0.811875</v>
+        <v>0.975</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6415,7 +6415,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
+          <t>Whey Protein - Bodylab24 1000 g - banán</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6446,16 +6446,16 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="G99" t="n">
-        <v>42.95</v>
+        <v>39.95</v>
       </c>
       <c r="H99" t="n">
-        <v>107.375</v>
+        <v>39.95</v>
       </c>
       <c r="I99" t="n">
-        <v>2.684375</v>
+        <v>0.99875</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
+          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
+          <t>Whey Protein - Bodylab24 2000 g - banán</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6495,16 +6495,16 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="G100" t="n">
-        <v>34.95</v>
+        <v>64.95</v>
       </c>
       <c r="H100" t="n">
-        <v>29.125</v>
+        <v>32.475</v>
       </c>
       <c r="I100" t="n">
-        <v>0.728125</v>
+        <v>0.811875</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6513,7 +6513,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
         </is>
       </c>
     </row>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
+          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6544,16 +6544,16 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>2400</v>
+        <v>400</v>
       </c>
       <c r="G101" t="n">
-        <v>62.95</v>
+        <v>42.95</v>
       </c>
       <c r="H101" t="n">
-        <v>26.22916666666667</v>
+        <v>107.375</v>
       </c>
       <c r="I101" t="n">
-        <v>0.6557291666666667</v>
+        <v>2.684375</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
+          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6593,16 +6593,16 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G102" t="n">
-        <v>19.5</v>
+        <v>34.95</v>
       </c>
       <c r="H102" t="n">
-        <v>32.5</v>
+        <v>29.125</v>
       </c>
       <c r="I102" t="n">
-        <v>0.8125</v>
+        <v>0.728125</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6642,16 +6642,16 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>1000</v>
+        <v>2400</v>
       </c>
       <c r="G103" t="n">
-        <v>16.5</v>
+        <v>62.95</v>
       </c>
       <c r="H103" t="n">
-        <v>16.5</v>
+        <v>26.22916666666667</v>
       </c>
       <c r="I103" t="n">
-        <v>0.4125</v>
+        <v>0.6557291666666667</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6677,7 +6677,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6691,16 +6691,16 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>2500</v>
+        <v>600</v>
       </c>
       <c r="G104" t="n">
-        <v>31.95</v>
+        <v>19.5</v>
       </c>
       <c r="H104" t="n">
-        <v>12.78</v>
+        <v>32.5</v>
       </c>
       <c r="I104" t="n">
-        <v>0.3195</v>
+        <v>0.8125</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -6709,7 +6709,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,16 +6740,16 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G105" t="n">
-        <v>11.95</v>
+        <v>16.5</v>
       </c>
       <c r="H105" t="n">
-        <v>23.9</v>
+        <v>16.5</v>
       </c>
       <c r="I105" t="n">
-        <v>0.5975</v>
+        <v>0.4125</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,16 +6789,16 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>1450</v>
+        <v>2500</v>
       </c>
       <c r="G106" t="n">
-        <v>39.95</v>
+        <v>31.95</v>
       </c>
       <c r="H106" t="n">
-        <v>27.55172413793104</v>
+        <v>12.78</v>
       </c>
       <c r="I106" t="n">
-        <v>0.6887931034482758</v>
+        <v>0.3195</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey + Isolate proteín s enzýmami DigeZyme® – GymBeam 1000 g - čokoláda</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,25 +6838,25 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G107" t="n">
-        <v>37.95</v>
+        <v>11.95</v>
       </c>
       <c r="H107" t="n">
-        <v>37.95</v>
+        <v>23.9</v>
       </c>
       <c r="I107" t="n">
-        <v>0.94875</v>
+        <v>0.5975</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-isolate-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Whey Protein Isolate 90 - GoNutrition banán - 1000 g</t>
+          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1000</v>
+        <v>1450</v>
       </c>
       <c r="G108" t="n">
-        <v>22.95</v>
+        <v>39.95</v>
       </c>
       <c r="H108" t="n">
-        <v>22.95</v>
+        <v>27.55172413793104</v>
       </c>
       <c r="I108" t="n">
-        <v>0.57375</v>
+        <v>0.6887931034482758</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-isolate-gonutrition.html</t>
+          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Whey Protein Isolate 90 - GoNutrition trojitá čokoláda - 2500 g</t>
+          <t>Whey + Isolate proteín s enzýmami DigeZyme® – GymBeam 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6936,25 +6936,25 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G109" t="n">
-        <v>45.95</v>
+        <v>37.95</v>
       </c>
       <c r="H109" t="n">
-        <v>18.38</v>
+        <v>37.95</v>
       </c>
       <c r="I109" t="n">
-        <v>0.4595</v>
+        <v>0.94875</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-isolate-gonutrition.html</t>
+          <t>https://gymbeam.sk/whey-isolate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6966,12 +6966,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Anabolic Whey - GymBeam + darček 1000 g - čokoláda</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6985,16 +6985,16 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="G110" t="n">
-        <v>27.95</v>
+        <v>15.95</v>
       </c>
       <c r="H110" t="n">
-        <v>27.95</v>
+        <v>39.875</v>
       </c>
       <c r="I110" t="n">
-        <v>0.69875</v>
+        <v>0.996875</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7015,12 +7015,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Anabolic Whey - GymBeam + darček 2500 g - čokoláda</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7034,16 +7034,16 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G111" t="n">
-        <v>59.95</v>
+        <v>33.95</v>
       </c>
       <c r="H111" t="n">
-        <v>23.98</v>
+        <v>33.95</v>
       </c>
       <c r="I111" t="n">
-        <v>0.5995</v>
+        <v>0.84875</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7083,16 +7083,16 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G112" t="n">
-        <v>15.95</v>
+        <v>14.95</v>
       </c>
       <c r="H112" t="n">
-        <v>39.875</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I112" t="n">
-        <v>0.996875</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7101,7 +7101,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7132,16 +7132,16 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G113" t="n">
-        <v>33.95</v>
+        <v>18.5</v>
       </c>
       <c r="H113" t="n">
-        <v>33.95</v>
+        <v>37</v>
       </c>
       <c r="I113" t="n">
-        <v>0.84875</v>
+        <v>0.925</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7181,25 +7181,25 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G114" t="n">
-        <v>14.95</v>
+        <v>12.95</v>
       </c>
       <c r="H114" t="n">
-        <v>49.83333333333334</v>
+        <v>25.9</v>
       </c>
       <c r="I114" t="n">
-        <v>1.245833333333333</v>
+        <v>0.6475</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7230,16 +7230,16 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G115" t="n">
-        <v>18.5</v>
+        <v>23.95</v>
       </c>
       <c r="H115" t="n">
-        <v>37</v>
+        <v>23.95</v>
       </c>
       <c r="I115" t="n">
-        <v>0.925</v>
+        <v>0.59875</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7248,7 +7248,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7279,25 +7279,25 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G116" t="n">
-        <v>12.95</v>
+        <v>33.95</v>
       </c>
       <c r="H116" t="n">
-        <v>25.9</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I116" t="n">
-        <v>0.6475</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7328,16 +7328,16 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="G117" t="n">
-        <v>23.95</v>
+        <v>7.5</v>
       </c>
       <c r="H117" t="n">
-        <v>23.95</v>
+        <v>30</v>
       </c>
       <c r="I117" t="n">
-        <v>0.59875</v>
+        <v>0.75</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7377,16 +7377,16 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="G118" t="n">
-        <v>33.95</v>
+        <v>12.95</v>
       </c>
       <c r="H118" t="n">
-        <v>22.63333333333333</v>
+        <v>25.9</v>
       </c>
       <c r="I118" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.6475</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="G119" t="n">
-        <v>7.5</v>
+        <v>18.5</v>
       </c>
       <c r="H119" t="n">
-        <v>30</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I119" t="n">
-        <v>0.75</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7475,25 +7475,25 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G120" t="n">
-        <v>12.95</v>
+        <v>13.95</v>
       </c>
       <c r="H120" t="n">
-        <v>25.9</v>
+        <v>46.5</v>
       </c>
       <c r="I120" t="n">
-        <v>0.6475</v>
+        <v>1.1625</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7524,123 +7524,123 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>750</v>
+        <v>400</v>
       </c>
       <c r="G121" t="n">
-        <v>18.5</v>
+        <v>12.5</v>
       </c>
       <c r="H121" t="n">
-        <v>24.66666666666667</v>
+        <v>31.25</v>
       </c>
       <c r="I121" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.78125</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>protein_works</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>The Protein Works</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G122" t="n">
-        <v>13.95</v>
+        <v>34.99</v>
       </c>
       <c r="H122" t="n">
-        <v>46.5</v>
+        <v>69.98</v>
       </c>
       <c r="I122" t="n">
-        <v>1.1625</v>
+        <v>1.7495</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>protein_works</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>The Protein Works</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="G123" t="n">
-        <v>12.5</v>
+        <v>61.49</v>
       </c>
       <c r="H123" t="n">
-        <v>31.25</v>
+        <v>61.49</v>
       </c>
       <c r="I123" t="n">
-        <v>0.78125</v>
+        <v>1.53725</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7671,16 +7671,16 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G124" t="n">
-        <v>34.99</v>
+        <v>111.49</v>
       </c>
       <c r="H124" t="n">
-        <v>69.98</v>
+        <v>55.745</v>
       </c>
       <c r="I124" t="n">
-        <v>1.7495</v>
+        <v>1.393625</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7720,20 +7720,20 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="G125" t="n">
-        <v>61.49</v>
+        <v>214.99</v>
       </c>
       <c r="H125" t="n">
-        <v>61.49</v>
+        <v>53.7475</v>
       </c>
       <c r="I125" t="n">
-        <v>1.53725</v>
+        <v>1.3436875</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7769,16 +7769,16 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G126" t="n">
-        <v>111.49</v>
+        <v>23.99</v>
       </c>
       <c r="H126" t="n">
-        <v>55.745</v>
+        <v>47.98</v>
       </c>
       <c r="I126" t="n">
-        <v>1.393625</v>
+        <v>1.1995</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7818,25 +7818,25 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="G127" t="n">
-        <v>214.99</v>
+        <v>44.99</v>
       </c>
       <c r="H127" t="n">
-        <v>53.7475</v>
+        <v>44.99</v>
       </c>
       <c r="I127" t="n">
-        <v>1.3436875</v>
+        <v>1.12475</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="G128" t="n">
-        <v>23.99</v>
+        <v>13.99</v>
       </c>
       <c r="H128" t="n">
-        <v>47.98</v>
+        <v>23.31666666666667</v>
       </c>
       <c r="I128" t="n">
-        <v>1.1995</v>
+        <v>0.5829166666666666</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="G129" t="n">
-        <v>44.99</v>
+        <v>22.29</v>
       </c>
       <c r="H129" t="n">
-        <v>44.99</v>
+        <v>18.575</v>
       </c>
       <c r="I129" t="n">
-        <v>1.12475</v>
+        <v>0.464375</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>600</v>
+        <v>2400</v>
       </c>
       <c r="G130" t="n">
-        <v>16.49</v>
+        <v>40.99</v>
       </c>
       <c r="H130" t="n">
-        <v>27.48333333333333</v>
+        <v>17.07916666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.6870833333333334</v>
+        <v>0.4269791666666667</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>1200</v>
+        <v>4800</v>
       </c>
       <c r="G131" t="n">
-        <v>26.49</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="H131" t="n">
-        <v>22.075</v>
+        <v>16.76875</v>
       </c>
       <c r="I131" t="n">
-        <v>0.551875</v>
+        <v>0.41921875</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8063,16 +8063,16 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>2400</v>
+        <v>600</v>
       </c>
       <c r="G132" t="n">
-        <v>47.99</v>
+        <v>14.99</v>
       </c>
       <c r="H132" t="n">
-        <v>19.99583333333333</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I132" t="n">
-        <v>0.4998958333333333</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8112,16 +8112,16 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>4800</v>
+        <v>1200</v>
       </c>
       <c r="G133" t="n">
-        <v>92.48999999999999</v>
+        <v>24.79</v>
       </c>
       <c r="H133" t="n">
-        <v>19.26875</v>
+        <v>20.65833333333333</v>
       </c>
       <c r="I133" t="n">
-        <v>0.48171875</v>
+        <v>0.5164583333333334</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8161,16 +8161,16 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>600</v>
+        <v>2400</v>
       </c>
       <c r="G134" t="n">
-        <v>17.99</v>
+        <v>45.49</v>
       </c>
       <c r="H134" t="n">
-        <v>29.98333333333333</v>
+        <v>18.95416666666667</v>
       </c>
       <c r="I134" t="n">
-        <v>0.7495833333333334</v>
+        <v>0.4738541666666667</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8210,16 +8210,16 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>1200</v>
+        <v>4800</v>
       </c>
       <c r="G135" t="n">
-        <v>29.49</v>
+        <v>88.98999999999999</v>
       </c>
       <c r="H135" t="n">
-        <v>24.575</v>
+        <v>18.53958333333333</v>
       </c>
       <c r="I135" t="n">
-        <v>0.614375</v>
+        <v>0.4634895833333333</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8245,7 +8245,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -8259,16 +8259,16 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>2400</v>
+        <v>500</v>
       </c>
       <c r="G136" t="n">
-        <v>53.49</v>
+        <v>17.99</v>
       </c>
       <c r="H136" t="n">
-        <v>22.2875</v>
+        <v>35.98</v>
       </c>
       <c r="I136" t="n">
-        <v>0.5571874999999999</v>
+        <v>0.8995</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -8308,16 +8308,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>4800</v>
+        <v>1000</v>
       </c>
       <c r="G137" t="n">
-        <v>102.49</v>
+        <v>31.99</v>
       </c>
       <c r="H137" t="n">
-        <v>21.35208333333333</v>
+        <v>31.99</v>
       </c>
       <c r="I137" t="n">
-        <v>0.5338020833333333</v>
+        <v>0.79975</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8357,16 +8357,16 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G138" t="n">
-        <v>17.99</v>
+        <v>58.99</v>
       </c>
       <c r="H138" t="n">
-        <v>35.98</v>
+        <v>29.495</v>
       </c>
       <c r="I138" t="n">
-        <v>0.8995</v>
+        <v>0.737375</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8406,16 +8406,16 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="G139" t="n">
-        <v>31.99</v>
+        <v>114.99</v>
       </c>
       <c r="H139" t="n">
-        <v>31.99</v>
+        <v>28.7475</v>
       </c>
       <c r="I139" t="n">
-        <v>0.79975</v>
+        <v>0.7186875</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360 - Vanilla</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8455,16 +8455,16 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>2000</v>
+        <v>600</v>
       </c>
       <c r="G140" t="n">
-        <v>58.99</v>
+        <v>11.49</v>
       </c>
       <c r="H140" t="n">
-        <v>29.495</v>
+        <v>19.15</v>
       </c>
       <c r="I140" t="n">
-        <v>0.737375</v>
+        <v>0.47875</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>
       </c>
     </row>
@@ -8490,7 +8490,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360 - Vanilla</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -8504,16 +8504,16 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
       <c r="G141" t="n">
-        <v>114.99</v>
+        <v>21.19</v>
       </c>
       <c r="H141" t="n">
-        <v>28.7475</v>
+        <v>17.65833333333333</v>
       </c>
       <c r="I141" t="n">
-        <v>0.7186875</v>
+        <v>0.4414583333333333</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8522,7 +8522,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>
       </c>
     </row>
@@ -8553,16 +8553,16 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>600</v>
+        <v>2400</v>
       </c>
       <c r="G142" t="n">
-        <v>11.49</v>
+        <v>39.99</v>
       </c>
       <c r="H142" t="n">
-        <v>19.15</v>
+        <v>16.6625</v>
       </c>
       <c r="I142" t="n">
-        <v>0.47875</v>
+        <v>0.4165625</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8602,16 +8602,16 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>1200</v>
+        <v>4800</v>
       </c>
       <c r="G143" t="n">
-        <v>21.19</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="H143" t="n">
-        <v>17.65833333333333</v>
+        <v>16.24791666666667</v>
       </c>
       <c r="I143" t="n">
-        <v>0.4414583333333333</v>
+        <v>0.4061979166666667</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -8619,104 +8619,6 @@
         </is>
       </c>
       <c r="P143" t="inlineStr">
-        <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>protein_works</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>whey_protein</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Whey Protein 360 - Vanilla</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>The Protein Works</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="F144" t="n">
-        <v>2400</v>
-      </c>
-      <c r="G144" t="n">
-        <v>39.99</v>
-      </c>
-      <c r="H144" t="n">
-        <v>16.6625</v>
-      </c>
-      <c r="I144" t="n">
-        <v>0.4165625</v>
-      </c>
-      <c r="O144" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P144" t="inlineStr">
-        <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>protein_works</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>whey_protein</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>Whey Protein 360 - Vanilla</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>The Protein Works</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="F145" t="n">
-        <v>4800</v>
-      </c>
-      <c r="G145" t="n">
-        <v>77.98999999999999</v>
-      </c>
-      <c r="H145" t="n">
-        <v>16.24791666666667</v>
-      </c>
-      <c r="I145" t="n">
-        <v>0.4061979166666667</v>
-      </c>
-      <c r="O145" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P145" t="inlineStr">
         <is>
           <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-28
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,25 +6740,25 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G105" t="n">
-        <v>16.5</v>
+        <v>28.95</v>
       </c>
       <c r="H105" t="n">
-        <v>16.5</v>
+        <v>57.9</v>
       </c>
       <c r="I105" t="n">
-        <v>0.4125</v>
+        <v>1.4475</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,16 +6789,16 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G106" t="n">
-        <v>31.95</v>
+        <v>16.5</v>
       </c>
       <c r="H106" t="n">
-        <v>12.78</v>
+        <v>16.5</v>
       </c>
       <c r="I106" t="n">
-        <v>0.3195</v>
+        <v>0.4125</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="G107" t="n">
-        <v>11.95</v>
+        <v>31.95</v>
       </c>
       <c r="H107" t="n">
-        <v>23.9</v>
+        <v>12.78</v>
       </c>
       <c r="I107" t="n">
-        <v>0.5975</v>
+        <v>0.3195</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1450</v>
+        <v>500</v>
       </c>
       <c r="G108" t="n">
-        <v>39.95</v>
+        <v>11.95</v>
       </c>
       <c r="H108" t="n">
-        <v>27.55172413793104</v>
+        <v>23.9</v>
       </c>
       <c r="I108" t="n">
-        <v>0.6887931034482758</v>
+        <v>0.5975</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Whey + Isolate proteín s enzýmami DigeZyme® – GymBeam 1000 g - čokoláda</t>
+          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6936,25 +6936,25 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>1000</v>
+        <v>1450</v>
       </c>
       <c r="G109" t="n">
-        <v>37.95</v>
+        <v>39.95</v>
       </c>
       <c r="H109" t="n">
-        <v>37.95</v>
+        <v>27.55172413793104</v>
       </c>
       <c r="I109" t="n">
-        <v>0.94875</v>
+        <v>0.6887931034482758</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-isolate-gymbeam.html</t>
+          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-30
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -484,7 +484,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>158.46</v>
+        <v>151.71</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -666,16 +666,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="G2" t="n">
-        <v>33.95</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>22.63333333333333</v>
+        <v>19.9</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.4975</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -715,16 +715,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G3" t="n">
-        <v>23.95</v>
+        <v>33.95</v>
       </c>
       <c r="H3" t="n">
-        <v>23.95</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I3" t="n">
-        <v>0.59875</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -764,16 +764,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="G4" t="n">
-        <v>18.5</v>
+        <v>5.95</v>
       </c>
       <c r="H4" t="n">
-        <v>24.66666666666667</v>
+        <v>23.8</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.595</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -799,30 +799,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
+          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1000</v>
       </c>
       <c r="G5" t="n">
-        <v>24.99</v>
+        <v>23.95</v>
       </c>
       <c r="H5" t="n">
-        <v>24.99</v>
+        <v>23.95</v>
       </c>
       <c r="I5" t="n">
-        <v>0.62475</v>
+        <v>0.59875</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -862,32 +862,32 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="G6" t="n">
-        <v>12.95</v>
+        <v>18.5</v>
       </c>
       <c r="H6" t="n">
-        <v>25.9</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6475</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -897,30 +897,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G7" t="n">
-        <v>12.95</v>
+        <v>24.99</v>
       </c>
       <c r="H7" t="n">
-        <v>25.9</v>
+        <v>24.99</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6475</v>
+        <v>0.62475</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -929,14 +929,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -946,39 +946,39 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>500</v>
       </c>
       <c r="G8" t="n">
-        <v>12.99</v>
+        <v>12.95</v>
       </c>
       <c r="H8" t="n">
-        <v>25.98</v>
+        <v>25.9</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6495</v>
+        <v>0.6475</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1009,16 +1009,16 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="G9" t="n">
-        <v>7.49</v>
+        <v>12.99</v>
       </c>
       <c r="H9" t="n">
-        <v>29.96</v>
+        <v>25.98</v>
       </c>
       <c r="I9" t="n">
-        <v>0.749</v>
+        <v>0.6495</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1034,7 +1034,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1044,30 +1044,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>250</v>
       </c>
       <c r="G10" t="n">
-        <v>7.5</v>
+        <v>7.49</v>
       </c>
       <c r="H10" t="n">
-        <v>30</v>
+        <v>29.96</v>
       </c>
       <c r="I10" t="n">
-        <v>0.75</v>
+        <v>0.749</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G34" t="n">
-        <v>18.99</v>
+        <v>15.99</v>
       </c>
       <c r="H34" t="n">
-        <v>15.192</v>
+        <v>31.98</v>
       </c>
       <c r="I34" t="n">
-        <v>0.3798</v>
+        <v>0.7995</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3310,25 +3310,25 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G35" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H35" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I35" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3359,16 +3359,16 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G36" t="n">
-        <v>15.99</v>
+        <v>18.99</v>
       </c>
       <c r="H36" t="n">
-        <v>31.98</v>
+        <v>15.192</v>
       </c>
       <c r="I36" t="n">
-        <v>0.7995</v>
+        <v>0.3798</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3408,25 +3408,25 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G37" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H37" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I37" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,25 +6740,25 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G105" t="n">
-        <v>28.95</v>
+        <v>16.5</v>
       </c>
       <c r="H105" t="n">
-        <v>57.9</v>
+        <v>16.5</v>
       </c>
       <c r="I105" t="n">
-        <v>1.4475</v>
+        <v>0.4125</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,16 +6789,16 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G106" t="n">
-        <v>16.5</v>
+        <v>31.95</v>
       </c>
       <c r="H106" t="n">
-        <v>16.5</v>
+        <v>12.78</v>
       </c>
       <c r="I106" t="n">
-        <v>0.4125</v>
+        <v>0.3195</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="G107" t="n">
-        <v>31.95</v>
+        <v>11.95</v>
       </c>
       <c r="H107" t="n">
-        <v>12.78</v>
+        <v>23.9</v>
       </c>
       <c r="I107" t="n">
-        <v>0.3195</v>
+        <v>0.5975</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6890,22 +6890,22 @@
         <v>500</v>
       </c>
       <c r="G108" t="n">
-        <v>11.95</v>
+        <v>28.95</v>
       </c>
       <c r="H108" t="n">
-        <v>23.9</v>
+        <v>57.9</v>
       </c>
       <c r="I108" t="n">
-        <v>0.5975</v>
+        <v>1.4475</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7331,13 +7331,13 @@
         <v>250</v>
       </c>
       <c r="G117" t="n">
-        <v>7.5</v>
+        <v>5.95</v>
       </c>
       <c r="H117" t="n">
-        <v>30</v>
+        <v>23.8</v>
       </c>
       <c r="I117" t="n">
-        <v>0.75</v>
+        <v>0.595</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7380,13 +7380,13 @@
         <v>500</v>
       </c>
       <c r="G118" t="n">
-        <v>12.95</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="H118" t="n">
-        <v>25.9</v>
+        <v>19.9</v>
       </c>
       <c r="I118" t="n">
-        <v>0.6475</v>
+        <v>0.4975</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-08-31
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1853,7 +1853,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G34" t="n">
-        <v>15.99</v>
+        <v>18.99</v>
       </c>
       <c r="H34" t="n">
-        <v>31.98</v>
+        <v>15.192</v>
       </c>
       <c r="I34" t="n">
-        <v>0.7995</v>
+        <v>0.3798</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3310,25 +3310,25 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G35" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H35" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I35" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3359,16 +3359,16 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G36" t="n">
-        <v>18.99</v>
+        <v>15.99</v>
       </c>
       <c r="H36" t="n">
-        <v>15.192</v>
+        <v>31.98</v>
       </c>
       <c r="I36" t="n">
-        <v>0.3798</v>
+        <v>0.7995</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3408,25 +3408,25 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G37" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H37" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I37" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-03
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -2490,7 +2490,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Clear Whey Protein - BeastPink 500 g - jahodová limonáda</t>
+          <t>Clear Whey Protein - BeastPink 500 g - citrón-limetka</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6691,25 +6691,25 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="G104" t="n">
-        <v>28.95</v>
+        <v>34.95</v>
       </c>
       <c r="H104" t="n">
-        <v>57.9</v>
+        <v>29.125</v>
       </c>
       <c r="I104" t="n">
-        <v>1.4475</v>
+        <v>0.728125</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,16 +6740,16 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G105" t="n">
-        <v>34.95</v>
+        <v>62.95</v>
       </c>
       <c r="H105" t="n">
-        <v>29.125</v>
+        <v>26.22916666666667</v>
       </c>
       <c r="I105" t="n">
-        <v>0.728125</v>
+        <v>0.6557291666666667</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
+          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,20 +6789,20 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>2400</v>
+        <v>600</v>
       </c>
       <c r="G106" t="n">
-        <v>62.95</v>
+        <v>19.5</v>
       </c>
       <c r="H106" t="n">
-        <v>26.22916666666667</v>
+        <v>32.5</v>
       </c>
       <c r="I106" t="n">
-        <v>0.6557291666666667</v>
+        <v>0.8125</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
+          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="G107" t="n">
-        <v>19.5</v>
+        <v>28.95</v>
       </c>
       <c r="H107" t="n">
-        <v>32.5</v>
+        <v>57.9</v>
       </c>
       <c r="I107" t="n">
-        <v>0.8125</v>
+        <v>1.4475</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
+          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -8360,13 +8360,13 @@
         <v>500</v>
       </c>
       <c r="G138" t="n">
-        <v>17.99</v>
+        <v>19.99</v>
       </c>
       <c r="H138" t="n">
-        <v>35.98</v>
+        <v>39.98</v>
       </c>
       <c r="I138" t="n">
-        <v>0.8995</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8409,13 +8409,13 @@
         <v>1000</v>
       </c>
       <c r="G139" t="n">
-        <v>31.99</v>
+        <v>33.99</v>
       </c>
       <c r="H139" t="n">
-        <v>31.99</v>
+        <v>33.99</v>
       </c>
       <c r="I139" t="n">
-        <v>0.79975</v>
+        <v>0.84975</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8458,13 +8458,13 @@
         <v>2000</v>
       </c>
       <c r="G140" t="n">
-        <v>58.99</v>
+        <v>63.49</v>
       </c>
       <c r="H140" t="n">
-        <v>29.495</v>
+        <v>31.745</v>
       </c>
       <c r="I140" t="n">
-        <v>0.737375</v>
+        <v>0.793625</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8507,13 +8507,13 @@
         <v>4000</v>
       </c>
       <c r="G141" t="n">
-        <v>114.99</v>
+        <v>119.49</v>
       </c>
       <c r="H141" t="n">
-        <v>28.7475</v>
+        <v>29.8725</v>
       </c>
       <c r="I141" t="n">
-        <v>0.7186875</v>
+        <v>0.7468125</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-04
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -449,19 +449,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>151.71</v>
+        <v>143.48</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -472,19 +472,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="C3" t="b">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>214.04</v>
+        <v>145.16</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -666,16 +666,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G2" t="n">
-        <v>9.949999999999999</v>
+        <v>33.95</v>
       </c>
       <c r="H2" t="n">
-        <v>19.9</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4975</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -715,16 +715,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="G3" t="n">
-        <v>33.95</v>
+        <v>23.95</v>
       </c>
       <c r="H3" t="n">
-        <v>22.63333333333333</v>
+        <v>23.95</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.59875</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -764,16 +764,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="G4" t="n">
-        <v>5.95</v>
+        <v>18.5</v>
       </c>
       <c r="H4" t="n">
-        <v>23.8</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I4" t="n">
-        <v>0.595</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -799,30 +799,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1000</v>
       </c>
       <c r="G5" t="n">
-        <v>23.95</v>
+        <v>24.99</v>
       </c>
       <c r="H5" t="n">
-        <v>23.95</v>
+        <v>24.99</v>
       </c>
       <c r="I5" t="n">
-        <v>0.59875</v>
+        <v>0.62475</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -862,32 +862,32 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="G6" t="n">
-        <v>18.5</v>
+        <v>12.95</v>
       </c>
       <c r="H6" t="n">
-        <v>24.66666666666667</v>
+        <v>25.9</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.6475</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -897,30 +897,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
+          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G7" t="n">
-        <v>24.99</v>
+        <v>12.95</v>
       </c>
       <c r="H7" t="n">
-        <v>24.99</v>
+        <v>25.9</v>
       </c>
       <c r="I7" t="n">
-        <v>0.62475</v>
+        <v>0.6475</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -929,14 +929,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -946,39 +946,39 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>500</v>
       </c>
       <c r="G8" t="n">
-        <v>12.95</v>
+        <v>12.99</v>
       </c>
       <c r="H8" t="n">
-        <v>25.9</v>
+        <v>25.98</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6475</v>
+        <v>0.6495</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1009,16 +1009,16 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G9" t="n">
-        <v>12.99</v>
+        <v>7.49</v>
       </c>
       <c r="H9" t="n">
-        <v>25.98</v>
+        <v>29.96</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6495</v>
+        <v>0.749</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1034,7 +1034,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1044,30 +1044,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>250</v>
       </c>
       <c r="G10" t="n">
-        <v>7.49</v>
+        <v>7.5</v>
       </c>
       <c r="H10" t="n">
-        <v>29.96</v>
+        <v>30</v>
       </c>
       <c r="I10" t="n">
-        <v>0.749</v>
+        <v>0.75</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3310,16 +3310,16 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G35" t="n">
-        <v>15.99</v>
+        <v>18.99</v>
       </c>
       <c r="H35" t="n">
-        <v>31.98</v>
+        <v>15.192</v>
       </c>
       <c r="I35" t="n">
-        <v>0.7995</v>
+        <v>0.3798</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3359,16 +3359,16 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G36" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H36" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I36" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3408,25 +3408,25 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G37" t="n">
-        <v>18.99</v>
+        <v>15.99</v>
       </c>
       <c r="H37" t="n">
-        <v>15.192</v>
+        <v>31.98</v>
       </c>
       <c r="I37" t="n">
-        <v>0.3798</v>
+        <v>0.7995</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3457,25 +3457,25 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G38" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H38" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I38" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -6155,13 +6155,13 @@
         <v>1000</v>
       </c>
       <c r="G93" t="n">
-        <v>27.95</v>
+        <v>21.95</v>
       </c>
       <c r="H93" t="n">
-        <v>27.95</v>
+        <v>21.95</v>
       </c>
       <c r="I93" t="n">
-        <v>0.69875</v>
+        <v>0.54875</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -6204,13 +6204,13 @@
         <v>2500</v>
       </c>
       <c r="G94" t="n">
-        <v>59.95</v>
+        <v>52.95</v>
       </c>
       <c r="H94" t="n">
-        <v>23.98</v>
+        <v>21.18</v>
       </c>
       <c r="I94" t="n">
-        <v>0.5995</v>
+        <v>0.5295</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1000 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7363,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 1500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 250 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7429,13 +7429,13 @@
         <v>250</v>
       </c>
       <c r="G119" t="n">
-        <v>5.95</v>
+        <v>7.5</v>
       </c>
       <c r="H119" t="n">
-        <v>23.8</v>
+        <v>30</v>
       </c>
       <c r="I119" t="n">
-        <v>0.595</v>
+        <v>0.75</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7478,13 +7478,13 @@
         <v>500</v>
       </c>
       <c r="G120" t="n">
-        <v>9.949999999999999</v>
+        <v>12.95</v>
       </c>
       <c r="H120" t="n">
-        <v>19.9</v>
+        <v>25.9</v>
       </c>
       <c r="I120" t="n">
-        <v>0.4975</v>
+        <v>0.6475</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>100% Mikronizovaný kreatín monohydrát 750 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7723,13 +7723,13 @@
         <v>1000</v>
       </c>
       <c r="G125" t="n">
-        <v>61.49</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="H125" t="n">
-        <v>61.49</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="I125" t="n">
-        <v>1.53725</v>
+        <v>1.72475</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -7772,13 +7772,13 @@
         <v>2000</v>
       </c>
       <c r="G126" t="n">
-        <v>111.49</v>
+        <v>129.49</v>
       </c>
       <c r="H126" t="n">
-        <v>55.745</v>
+        <v>64.745</v>
       </c>
       <c r="I126" t="n">
-        <v>1.393625</v>
+        <v>1.618625</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7821,13 +7821,13 @@
         <v>4000</v>
       </c>
       <c r="G127" t="n">
-        <v>214.99</v>
+        <v>245.99</v>
       </c>
       <c r="H127" t="n">
-        <v>53.7475</v>
+        <v>61.4975</v>
       </c>
       <c r="I127" t="n">
-        <v>1.3436875</v>
+        <v>1.5374375</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7968,13 +7968,13 @@
         <v>600</v>
       </c>
       <c r="G130" t="n">
-        <v>13.99</v>
+        <v>14.99</v>
       </c>
       <c r="H130" t="n">
-        <v>23.31666666666667</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I130" t="n">
-        <v>0.5829166666666666</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -8017,13 +8017,13 @@
         <v>1200</v>
       </c>
       <c r="G131" t="n">
-        <v>22.29</v>
+        <v>23.99</v>
       </c>
       <c r="H131" t="n">
-        <v>18.575</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.464375</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8066,13 +8066,13 @@
         <v>2400</v>
       </c>
       <c r="G132" t="n">
-        <v>40.99</v>
+        <v>44.49</v>
       </c>
       <c r="H132" t="n">
-        <v>17.07916666666667</v>
+        <v>18.5375</v>
       </c>
       <c r="I132" t="n">
-        <v>0.4269791666666667</v>
+        <v>0.4634375</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8115,13 +8115,13 @@
         <v>4800</v>
       </c>
       <c r="G133" t="n">
-        <v>80.48999999999999</v>
+        <v>84.48999999999999</v>
       </c>
       <c r="H133" t="n">
-        <v>16.76875</v>
+        <v>17.60208333333333</v>
       </c>
       <c r="I133" t="n">
-        <v>0.41921875</v>
+        <v>0.4400520833333333</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8164,13 +8164,13 @@
         <v>600</v>
       </c>
       <c r="G134" t="n">
-        <v>14.99</v>
+        <v>15.99</v>
       </c>
       <c r="H134" t="n">
-        <v>24.98333333333333</v>
+        <v>26.65</v>
       </c>
       <c r="I134" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.66625</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8213,13 +8213,13 @@
         <v>1200</v>
       </c>
       <c r="G135" t="n">
-        <v>24.79</v>
+        <v>26.99</v>
       </c>
       <c r="H135" t="n">
-        <v>20.65833333333333</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I135" t="n">
-        <v>0.5164583333333334</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8262,13 +8262,13 @@
         <v>2400</v>
       </c>
       <c r="G136" t="n">
-        <v>45.49</v>
+        <v>49.49</v>
       </c>
       <c r="H136" t="n">
-        <v>18.95416666666667</v>
+        <v>20.62083333333333</v>
       </c>
       <c r="I136" t="n">
-        <v>0.4738541666666667</v>
+        <v>0.5155208333333333</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8311,13 +8311,13 @@
         <v>4800</v>
       </c>
       <c r="G137" t="n">
-        <v>88.98999999999999</v>
+        <v>93.48999999999999</v>
       </c>
       <c r="H137" t="n">
-        <v>18.53958333333333</v>
+        <v>19.47708333333333</v>
       </c>
       <c r="I137" t="n">
-        <v>0.4634895833333333</v>
+        <v>0.4869270833333333</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8703,13 +8703,13 @@
         <v>4800</v>
       </c>
       <c r="G145" t="n">
-        <v>77.98999999999999</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="H145" t="n">
-        <v>16.24791666666667</v>
+        <v>16.14375</v>
       </c>
       <c r="I145" t="n">
-        <v>0.4061979166666667</v>
+        <v>0.40359375</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-05
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P145"/>
+  <dimension ref="A1:P144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1794,13 +1794,13 @@
         <v>5000</v>
       </c>
       <c r="G4" t="n">
-        <v>139.99</v>
+        <v>144.99</v>
       </c>
       <c r="H4" t="n">
-        <v>27.998</v>
+        <v>28.998</v>
       </c>
       <c r="I4" t="n">
-        <v>0.69995</v>
+        <v>0.72495</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pure Whey Isolate™ Unflavoured 450g</t>
+          <t>Pure Whey Isolate™ Chocolate Caramel 450g</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2725,13 +2725,13 @@
         <v>2000</v>
       </c>
       <c r="G23" t="n">
-        <v>49.99</v>
+        <v>52.99</v>
       </c>
       <c r="H23" t="n">
-        <v>24.995</v>
+        <v>26.495</v>
       </c>
       <c r="I23" t="n">
-        <v>0.624875</v>
+        <v>0.662375</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -4146,13 +4146,13 @@
         <v>2000</v>
       </c>
       <c r="G52" t="n">
-        <v>87.95</v>
+        <v>73.95</v>
       </c>
       <c r="H52" t="n">
-        <v>43.975</v>
+        <v>36.975</v>
       </c>
       <c r="I52" t="n">
-        <v>1.099375</v>
+        <v>0.9243749999999999</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -4195,13 +4195,13 @@
         <v>900</v>
       </c>
       <c r="G53" t="n">
-        <v>44.95</v>
+        <v>37.95</v>
       </c>
       <c r="H53" t="n">
-        <v>49.94444444444444</v>
+        <v>42.16666666666666</v>
       </c>
       <c r="I53" t="n">
-        <v>1.248611111111111</v>
+        <v>1.054166666666667</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,25 +6838,25 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G107" t="n">
-        <v>28.95</v>
+        <v>16.5</v>
       </c>
       <c r="H107" t="n">
-        <v>57.9</v>
+        <v>16.5</v>
       </c>
       <c r="I107" t="n">
-        <v>1.4475</v>
+        <v>0.4125</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G108" t="n">
-        <v>16.5</v>
+        <v>31.95</v>
       </c>
       <c r="H108" t="n">
-        <v>16.5</v>
+        <v>12.78</v>
       </c>
       <c r="I108" t="n">
-        <v>0.4125</v>
+        <v>0.3195</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6936,16 +6936,16 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="G109" t="n">
-        <v>31.95</v>
+        <v>11.95</v>
       </c>
       <c r="H109" t="n">
-        <v>12.78</v>
+        <v>23.9</v>
       </c>
       <c r="I109" t="n">
-        <v>0.3195</v>
+        <v>0.5975</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -6971,7 +6971,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6985,16 +6985,16 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>500</v>
+        <v>1450</v>
       </c>
       <c r="G110" t="n">
-        <v>11.95</v>
+        <v>29.95</v>
       </c>
       <c r="H110" t="n">
-        <v>23.9</v>
+        <v>20.6551724137931</v>
       </c>
       <c r="I110" t="n">
-        <v>0.5975</v>
+        <v>0.5163793103448275</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7015,12 +7015,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7034,25 +7034,25 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>1450</v>
+        <v>400</v>
       </c>
       <c r="G111" t="n">
-        <v>39.95</v>
+        <v>15.95</v>
       </c>
       <c r="H111" t="n">
-        <v>27.55172413793104</v>
+        <v>39.875</v>
       </c>
       <c r="I111" t="n">
-        <v>0.6887931034482758</v>
+        <v>0.996875</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7083,16 +7083,16 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="G112" t="n">
-        <v>15.95</v>
+        <v>33.95</v>
       </c>
       <c r="H112" t="n">
-        <v>39.875</v>
+        <v>33.95</v>
       </c>
       <c r="I112" t="n">
-        <v>0.996875</v>
+        <v>0.84875</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7101,7 +7101,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7132,16 +7132,16 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="G113" t="n">
-        <v>33.95</v>
+        <v>14.95</v>
       </c>
       <c r="H113" t="n">
-        <v>33.95</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I113" t="n">
-        <v>0.84875</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7181,16 +7181,16 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G114" t="n">
-        <v>14.95</v>
+        <v>18.5</v>
       </c>
       <c r="H114" t="n">
-        <v>49.83333333333334</v>
+        <v>37</v>
       </c>
       <c r="I114" t="n">
-        <v>1.245833333333333</v>
+        <v>0.925</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7233,22 +7233,22 @@
         <v>500</v>
       </c>
       <c r="G115" t="n">
-        <v>18.5</v>
+        <v>12.95</v>
       </c>
       <c r="H115" t="n">
-        <v>37</v>
+        <v>25.9</v>
       </c>
       <c r="I115" t="n">
-        <v>0.925</v>
+        <v>0.6475</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7279,25 +7279,25 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G116" t="n">
-        <v>12.95</v>
+        <v>23.95</v>
       </c>
       <c r="H116" t="n">
-        <v>25.9</v>
+        <v>23.95</v>
       </c>
       <c r="I116" t="n">
-        <v>0.6475</v>
+        <v>0.59875</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7328,16 +7328,16 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G117" t="n">
-        <v>23.95</v>
+        <v>33.95</v>
       </c>
       <c r="H117" t="n">
-        <v>23.95</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I117" t="n">
-        <v>0.59875</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7377,16 +7377,16 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>1500</v>
+        <v>250</v>
       </c>
       <c r="G118" t="n">
-        <v>33.95</v>
+        <v>7.5</v>
       </c>
       <c r="H118" t="n">
-        <v>22.63333333333333</v>
+        <v>30</v>
       </c>
       <c r="I118" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.75</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="G119" t="n">
-        <v>7.5</v>
+        <v>12.95</v>
       </c>
       <c r="H119" t="n">
-        <v>30</v>
+        <v>25.9</v>
       </c>
       <c r="I119" t="n">
-        <v>0.75</v>
+        <v>0.6475</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7475,16 +7475,16 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="G120" t="n">
-        <v>12.95</v>
+        <v>18.5</v>
       </c>
       <c r="H120" t="n">
-        <v>25.9</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I120" t="n">
-        <v>0.6475</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7524,25 +7524,25 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>750</v>
+        <v>300</v>
       </c>
       <c r="G121" t="n">
-        <v>18.5</v>
+        <v>13.95</v>
       </c>
       <c r="H121" t="n">
-        <v>24.66666666666667</v>
+        <v>46.5</v>
       </c>
       <c r="I121" t="n">
-        <v>0.6166666666666667</v>
+        <v>1.1625</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
@@ -7559,7 +7559,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7573,16 +7573,16 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="G122" t="n">
-        <v>13.95</v>
+        <v>12.5</v>
       </c>
       <c r="H122" t="n">
-        <v>46.5</v>
+        <v>31.25</v>
       </c>
       <c r="I122" t="n">
-        <v>1.1625</v>
+        <v>0.78125</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -7591,56 +7591,56 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>protein_works</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>The Protein Works</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="G123" t="n">
-        <v>12.5</v>
+        <v>34.99</v>
       </c>
       <c r="H123" t="n">
-        <v>31.25</v>
+        <v>69.98</v>
       </c>
       <c r="I123" t="n">
-        <v>0.78125</v>
+        <v>1.7495</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7671,16 +7671,16 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G124" t="n">
-        <v>34.99</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="H124" t="n">
-        <v>69.98</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="I124" t="n">
-        <v>1.7495</v>
+        <v>1.72475</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7720,16 +7720,16 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G125" t="n">
-        <v>68.98999999999999</v>
+        <v>129.49</v>
       </c>
       <c r="H125" t="n">
-        <v>68.98999999999999</v>
+        <v>64.745</v>
       </c>
       <c r="I125" t="n">
-        <v>1.72475</v>
+        <v>1.618625</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -7769,20 +7769,20 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="G126" t="n">
-        <v>129.49</v>
+        <v>245.99</v>
       </c>
       <c r="H126" t="n">
-        <v>64.745</v>
+        <v>61.4975</v>
       </c>
       <c r="I126" t="n">
-        <v>1.618625</v>
+        <v>1.5374375</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -7804,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7818,25 +7818,25 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>4000</v>
+        <v>500</v>
       </c>
       <c r="G127" t="n">
-        <v>245.99</v>
+        <v>23.99</v>
       </c>
       <c r="H127" t="n">
-        <v>61.4975</v>
+        <v>47.98</v>
       </c>
       <c r="I127" t="n">
-        <v>1.5374375</v>
+        <v>1.1995</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G128" t="n">
-        <v>23.99</v>
+        <v>44.99</v>
       </c>
       <c r="H128" t="n">
-        <v>47.98</v>
+        <v>44.99</v>
       </c>
       <c r="I128" t="n">
-        <v>1.1995</v>
+        <v>1.12475</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="G129" t="n">
-        <v>44.99</v>
+        <v>14.99</v>
       </c>
       <c r="H129" t="n">
-        <v>44.99</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I129" t="n">
-        <v>1.12475</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G130" t="n">
-        <v>14.99</v>
+        <v>23.99</v>
       </c>
       <c r="H130" t="n">
-        <v>24.98333333333333</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G131" t="n">
-        <v>23.99</v>
+        <v>44.49</v>
       </c>
       <c r="H131" t="n">
-        <v>19.99166666666667</v>
+        <v>18.5375</v>
       </c>
       <c r="I131" t="n">
-        <v>0.4997916666666667</v>
+        <v>0.4634375</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8063,16 +8063,16 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G132" t="n">
-        <v>44.49</v>
+        <v>84.48999999999999</v>
       </c>
       <c r="H132" t="n">
-        <v>18.5375</v>
+        <v>17.60208333333333</v>
       </c>
       <c r="I132" t="n">
-        <v>0.4634375</v>
+        <v>0.4400520833333333</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8112,16 +8112,16 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>4800</v>
+        <v>600</v>
       </c>
       <c r="G133" t="n">
-        <v>84.48999999999999</v>
+        <v>15.99</v>
       </c>
       <c r="H133" t="n">
-        <v>17.60208333333333</v>
+        <v>26.65</v>
       </c>
       <c r="I133" t="n">
-        <v>0.4400520833333333</v>
+        <v>0.66625</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8161,16 +8161,16 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G134" t="n">
-        <v>15.99</v>
+        <v>26.99</v>
       </c>
       <c r="H134" t="n">
-        <v>26.65</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I134" t="n">
-        <v>0.66625</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8210,16 +8210,16 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G135" t="n">
-        <v>26.99</v>
+        <v>49.49</v>
       </c>
       <c r="H135" t="n">
-        <v>22.49166666666667</v>
+        <v>20.62083333333333</v>
       </c>
       <c r="I135" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.5155208333333333</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8259,16 +8259,16 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G136" t="n">
-        <v>49.49</v>
+        <v>93.48999999999999</v>
       </c>
       <c r="H136" t="n">
-        <v>20.62083333333333</v>
+        <v>19.47708333333333</v>
       </c>
       <c r="I136" t="n">
-        <v>0.5155208333333333</v>
+        <v>0.4869270833333333</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -8308,16 +8308,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>4800</v>
+        <v>500</v>
       </c>
       <c r="G137" t="n">
-        <v>93.48999999999999</v>
+        <v>19.99</v>
       </c>
       <c r="H137" t="n">
-        <v>19.47708333333333</v>
+        <v>39.98</v>
       </c>
       <c r="I137" t="n">
-        <v>0.4869270833333333</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8357,16 +8357,16 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G138" t="n">
-        <v>19.99</v>
+        <v>33.99</v>
       </c>
       <c r="H138" t="n">
-        <v>39.98</v>
+        <v>33.99</v>
       </c>
       <c r="I138" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.84975</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8406,16 +8406,16 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G139" t="n">
-        <v>33.99</v>
+        <v>63.49</v>
       </c>
       <c r="H139" t="n">
-        <v>33.99</v>
+        <v>31.745</v>
       </c>
       <c r="I139" t="n">
-        <v>0.84975</v>
+        <v>0.793625</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8455,16 +8455,16 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="G140" t="n">
-        <v>63.49</v>
+        <v>119.49</v>
       </c>
       <c r="H140" t="n">
-        <v>31.745</v>
+        <v>29.8725</v>
       </c>
       <c r="I140" t="n">
-        <v>0.793625</v>
+        <v>0.7468125</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8490,7 +8490,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360 - Vanilla</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -8504,16 +8504,16 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>4000</v>
+        <v>600</v>
       </c>
       <c r="G141" t="n">
-        <v>119.49</v>
+        <v>11.49</v>
       </c>
       <c r="H141" t="n">
-        <v>29.8725</v>
+        <v>19.15</v>
       </c>
       <c r="I141" t="n">
-        <v>0.7468125</v>
+        <v>0.47875</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8522,7 +8522,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>
       </c>
     </row>
@@ -8553,16 +8553,16 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G142" t="n">
-        <v>11.49</v>
+        <v>21.19</v>
       </c>
       <c r="H142" t="n">
-        <v>19.15</v>
+        <v>17.65833333333333</v>
       </c>
       <c r="I142" t="n">
-        <v>0.47875</v>
+        <v>0.4414583333333333</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8602,16 +8602,16 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G143" t="n">
-        <v>21.19</v>
+        <v>39.99</v>
       </c>
       <c r="H143" t="n">
-        <v>17.65833333333333</v>
+        <v>16.6625</v>
       </c>
       <c r="I143" t="n">
-        <v>0.4414583333333333</v>
+        <v>0.4165625</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -8651,16 +8651,16 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G144" t="n">
-        <v>39.99</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="H144" t="n">
-        <v>16.6625</v>
+        <v>16.14375</v>
       </c>
       <c r="I144" t="n">
-        <v>0.4165625</v>
+        <v>0.40359375</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -8668,55 +8668,6 @@
         </is>
       </c>
       <c r="P144" t="inlineStr">
-        <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>protein_works</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>whey_protein</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>Whey Protein 360 - Vanilla</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>The Protein Works</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="F145" t="n">
-        <v>4800</v>
-      </c>
-      <c r="G145" t="n">
-        <v>77.48999999999999</v>
-      </c>
-      <c r="H145" t="n">
-        <v>16.14375</v>
-      </c>
-      <c r="I145" t="n">
-        <v>0.40359375</v>
-      </c>
-      <c r="O145" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P145" t="inlineStr">
         <is>
           <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-06
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -985,7 +985,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -995,30 +995,30 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="G9" t="n">
-        <v>7.49</v>
+        <v>10.95</v>
       </c>
       <c r="H9" t="n">
-        <v>29.96</v>
+        <v>27.375</v>
       </c>
       <c r="I9" t="n">
-        <v>0.749</v>
+        <v>0.684375</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1027,14 +1027,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1044,30 +1044,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>250</v>
       </c>
       <c r="G10" t="n">
-        <v>7.5</v>
+        <v>7.49</v>
       </c>
       <c r="H10" t="n">
-        <v>30</v>
+        <v>29.96</v>
       </c>
       <c r="I10" t="n">
-        <v>0.75</v>
+        <v>0.749</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1107,25 +1107,25 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="G11" t="n">
-        <v>12.5</v>
+        <v>7.5</v>
       </c>
       <c r="H11" t="n">
-        <v>31.25</v>
+        <v>30</v>
       </c>
       <c r="I11" t="n">
-        <v>0.78125</v>
+        <v>0.75</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1156,25 +1156,25 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="G12" t="n">
-        <v>33.95</v>
+        <v>12.5</v>
       </c>
       <c r="H12" t="n">
-        <v>33.95</v>
+        <v>31.25</v>
       </c>
       <c r="I12" t="n">
-        <v>0.84875</v>
+        <v>0.78125</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1205,16 +1205,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G13" t="n">
-        <v>18.5</v>
+        <v>33.95</v>
       </c>
       <c r="H13" t="n">
-        <v>37</v>
+        <v>33.95</v>
       </c>
       <c r="I13" t="n">
-        <v>0.925</v>
+        <v>0.84875</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1254,16 +1254,16 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="G14" t="n">
-        <v>15.95</v>
+        <v>18.5</v>
       </c>
       <c r="H14" t="n">
-        <v>39.875</v>
+        <v>37</v>
       </c>
       <c r="I14" t="n">
-        <v>0.996875</v>
+        <v>0.925</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -7037,13 +7037,13 @@
         <v>400</v>
       </c>
       <c r="G111" t="n">
-        <v>15.95</v>
+        <v>10.95</v>
       </c>
       <c r="H111" t="n">
-        <v>39.875</v>
+        <v>27.375</v>
       </c>
       <c r="I111" t="n">
-        <v>0.996875</v>
+        <v>0.684375</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-08
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P144"/>
+  <dimension ref="A1:P143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pure Whey Protein™ - Lemon &amp; Coconut 500g </t>
+          <t>Clear Whey Isolate - Apple &amp; Blackcurrant 500g</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2970,22 +2970,22 @@
         <v>500</v>
       </c>
       <c r="G28" t="n">
-        <v>18.99</v>
+        <v>25.99</v>
       </c>
       <c r="H28" t="n">
-        <v>37.98</v>
+        <v>51.98</v>
       </c>
       <c r="I28" t="n">
-        <v>0.9495</v>
+        <v>1.2995</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/pure-whey-protein-lemon-coconut-500/bpb-wpc8-lcoc-0500</t>
+          <t>https://www.bulk.com/uk/products/clear-whey-isolate/bpb-cwhe</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Clear Whey Isolate - Apple &amp; Blackcurrant 500g</t>
+          <t>Clear Whey Isolate - Strawberry &amp; Watermelon 1kg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3016,16 +3016,16 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G29" t="n">
-        <v>25.99</v>
+        <v>49.99</v>
       </c>
       <c r="H29" t="n">
-        <v>51.98</v>
+        <v>49.99</v>
       </c>
       <c r="I29" t="n">
-        <v>1.2995</v>
+        <v>1.24975</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Clear Whey Isolate - Strawberry &amp; Watermelon 1kg</t>
+          <t>Clear Whey Isolate - Peach Iced Tea 2kg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3065,16 +3065,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G30" t="n">
-        <v>49.99</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="H30" t="n">
-        <v>49.99</v>
+        <v>47.495</v>
       </c>
       <c r="I30" t="n">
-        <v>1.24975</v>
+        <v>1.187375</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Clear Whey Isolate - Peach Iced Tea 2kg</t>
+          <t>Hydrolysed Whey Protein Isolate - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3114,16 +3114,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G31" t="n">
-        <v>94.98999999999999</v>
+        <v>27.99</v>
       </c>
       <c r="H31" t="n">
-        <v>47.495</v>
+        <v>55.98</v>
       </c>
       <c r="I31" t="n">
-        <v>1.187375</v>
+        <v>1.3995</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/clear-whey-isolate/bpb-cwhe</t>
+          <t>https://www.bulk.com/uk/products/hydrolysed-whey-protein-isolate/bpb-hwpi-0000</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hydrolysed Whey Protein Isolate - Unflavoured 500g</t>
+          <t>Hydrolysed Whey Protein Isolate - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3163,16 +3163,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G32" t="n">
-        <v>27.99</v>
+        <v>49.99</v>
       </c>
       <c r="H32" t="n">
-        <v>55.98</v>
+        <v>49.99</v>
       </c>
       <c r="I32" t="n">
-        <v>1.3995</v>
+        <v>1.24975</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Hydrolysed Whey Protein Isolate - Unflavoured 1kg</t>
+          <t>Hydrolysed Whey Protein Isolate - Unflavoured 2.5kg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3212,16 +3212,16 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G33" t="n">
-        <v>49.99</v>
+        <v>119.99</v>
       </c>
       <c r="H33" t="n">
-        <v>49.99</v>
+        <v>47.996</v>
       </c>
       <c r="I33" t="n">
-        <v>1.24975</v>
+        <v>1.1999</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Hydrolysed Whey Protein Isolate - Unflavoured 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="G34" t="n">
-        <v>119.99</v>
+        <v>15.99</v>
       </c>
       <c r="H34" t="n">
-        <v>47.996</v>
+        <v>31.98</v>
       </c>
       <c r="I34" t="n">
-        <v>1.1999</v>
+        <v>0.7995</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/hydrolysed-whey-protein-isolate/bpb-hwpi-0000</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3310,16 +3310,16 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="G35" t="n">
-        <v>18.99</v>
+        <v>39.99</v>
       </c>
       <c r="H35" t="n">
-        <v>15.192</v>
+        <v>39.99</v>
       </c>
       <c r="I35" t="n">
-        <v>0.3798</v>
+        <v>0.99975</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3359,16 +3359,16 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2500</v>
+        <v>1250</v>
       </c>
       <c r="G36" t="n">
-        <v>35.99</v>
+        <v>18.99</v>
       </c>
       <c r="H36" t="n">
-        <v>14.396</v>
+        <v>15.192</v>
       </c>
       <c r="I36" t="n">
-        <v>0.3599</v>
+        <v>0.3798</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3408,16 +3408,16 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="G37" t="n">
-        <v>15.99</v>
+        <v>35.99</v>
       </c>
       <c r="H37" t="n">
-        <v>31.98</v>
+        <v>14.396</v>
       </c>
       <c r="I37" t="n">
-        <v>0.7995</v>
+        <v>0.3599</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Whey Protein Coffee - Iced Caramel Latte 500g</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3457,16 +3457,16 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G38" t="n">
-        <v>39.99</v>
+        <v>17.99</v>
       </c>
       <c r="H38" t="n">
-        <v>39.99</v>
+        <v>35.98</v>
       </c>
       <c r="I38" t="n">
-        <v>0.99975</v>
+        <v>0.8995</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/whey-protein-coffee/bpb-pico</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Whey Protein Coffee - Iced Caramel Latte 500g</t>
+          <t>Whey Protein Coffee - Iced Latte 1kg</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3506,16 +3506,16 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G39" t="n">
-        <v>17.99</v>
+        <v>33.99</v>
       </c>
       <c r="H39" t="n">
-        <v>35.98</v>
+        <v>33.99</v>
       </c>
       <c r="I39" t="n">
-        <v>0.8995</v>
+        <v>0.84975</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Whey Protein Coffee - Iced Latte 1kg</t>
+          <t>Clear Whey All In One - Apple &amp; Blackcurrant 500g</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3555,16 +3555,16 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G40" t="n">
-        <v>33.99</v>
+        <v>22.49</v>
       </c>
       <c r="H40" t="n">
-        <v>33.99</v>
+        <v>44.98</v>
       </c>
       <c r="I40" t="n">
-        <v>0.84975</v>
+        <v>1.1245</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/whey-protein-coffee/bpb-pico</t>
+          <t>https://www.bulk.com/uk/products/clear-all-in-one/bble-cwa1</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Clear Whey All In One - Apple &amp; Blackcurrant 500g</t>
+          <t>Clear Whey All In One - Apple &amp; Blackcurrant 1kg</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3604,16 +3604,16 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G41" t="n">
-        <v>22.49</v>
+        <v>38.99</v>
       </c>
       <c r="H41" t="n">
-        <v>44.98</v>
+        <v>38.99</v>
       </c>
       <c r="I41" t="n">
-        <v>1.1245</v>
+        <v>0.97475</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -3634,12 +3634,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Clear Whey All In One - Apple &amp; Blackcurrant 1kg</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3653,16 +3653,16 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>38.99</v>
+        <v>4.99</v>
       </c>
       <c r="H42" t="n">
-        <v>38.99</v>
+        <v>49.9</v>
       </c>
       <c r="I42" t="n">
-        <v>0.97475</v>
+        <v>1.2475</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/clear-all-in-one/bble-cwa1</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 100g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3702,16 +3702,16 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="G43" t="n">
-        <v>4.99</v>
+        <v>12.99</v>
       </c>
       <c r="H43" t="n">
-        <v>49.9</v>
+        <v>25.98</v>
       </c>
       <c r="I43" t="n">
-        <v>1.2475</v>
+        <v>0.6495</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -3737,7 +3737,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3751,16 +3751,16 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G44" t="n">
-        <v>12.99</v>
+        <v>24.99</v>
       </c>
       <c r="H44" t="n">
-        <v>25.98</v>
+        <v>24.99</v>
       </c>
       <c r="I44" t="n">
-        <v>0.6495</v>
+        <v>0.62475</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -3786,7 +3786,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3800,16 +3800,16 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="G45" t="n">
-        <v>24.99</v>
+        <v>7.49</v>
       </c>
       <c r="H45" t="n">
-        <v>24.99</v>
+        <v>29.96</v>
       </c>
       <c r="I45" t="n">
-        <v>0.62475</v>
+        <v>0.749</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 100g</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3849,16 +3849,16 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="G46" t="n">
-        <v>7.49</v>
+        <v>9.99</v>
       </c>
       <c r="H46" t="n">
-        <v>29.96</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="I46" t="n">
-        <v>0.749</v>
+        <v>2.4975</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://www.bulk.com/uk/products/creapure-creatine-monohydrate/bpb-crea-0000</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 100g</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3898,16 +3898,16 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="G47" t="n">
-        <v>9.99</v>
+        <v>39.99</v>
       </c>
       <c r="H47" t="n">
-        <v>99.90000000000001</v>
+        <v>79.98</v>
       </c>
       <c r="I47" t="n">
-        <v>2.4975</v>
+        <v>1.9995</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 500g</t>
+          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3947,16 +3947,16 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G48" t="n">
-        <v>39.99</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="H48" t="n">
-        <v>79.98</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="I48" t="n">
-        <v>1.9995</v>
+        <v>1.87475</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -3972,40 +3972,40 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate (Creapure®️) - Unflavoured 1kg</t>
+          <t>Proteín True Whey - GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>1000</v>
       </c>
       <c r="G49" t="n">
-        <v>74.98999999999999</v>
+        <v>33.95</v>
       </c>
       <c r="H49" t="n">
-        <v>74.98999999999999</v>
+        <v>33.95</v>
       </c>
       <c r="I49" t="n">
-        <v>1.87475</v>
+        <v>0.84875</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creapure-creatine-monohydrate/bpb-crea-0000</t>
+          <t>https://gymbeam.sk/true-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Proteín True Whey - GymBeam 1000 g - bez príchute - 01</t>
+          <t>Proteín True Whey - GymBeam 2500 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4045,16 +4045,16 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G50" t="n">
-        <v>33.95</v>
+        <v>79.95</v>
       </c>
       <c r="H50" t="n">
-        <v>33.95</v>
+        <v>31.98</v>
       </c>
       <c r="I50" t="n">
-        <v>0.84875</v>
+        <v>0.7995</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -4080,7 +4080,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Proteín True Whey - GymBeam 2500 g - bez príchute - 01</t>
+          <t>Proteín ASAP True Whey - GymBeam 2000 g - banán</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4094,16 +4094,16 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="G51" t="n">
-        <v>79.95</v>
+        <v>73.95</v>
       </c>
       <c r="H51" t="n">
-        <v>31.98</v>
+        <v>36.975</v>
       </c>
       <c r="I51" t="n">
-        <v>0.7995</v>
+        <v>0.9243749999999999</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/true-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/asap-true-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Proteín ASAP True Whey - GymBeam 2000 g - banán</t>
+          <t>Proteín ASAP True Whey - GymBeam 900 g - banán</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4143,16 +4143,16 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>2000</v>
+        <v>900</v>
       </c>
       <c r="G52" t="n">
-        <v>73.95</v>
+        <v>37.95</v>
       </c>
       <c r="H52" t="n">
-        <v>36.975</v>
+        <v>42.16666666666666</v>
       </c>
       <c r="I52" t="n">
-        <v>0.9243749999999999</v>
+        <v>1.054166666666667</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Proteín ASAP True Whey - GymBeam 900 g - banán</t>
+          <t>Clear Whey Protein - BeastPink 500 g - citrón-limetka</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4192,16 +4192,16 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="G53" t="n">
-        <v>37.95</v>
+        <v>20.95</v>
       </c>
       <c r="H53" t="n">
-        <v>42.16666666666666</v>
+        <v>41.9</v>
       </c>
       <c r="I53" t="n">
-        <v>1.054166666666667</v>
+        <v>1.0475</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/asap-true-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/cisty-srvatkovy-protein-beastpink-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Clear Whey Protein - BeastPink 500 g - citrón-limetka</t>
+          <t>Proteín Pure IsoWhey - GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4241,16 +4241,16 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G54" t="n">
-        <v>20.95</v>
+        <v>39.95</v>
       </c>
       <c r="H54" t="n">
-        <v>41.9</v>
+        <v>39.95</v>
       </c>
       <c r="I54" t="n">
-        <v>1.0475</v>
+        <v>0.99875</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -4259,7 +4259,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/cisty-srvatkovy-protein-beastpink-gymbeam.html</t>
+          <t>https://gymbeam.sk/pure-isowhey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Proteín Pure IsoWhey - GymBeam 1000 g - bez príchute - 01</t>
+          <t>Proteín Pure IsoWhey - GymBeam 2500 g - čokoláda - 00</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4290,16 +4290,16 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G55" t="n">
-        <v>39.95</v>
+        <v>87.95</v>
       </c>
       <c r="H55" t="n">
-        <v>39.95</v>
+        <v>35.18</v>
       </c>
       <c r="I55" t="n">
-        <v>0.99875</v>
+        <v>0.8794999999999999</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Proteín Pure IsoWhey - GymBeam 2500 g - čokoláda - 00</t>
+          <t>100% Whey - Nutrend 2250 g - banán</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4339,25 +4339,25 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>2500</v>
+        <v>2250</v>
       </c>
       <c r="G56" t="n">
-        <v>87.95</v>
+        <v>67.95</v>
       </c>
       <c r="H56" t="n">
-        <v>35.18</v>
+        <v>30.2</v>
       </c>
       <c r="I56" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.755</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/pure-isowhey-gymbeam.html</t>
+          <t>https://gymbeam.sk/614-protein-whey-core-100-nutrend.html</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>100% Whey - Nutrend 2250 g - banán</t>
+          <t>Whey Protein 100 - Bodylab 1000 g - banán</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4388,16 +4388,16 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>2250</v>
+        <v>1000</v>
       </c>
       <c r="G57" t="n">
-        <v>67.95</v>
+        <v>19.5</v>
       </c>
       <c r="H57" t="n">
-        <v>30.2</v>
+        <v>19.5</v>
       </c>
       <c r="I57" t="n">
-        <v>0.755</v>
+        <v>0.4875</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/614-protein-whey-core-100-nutrend.html</t>
+          <t>https://gymbeam.sk/protein-whey100-bodylab.html</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Whey Protein 100 - Bodylab 1000 g - banán</t>
+          <t>100% Whey - Stacker2 2000 g - čokoláda</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4437,16 +4437,16 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G58" t="n">
-        <v>19.5</v>
+        <v>61.95</v>
       </c>
       <c r="H58" t="n">
-        <v>19.5</v>
+        <v>30.975</v>
       </c>
       <c r="I58" t="n">
-        <v>0.4875</v>
+        <v>0.774375</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-whey100-bodylab.html</t>
+          <t>https://gymbeam.sk/protein-100-whey-stacker2.html</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>100% Whey - Stacker2 2000 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 1850 g - čokoláda</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4486,16 +4486,16 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>2000</v>
+        <v>1850</v>
       </c>
       <c r="G59" t="n">
-        <v>61.95</v>
+        <v>34.95</v>
       </c>
       <c r="H59" t="n">
-        <v>30.975</v>
+        <v>18.89189189189189</v>
       </c>
       <c r="I59" t="n">
-        <v>0.774375</v>
+        <v>0.4722972972972973</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-100-whey-stacker2.html</t>
+          <t>https://gymbeam.sk/510-protein-100-whey-2350-g-scitec-nutrition-3.html</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 1850 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 920 g - čokoláda</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4535,16 +4535,16 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>1850</v>
+        <v>920</v>
       </c>
       <c r="G60" t="n">
-        <v>34.95</v>
+        <v>23.95</v>
       </c>
       <c r="H60" t="n">
-        <v>18.89189189189189</v>
+        <v>26.03260869565218</v>
       </c>
       <c r="I60" t="n">
-        <v>0.4722972972972973</v>
+        <v>0.6508152173913043</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 920 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 2350 g - čokoláda</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4584,16 +4584,16 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>920</v>
+        <v>2350</v>
       </c>
       <c r="G61" t="n">
-        <v>23.95</v>
+        <v>45.95</v>
       </c>
       <c r="H61" t="n">
-        <v>26.03260869565218</v>
+        <v>19.5531914893617</v>
       </c>
       <c r="I61" t="n">
-        <v>0.6508152173913043</v>
+        <v>0.4888297872340426</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 2350 g - čokoláda</t>
+          <t>Proteín 100% Whey - Scitec Nutrition 5000 g - čokoláda</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4633,16 +4633,16 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>2350</v>
+        <v>5000</v>
       </c>
       <c r="G62" t="n">
-        <v>45.95</v>
+        <v>95.95</v>
       </c>
       <c r="H62" t="n">
-        <v>19.5531914893617</v>
+        <v>19.19</v>
       </c>
       <c r="I62" t="n">
-        <v>0.4888297872340426</v>
+        <v>0.47975</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey - Scitec Nutrition 5000 g - čokoláda</t>
+          <t>100% Whey Premium - ActivLab 2000 g - čokoláda</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4682,25 +4682,25 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="G63" t="n">
-        <v>95.95</v>
+        <v>50.95</v>
       </c>
       <c r="H63" t="n">
-        <v>19.19</v>
+        <v>25.475</v>
       </c>
       <c r="I63" t="n">
-        <v>0.47975</v>
+        <v>0.636875</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/510-protein-100-whey-2350-g-scitec-nutrition-3.html</t>
+          <t>https://gymbeam.sk/100-whey-premium-activlab.html</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>100% Whey Premium - ActivLab 2000 g - čokoláda</t>
+          <t>Proteín Combat 100% Whey - MusclePharm 2270 g - čokoláda</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4731,25 +4731,25 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>2000</v>
+        <v>2270</v>
       </c>
       <c r="G64" t="n">
-        <v>50.95</v>
+        <v>43.95</v>
       </c>
       <c r="H64" t="n">
-        <v>25.475</v>
+        <v>19.36123348017621</v>
       </c>
       <c r="I64" t="n">
-        <v>0.636875</v>
+        <v>0.4840308370044053</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-whey-premium-activlab.html</t>
+          <t>https://gymbeam.sk/protein-combat-100-whey-musclepharm.html</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Proteín Combat 100% Whey - MusclePharm 2270 g - čokoláda</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 1110 g - chocolate</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4780,16 +4780,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>2270</v>
+        <v>1110</v>
       </c>
       <c r="G65" t="n">
-        <v>43.95</v>
+        <v>23.95</v>
       </c>
       <c r="H65" t="n">
-        <v>19.36123348017621</v>
+        <v>21.57657657657658</v>
       </c>
       <c r="I65" t="n">
-        <v>0.4840308370044053</v>
+        <v>0.5394144144144144</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-combat-100-whey-musclepharm.html</t>
+          <t>https://gymbeam.sk/10-protein-100-whey-professional-2350-g-scitec-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 1110 g - chocolate</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 2820 g - čokoláda</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4829,16 +4829,16 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>1110</v>
+        <v>2820</v>
       </c>
       <c r="G66" t="n">
-        <v>23.95</v>
+        <v>45.95</v>
       </c>
       <c r="H66" t="n">
-        <v>21.57657657657658</v>
+        <v>16.29432624113475</v>
       </c>
       <c r="I66" t="n">
-        <v>0.5394144144144144</v>
+        <v>0.4073581560283688</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 2820 g - čokoláda</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition - 500 g - chocolate</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4878,16 +4878,16 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>2820</v>
+        <v>500</v>
       </c>
       <c r="G67" t="n">
-        <v>45.95</v>
+        <v>21.95</v>
       </c>
       <c r="H67" t="n">
-        <v>16.29432624113475</v>
+        <v>43.9</v>
       </c>
       <c r="I67" t="n">
-        <v>0.4073581560283688</v>
+        <v>1.0975</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition - 500 g - chocolate</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 750 g - banán</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4927,16 +4927,16 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="G68" t="n">
-        <v>21.95</v>
+        <v>20.95</v>
       </c>
       <c r="H68" t="n">
-        <v>43.9</v>
+        <v>27.93333333333333</v>
       </c>
       <c r="I68" t="n">
-        <v>1.0975</v>
+        <v>0.6983333333333334</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -4962,7 +4962,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 750 g - banán</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 920 g - čokoláda</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4976,16 +4976,16 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>750</v>
+        <v>920</v>
       </c>
       <c r="G69" t="n">
-        <v>20.95</v>
+        <v>21.95</v>
       </c>
       <c r="H69" t="n">
-        <v>27.93333333333333</v>
+        <v>23.85869565217391</v>
       </c>
       <c r="I69" t="n">
-        <v>0.6983333333333334</v>
+        <v>0.5964673913043478</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 920 g - čokoláda</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 2350 g - banán</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -5025,16 +5025,16 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>920</v>
+        <v>2350</v>
       </c>
       <c r="G70" t="n">
-        <v>21.95</v>
+        <v>45.95</v>
       </c>
       <c r="H70" t="n">
-        <v>23.85869565217391</v>
+        <v>19.5531914893617</v>
       </c>
       <c r="I70" t="n">
-        <v>0.5964673913043478</v>
+        <v>0.4888297872340426</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 2350 g - banán</t>
+          <t>Protein 100% Whey Professional - Scitec Nutrition 5000 g - banán</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -5074,16 +5074,16 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>2350</v>
+        <v>5000</v>
       </c>
       <c r="G71" t="n">
-        <v>45.95</v>
+        <v>99.95</v>
       </c>
       <c r="H71" t="n">
-        <v>19.5531914893617</v>
+        <v>19.99</v>
       </c>
       <c r="I71" t="n">
-        <v>0.4888297872340426</v>
+        <v>0.49975</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Professional - Scitec Nutrition 5000 g - banán</t>
+          <t>Protein 100% Whey Isolate - Scitec Nutrition 2000 g - banán</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -5123,16 +5123,16 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="G72" t="n">
-        <v>99.95</v>
+        <v>59.95</v>
       </c>
       <c r="H72" t="n">
-        <v>19.99</v>
+        <v>29.975</v>
       </c>
       <c r="I72" t="n">
-        <v>0.49975</v>
+        <v>0.749375</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/10-protein-100-whey-professional-2350-g-scitec-nutrition.html</t>
+          <t>https://gymbeam.sk/12-protein-100-whey-isolate-20-kg.html</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Isolate - Scitec Nutrition 2000 g - banán</t>
+          <t>Protein 100% Whey Isolate - Scitec Nutrition 4000 g - čokoláda</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -5172,16 +5172,16 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="G73" t="n">
-        <v>59.95</v>
+        <v>87.95</v>
       </c>
       <c r="H73" t="n">
-        <v>29.975</v>
+        <v>21.9875</v>
       </c>
       <c r="I73" t="n">
-        <v>0.749375</v>
+        <v>0.5496875</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Isolate - Scitec Nutrition 4000 g - čokoláda</t>
+          <t>Protein 100% Whey Isolate - Scitec Nutrition 700 g - banán</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -5221,16 +5221,16 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>4000</v>
+        <v>700</v>
       </c>
       <c r="G74" t="n">
-        <v>87.95</v>
+        <v>25.95</v>
       </c>
       <c r="H74" t="n">
-        <v>21.9875</v>
+        <v>37.07142857142857</v>
       </c>
       <c r="I74" t="n">
-        <v>0.5496875</v>
+        <v>0.9267857142857143</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Protein 100% Whey Isolate - Scitec Nutrition 700 g - banán</t>
+          <t>Proteín 100% Whey Protein - MuscleTech  2270 g - trojitá čokoláda</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5270,16 +5270,16 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>700</v>
+        <v>2270</v>
       </c>
       <c r="G75" t="n">
-        <v>25.95</v>
+        <v>33.95</v>
       </c>
       <c r="H75" t="n">
-        <v>37.07142857142857</v>
+        <v>14.95594713656388</v>
       </c>
       <c r="I75" t="n">
-        <v>0.9267857142857143</v>
+        <v>0.3738986784140969</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/12-protein-100-whey-isolate-20-kg.html</t>
+          <t>https://gymbeam.sk/100-premium-whey-protein-plus-muscletech.html</t>
         </is>
       </c>
     </row>
@@ -5305,7 +5305,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Proteín 100% Whey Protein - MuscleTech  2270 g - trojitá čokoláda</t>
+          <t>Animal 100 % Whey Proteín - Universal Nutrition 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -5319,16 +5319,16 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>2270</v>
+        <v>1000</v>
       </c>
       <c r="G76" t="n">
-        <v>33.95</v>
+        <v>31.95</v>
       </c>
       <c r="H76" t="n">
-        <v>14.95594713656388</v>
+        <v>31.95</v>
       </c>
       <c r="I76" t="n">
-        <v>0.3738986784140969</v>
+        <v>0.79875</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -5337,7 +5337,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-premium-whey-protein-plus-muscletech.html</t>
+          <t>https://gymbeam.sk/animal-100-whey-protein-universal-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Animal 100 % Whey Proteín - Universal Nutrition 1000 g - čokoláda</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 2250 g - vanilková zmrzlina</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5368,16 +5368,16 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>1000</v>
+        <v>2250</v>
       </c>
       <c r="G77" t="n">
-        <v>31.95</v>
+        <v>70.95</v>
       </c>
       <c r="H77" t="n">
-        <v>31.95</v>
+        <v>31.53333333333333</v>
       </c>
       <c r="I77" t="n">
-        <v>0.79875</v>
+        <v>0.7883333333333333</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/animal-100-whey-protein-universal-nutrition.html</t>
+          <t>https://gymbeam.sk/100-whey-gold-standard-optimum-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -5403,7 +5403,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 2250 g - vanilková zmrzlina</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 450 g - dvojitá bohatá čokoláda</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5417,20 +5417,20 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>2250</v>
+        <v>450</v>
       </c>
       <c r="G78" t="n">
-        <v>70.95</v>
+        <v>22.95</v>
       </c>
       <c r="H78" t="n">
-        <v>31.53333333333333</v>
+        <v>51</v>
       </c>
       <c r="I78" t="n">
-        <v>0.7883333333333333</v>
+        <v>1.275</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 450 g - dvojitá bohatá čokoláda</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 4540 g - dvojitá bohatá čokoláda</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5466,16 +5466,16 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>450</v>
+        <v>4540</v>
       </c>
       <c r="G79" t="n">
-        <v>22.95</v>
+        <v>169.95</v>
       </c>
       <c r="H79" t="n">
-        <v>51</v>
+        <v>37.43392070484582</v>
       </c>
       <c r="I79" t="n">
-        <v>1.275</v>
+        <v>0.9358480176211453</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 4540 g - dvojitá bohatá čokoláda</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 768 g - banánový krém</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5515,16 +5515,16 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>4540</v>
+        <v>768</v>
       </c>
       <c r="G80" t="n">
-        <v>169.95</v>
+        <v>39.95</v>
       </c>
       <c r="H80" t="n">
-        <v>37.43392070484582</v>
+        <v>52.01822916666666</v>
       </c>
       <c r="I80" t="n">
-        <v>0.9358480176211453</v>
+        <v>1.300455729166667</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 768 g - banánový krém</t>
+          <t>100% Whey Gold Standard - Optimum Nutrition 2010 g - banánový krém</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5564,16 +5564,16 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>768</v>
+        <v>2010</v>
       </c>
       <c r="G81" t="n">
-        <v>39.95</v>
+        <v>79.95</v>
       </c>
       <c r="H81" t="n">
-        <v>52.01822916666666</v>
+        <v>39.77611940298507</v>
       </c>
       <c r="I81" t="n">
-        <v>1.300455729166667</v>
+        <v>0.9944029850746269</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>100% Whey Gold Standard - Optimum Nutrition 2010 g - banánový krém</t>
+          <t>Proteín 100% Premium Whey Protein Plus - MuscleTech 2720 g - deluxe čokoláda</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5613,25 +5613,25 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>2010</v>
+        <v>2720</v>
       </c>
       <c r="G82" t="n">
-        <v>79.95</v>
+        <v>39.95</v>
       </c>
       <c r="H82" t="n">
-        <v>39.77611940298507</v>
+        <v>14.6875</v>
       </c>
       <c r="I82" t="n">
-        <v>0.9944029850746269</v>
+        <v>0.3671875</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-whey-gold-standard-optimum-nutrition.html</t>
+          <t>https://gymbeam.sk/100-premium-whey-protein-plus-muscletech-2.html</t>
         </is>
       </c>
     </row>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Proteín 100% Premium Whey Protein Plus - MuscleTech 2720 g - deluxe čokoláda</t>
+          <t>Proteín 100% Premium Whey Isolate Plus 1360 g - MuscleTech deluxe čokoláda</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5662,16 +5662,16 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>2720</v>
+        <v>1360</v>
       </c>
       <c r="G83" t="n">
-        <v>39.95</v>
+        <v>29.95</v>
       </c>
       <c r="H83" t="n">
-        <v>14.6875</v>
+        <v>22.02205882352941</v>
       </c>
       <c r="I83" t="n">
-        <v>0.3671875</v>
+        <v>0.5505514705882353</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -5680,7 +5680,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/100-premium-whey-protein-plus-muscletech-2.html</t>
+          <t>https://gymbeam.sk/protein-100-premium-whey-isolate-plus-1380-g-muscletech.html</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Proteín 100% Premium Whey Isolate Plus 1360 g - MuscleTech deluxe čokoláda</t>
+          <t>Clear Whey - Ghost 640 g - modrá malina</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5711,25 +5711,25 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>1360</v>
+        <v>640</v>
       </c>
       <c r="G84" t="n">
-        <v>29.95</v>
+        <v>46.95</v>
       </c>
       <c r="H84" t="n">
-        <v>22.02205882352941</v>
+        <v>73.359375</v>
       </c>
       <c r="I84" t="n">
-        <v>0.5505514705882353</v>
+        <v>1.833984375</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-100-premium-whey-isolate-plus-1380-g-muscletech.html</t>
+          <t>https://gymbeam.sk/clear-whey-ghost.html</t>
         </is>
       </c>
     </row>
@@ -5746,7 +5746,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Clear Whey - Ghost 640 g - modrá malina</t>
+          <t>Protein Gold Whey - Weider 500 g - jahoda</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5760,25 +5760,25 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>640</v>
+        <v>500</v>
       </c>
       <c r="G85" t="n">
-        <v>46.95</v>
+        <v>19.95</v>
       </c>
       <c r="H85" t="n">
-        <v>73.359375</v>
+        <v>39.9</v>
       </c>
       <c r="I85" t="n">
-        <v>1.833984375</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-ghost.html</t>
+          <t>https://gymbeam.sk/protein-gold-whey-weider.html</t>
         </is>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Protein Gold Whey - Weider 500 g - jahoda</t>
+          <t>BIO Whey Protein - GymBeam 900 g - kakao</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5809,25 +5809,25 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="G86" t="n">
-        <v>19.95</v>
+        <v>45.95</v>
       </c>
       <c r="H86" t="n">
-        <v>39.9</v>
+        <v>51.05555555555556</v>
       </c>
       <c r="I86" t="n">
-        <v>0.9975000000000001</v>
+        <v>1.276388888888889</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-gold-whey-weider.html</t>
+          <t>https://gymbeam.sk/bio-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>BIO Whey Protein - GymBeam 900 g - kakao</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5858,16 +5858,16 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="G87" t="n">
-        <v>45.95</v>
+        <v>37.95</v>
       </c>
       <c r="H87" t="n">
-        <v>51.05555555555556</v>
+        <v>37.95</v>
       </c>
       <c r="I87" t="n">
-        <v>1.276388888888889</v>
+        <v>0.94875</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/bio-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5907,16 +5907,16 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G88" t="n">
-        <v>37.95</v>
+        <v>67.95</v>
       </c>
       <c r="H88" t="n">
-        <v>37.95</v>
+        <v>33.975</v>
       </c>
       <c r="I88" t="n">
-        <v>0.94875</v>
+        <v>0.849375</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5956,16 +5956,16 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G89" t="n">
-        <v>67.95</v>
+        <v>24.95</v>
       </c>
       <c r="H89" t="n">
-        <v>33.975</v>
+        <v>49.9</v>
       </c>
       <c r="I89" t="n">
-        <v>0.849375</v>
+        <v>1.2475</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
+          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6005,16 +6005,16 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G90" t="n">
-        <v>24.95</v>
+        <v>37.95</v>
       </c>
       <c r="H90" t="n">
-        <v>49.9</v>
+        <v>37.95</v>
       </c>
       <c r="I90" t="n">
-        <v>1.2475</v>
+        <v>0.94875</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6054,16 +6054,16 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G91" t="n">
-        <v>37.95</v>
+        <v>24.95</v>
       </c>
       <c r="H91" t="n">
-        <v>37.95</v>
+        <v>49.9</v>
       </c>
       <c r="I91" t="n">
-        <v>0.94875</v>
+        <v>1.2475</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Anabolic Whey - GymBeam 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6103,16 +6103,16 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G92" t="n">
-        <v>24.95</v>
+        <v>21.95</v>
       </c>
       <c r="H92" t="n">
-        <v>49.9</v>
+        <v>21.95</v>
       </c>
       <c r="I92" t="n">
-        <v>1.2475</v>
+        <v>0.54875</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -6121,7 +6121,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
+          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Proteín Anabolic Whey - GymBeam 1000 g - čokoláda</t>
+          <t>Proteín Anabolic Whey - GymBeam 2500 g - čokoláda</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6152,16 +6152,16 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G93" t="n">
-        <v>21.95</v>
+        <v>52.95</v>
       </c>
       <c r="H93" t="n">
-        <v>21.95</v>
+        <v>21.18</v>
       </c>
       <c r="I93" t="n">
-        <v>0.54875</v>
+        <v>0.5295</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Proteín Anabolic Whey - GymBeam 2500 g - čokoláda</t>
+          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6201,16 +6201,16 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G94" t="n">
-        <v>52.95</v>
+        <v>31.95</v>
       </c>
       <c r="H94" t="n">
-        <v>21.18</v>
+        <v>31.95</v>
       </c>
       <c r="I94" t="n">
-        <v>0.5295</v>
+        <v>0.79875</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
+          <t>Whey Proteín - Mammut Nutrition 3000 g - vanilka</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6250,16 +6250,16 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="G95" t="n">
-        <v>31.95</v>
+        <v>93.95</v>
       </c>
       <c r="H95" t="n">
-        <v>31.95</v>
+        <v>31.31666666666667</v>
       </c>
       <c r="I95" t="n">
-        <v>0.79875</v>
+        <v>0.7829166666666667</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 3000 g - vanilka</t>
+          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6299,25 +6299,25 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G96" t="n">
-        <v>93.95</v>
+        <v>21.95</v>
       </c>
       <c r="H96" t="n">
-        <v>31.31666666666667</v>
+        <v>43.9</v>
       </c>
       <c r="I96" t="n">
-        <v>0.7829166666666667</v>
+        <v>1.0975</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
+          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
+          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6348,16 +6348,16 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G97" t="n">
-        <v>21.95</v>
+        <v>34.95</v>
       </c>
       <c r="H97" t="n">
-        <v>43.9</v>
+        <v>34.95</v>
       </c>
       <c r="I97" t="n">
-        <v>1.0975</v>
+        <v>0.87375</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
+          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6397,16 +6397,16 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G98" t="n">
-        <v>34.95</v>
+        <v>62.95</v>
       </c>
       <c r="H98" t="n">
-        <v>34.95</v>
+        <v>31.475</v>
       </c>
       <c r="I98" t="n">
-        <v>0.87375</v>
+        <v>0.786875</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
+          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6446,16 +6446,16 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G99" t="n">
-        <v>62.95</v>
+        <v>19.5</v>
       </c>
       <c r="H99" t="n">
-        <v>31.475</v>
+        <v>39</v>
       </c>
       <c r="I99" t="n">
-        <v>0.786875</v>
+        <v>0.975</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
+          <t>Whey Protein - Bodylab24 1000 g - banán</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6495,16 +6495,16 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G100" t="n">
-        <v>19.5</v>
+        <v>39.95</v>
       </c>
       <c r="H100" t="n">
-        <v>39</v>
+        <v>39.95</v>
       </c>
       <c r="I100" t="n">
-        <v>0.975</v>
+        <v>0.99875</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6513,7 +6513,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
         </is>
       </c>
     </row>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 1000 g - banán</t>
+          <t>Whey Protein - Bodylab24 2000 g - banán</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6544,16 +6544,16 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G101" t="n">
-        <v>39.95</v>
+        <v>64.95</v>
       </c>
       <c r="H101" t="n">
-        <v>39.95</v>
+        <v>32.475</v>
       </c>
       <c r="I101" t="n">
-        <v>0.99875</v>
+        <v>0.811875</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 2000 g - banán</t>
+          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6593,16 +6593,16 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>2000</v>
+        <v>400</v>
       </c>
       <c r="G102" t="n">
-        <v>64.95</v>
+        <v>42.95</v>
       </c>
       <c r="H102" t="n">
-        <v>32.475</v>
+        <v>107.375</v>
       </c>
       <c r="I102" t="n">
-        <v>0.811875</v>
+        <v>2.684375</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -6611,7 +6611,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
+          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6642,16 +6642,16 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>400</v>
+        <v>1200</v>
       </c>
       <c r="G103" t="n">
-        <v>42.95</v>
+        <v>34.95</v>
       </c>
       <c r="H103" t="n">
-        <v>107.375</v>
+        <v>29.125</v>
       </c>
       <c r="I103" t="n">
-        <v>2.684375</v>
+        <v>0.728125</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
+          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6677,7 +6677,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6691,16 +6691,16 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G104" t="n">
-        <v>34.95</v>
+        <v>62.95</v>
       </c>
       <c r="H104" t="n">
-        <v>29.125</v>
+        <v>26.22916666666667</v>
       </c>
       <c r="I104" t="n">
-        <v>0.728125</v>
+        <v>0.6557291666666667</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
+          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,20 +6740,20 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>2400</v>
+        <v>600</v>
       </c>
       <c r="G105" t="n">
-        <v>62.95</v>
+        <v>19.5</v>
       </c>
       <c r="H105" t="n">
-        <v>26.22916666666667</v>
+        <v>32.5</v>
       </c>
       <c r="I105" t="n">
-        <v>0.6557291666666667</v>
+        <v>0.8125</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,25 +6789,25 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="G106" t="n">
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
       <c r="H106" t="n">
-        <v>32.5</v>
+        <v>16.5</v>
       </c>
       <c r="I106" t="n">
-        <v>0.8125</v>
+        <v>0.4125</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G107" t="n">
-        <v>16.5</v>
+        <v>31.95</v>
       </c>
       <c r="H107" t="n">
-        <v>16.5</v>
+        <v>12.78</v>
       </c>
       <c r="I107" t="n">
-        <v>0.4125</v>
+        <v>0.3195</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="G108" t="n">
-        <v>31.95</v>
+        <v>11.95</v>
       </c>
       <c r="H108" t="n">
-        <v>12.78</v>
+        <v>23.9</v>
       </c>
       <c r="I108" t="n">
-        <v>0.3195</v>
+        <v>0.5975</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6936,16 +6936,16 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>500</v>
+        <v>1450</v>
       </c>
       <c r="G109" t="n">
-        <v>11.95</v>
+        <v>29.95</v>
       </c>
       <c r="H109" t="n">
-        <v>23.9</v>
+        <v>20.6551724137931</v>
       </c>
       <c r="I109" t="n">
-        <v>0.5975</v>
+        <v>0.5163793103448275</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6966,12 +6966,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6985,25 +6985,25 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1450</v>
+        <v>400</v>
       </c>
       <c r="G110" t="n">
-        <v>29.95</v>
+        <v>10.95</v>
       </c>
       <c r="H110" t="n">
-        <v>20.6551724137931</v>
+        <v>27.375</v>
       </c>
       <c r="I110" t="n">
-        <v>0.5163793103448275</v>
+        <v>0.684375</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7034,16 +7034,16 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="G111" t="n">
-        <v>10.95</v>
+        <v>33.95</v>
       </c>
       <c r="H111" t="n">
-        <v>27.375</v>
+        <v>33.95</v>
       </c>
       <c r="I111" t="n">
-        <v>0.684375</v>
+        <v>0.84875</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7083,16 +7083,16 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="G112" t="n">
-        <v>33.95</v>
+        <v>14.95</v>
       </c>
       <c r="H112" t="n">
-        <v>33.95</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I112" t="n">
-        <v>0.84875</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7132,16 +7132,16 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G113" t="n">
-        <v>14.95</v>
+        <v>18.5</v>
       </c>
       <c r="H113" t="n">
-        <v>49.83333333333334</v>
+        <v>37</v>
       </c>
       <c r="I113" t="n">
-        <v>1.245833333333333</v>
+        <v>0.925</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7184,22 +7184,22 @@
         <v>500</v>
       </c>
       <c r="G114" t="n">
-        <v>18.5</v>
+        <v>12.95</v>
       </c>
       <c r="H114" t="n">
-        <v>37</v>
+        <v>25.9</v>
       </c>
       <c r="I114" t="n">
-        <v>0.925</v>
+        <v>0.6475</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7230,25 +7230,25 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G115" t="n">
-        <v>12.95</v>
+        <v>23.95</v>
       </c>
       <c r="H115" t="n">
-        <v>25.9</v>
+        <v>23.95</v>
       </c>
       <c r="I115" t="n">
-        <v>0.6475</v>
+        <v>0.59875</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7279,16 +7279,16 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G116" t="n">
-        <v>23.95</v>
+        <v>33.95</v>
       </c>
       <c r="H116" t="n">
-        <v>23.95</v>
+        <v>22.63333333333333</v>
       </c>
       <c r="I116" t="n">
-        <v>0.59875</v>
+        <v>0.5658333333333333</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7328,16 +7328,16 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>1500</v>
+        <v>250</v>
       </c>
       <c r="G117" t="n">
-        <v>33.95</v>
+        <v>7.5</v>
       </c>
       <c r="H117" t="n">
-        <v>22.63333333333333</v>
+        <v>30</v>
       </c>
       <c r="I117" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.75</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7377,16 +7377,16 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="G118" t="n">
-        <v>7.5</v>
+        <v>12.95</v>
       </c>
       <c r="H118" t="n">
-        <v>30</v>
+        <v>25.9</v>
       </c>
       <c r="I118" t="n">
-        <v>0.75</v>
+        <v>0.6475</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="G119" t="n">
-        <v>12.95</v>
+        <v>18.5</v>
       </c>
       <c r="H119" t="n">
-        <v>25.9</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="I119" t="n">
-        <v>0.6475</v>
+        <v>0.6166666666666667</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7475,25 +7475,25 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>750</v>
+        <v>300</v>
       </c>
       <c r="G120" t="n">
-        <v>18.5</v>
+        <v>13.95</v>
       </c>
       <c r="H120" t="n">
-        <v>24.66666666666667</v>
+        <v>46.5</v>
       </c>
       <c r="I120" t="n">
-        <v>0.6166666666666667</v>
+        <v>1.1625</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7524,16 +7524,16 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="G121" t="n">
-        <v>13.95</v>
+        <v>12.5</v>
       </c>
       <c r="H121" t="n">
-        <v>46.5</v>
+        <v>31.25</v>
       </c>
       <c r="I121" t="n">
-        <v>1.1625</v>
+        <v>0.78125</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -7542,56 +7542,56 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>protein_works</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>The Protein Works</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="G122" t="n">
-        <v>12.5</v>
+        <v>34.99</v>
       </c>
       <c r="H122" t="n">
-        <v>31.25</v>
+        <v>69.98</v>
       </c>
       <c r="I122" t="n">
-        <v>0.78125</v>
+        <v>1.7495</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7622,16 +7622,16 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G123" t="n">
-        <v>34.99</v>
+        <v>58.99</v>
       </c>
       <c r="H123" t="n">
-        <v>69.98</v>
+        <v>58.99</v>
       </c>
       <c r="I123" t="n">
-        <v>1.7495</v>
+        <v>1.47475</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -7671,16 +7671,16 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G124" t="n">
-        <v>68.98999999999999</v>
+        <v>109.99</v>
       </c>
       <c r="H124" t="n">
-        <v>68.98999999999999</v>
+        <v>54.995</v>
       </c>
       <c r="I124" t="n">
-        <v>1.72475</v>
+        <v>1.374875</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7720,20 +7720,20 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="G125" t="n">
-        <v>129.49</v>
+        <v>208.49</v>
       </c>
       <c r="H125" t="n">
-        <v>64.745</v>
+        <v>52.1225</v>
       </c>
       <c r="I125" t="n">
-        <v>1.618625</v>
+        <v>1.3030625</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7769,25 +7769,25 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>4000</v>
+        <v>500</v>
       </c>
       <c r="G126" t="n">
-        <v>245.99</v>
+        <v>23.99</v>
       </c>
       <c r="H126" t="n">
-        <v>61.4975</v>
+        <v>47.98</v>
       </c>
       <c r="I126" t="n">
-        <v>1.5374375</v>
+        <v>1.1995</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7818,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G127" t="n">
-        <v>23.99</v>
+        <v>44.99</v>
       </c>
       <c r="H127" t="n">
-        <v>47.98</v>
+        <v>44.99</v>
       </c>
       <c r="I127" t="n">
-        <v>1.1995</v>
+        <v>1.12475</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="G128" t="n">
-        <v>44.99</v>
+        <v>16.99</v>
       </c>
       <c r="H128" t="n">
-        <v>44.99</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I128" t="n">
-        <v>1.12475</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G129" t="n">
-        <v>14.99</v>
+        <v>26.99</v>
       </c>
       <c r="H129" t="n">
-        <v>24.98333333333333</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I129" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G130" t="n">
-        <v>23.99</v>
+        <v>49.99</v>
       </c>
       <c r="H130" t="n">
-        <v>19.99166666666667</v>
+        <v>20.82916666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.4997916666666667</v>
+        <v>0.5207291666666667</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G131" t="n">
-        <v>44.49</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="H131" t="n">
-        <v>18.5375</v>
+        <v>19.99791666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.4634375</v>
+        <v>0.4999479166666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8049,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -8063,16 +8063,16 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>4800</v>
+        <v>500</v>
       </c>
       <c r="G132" t="n">
-        <v>84.48999999999999</v>
+        <v>19.99</v>
       </c>
       <c r="H132" t="n">
-        <v>17.60208333333333</v>
+        <v>39.98</v>
       </c>
       <c r="I132" t="n">
-        <v>0.4400520833333333</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8098,7 +8098,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -8112,16 +8112,16 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="G133" t="n">
-        <v>15.99</v>
+        <v>33.99</v>
       </c>
       <c r="H133" t="n">
-        <v>26.65</v>
+        <v>33.99</v>
       </c>
       <c r="I133" t="n">
-        <v>0.66625</v>
+        <v>0.84975</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8147,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -8161,16 +8161,16 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="G134" t="n">
-        <v>26.99</v>
+        <v>63.49</v>
       </c>
       <c r="H134" t="n">
-        <v>22.49166666666667</v>
+        <v>31.745</v>
       </c>
       <c r="I134" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.793625</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8196,7 +8196,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8210,16 +8210,16 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>2400</v>
+        <v>4000</v>
       </c>
       <c r="G135" t="n">
-        <v>49.49</v>
+        <v>122.99</v>
       </c>
       <c r="H135" t="n">
-        <v>20.62083333333333</v>
+        <v>30.7475</v>
       </c>
       <c r="I135" t="n">
-        <v>0.5155208333333333</v>
+        <v>0.7686875</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8259,16 +8259,16 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>4800</v>
+        <v>600</v>
       </c>
       <c r="G136" t="n">
-        <v>93.48999999999999</v>
+        <v>14.99</v>
       </c>
       <c r="H136" t="n">
-        <v>19.47708333333333</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I136" t="n">
-        <v>0.4869270833333333</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -8308,16 +8308,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="G137" t="n">
-        <v>19.99</v>
+        <v>23.99</v>
       </c>
       <c r="H137" t="n">
-        <v>39.98</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I137" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8357,16 +8357,16 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>1000</v>
+        <v>2400</v>
       </c>
       <c r="G138" t="n">
-        <v>33.99</v>
+        <v>44.49</v>
       </c>
       <c r="H138" t="n">
-        <v>33.99</v>
+        <v>18.5375</v>
       </c>
       <c r="I138" t="n">
-        <v>0.84975</v>
+        <v>0.4634375</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8406,16 +8406,16 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>2000</v>
+        <v>4800</v>
       </c>
       <c r="G139" t="n">
-        <v>63.49</v>
+        <v>85.48999999999999</v>
       </c>
       <c r="H139" t="n">
-        <v>31.745</v>
+        <v>17.81041666666667</v>
       </c>
       <c r="I139" t="n">
-        <v>0.793625</v>
+        <v>0.4452604166666667</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360 - Vanilla</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8455,16 +8455,16 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>4000</v>
+        <v>600</v>
       </c>
       <c r="G140" t="n">
-        <v>119.49</v>
+        <v>11.49</v>
       </c>
       <c r="H140" t="n">
-        <v>29.8725</v>
+        <v>19.15</v>
       </c>
       <c r="I140" t="n">
-        <v>0.7468125</v>
+        <v>0.47875</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>
       </c>
     </row>
@@ -8504,16 +8504,16 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G141" t="n">
-        <v>11.49</v>
+        <v>21.19</v>
       </c>
       <c r="H141" t="n">
-        <v>19.15</v>
+        <v>17.65833333333333</v>
       </c>
       <c r="I141" t="n">
-        <v>0.47875</v>
+        <v>0.4414583333333333</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8553,16 +8553,16 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G142" t="n">
-        <v>21.19</v>
+        <v>39.99</v>
       </c>
       <c r="H142" t="n">
-        <v>17.65833333333333</v>
+        <v>16.6625</v>
       </c>
       <c r="I142" t="n">
-        <v>0.4414583333333333</v>
+        <v>0.4165625</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8602,16 +8602,16 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G143" t="n">
-        <v>39.99</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="H143" t="n">
-        <v>16.6625</v>
+        <v>16.14375</v>
       </c>
       <c r="I143" t="n">
-        <v>0.4165625</v>
+        <v>0.40359375</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -8619,55 +8619,6 @@
         </is>
       </c>
       <c r="P143" t="inlineStr">
-        <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>protein_works</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>whey_protein</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Whey Protein 360 - Vanilla</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>The Protein Works</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="F144" t="n">
-        <v>4800</v>
-      </c>
-      <c r="G144" t="n">
-        <v>77.48999999999999</v>
-      </c>
-      <c r="H144" t="n">
-        <v>16.14375</v>
-      </c>
-      <c r="I144" t="n">
-        <v>0.40359375</v>
-      </c>
-      <c r="O144" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P144" t="inlineStr">
         <is>
           <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-09
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -449,19 +449,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>143.48</v>
+        <v>131.43</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -472,19 +472,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="C3" t="b">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>145.16</v>
+        <v>143.48</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -669,13 +669,13 @@
         <v>1500</v>
       </c>
       <c r="G2" t="n">
-        <v>33.95</v>
+        <v>23.5</v>
       </c>
       <c r="H2" t="n">
-        <v>22.63333333333333</v>
+        <v>15.66666666666667</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.3916666666666667</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -718,13 +718,13 @@
         <v>1000</v>
       </c>
       <c r="G3" t="n">
-        <v>23.95</v>
+        <v>16.5</v>
       </c>
       <c r="H3" t="n">
-        <v>23.95</v>
+        <v>16.5</v>
       </c>
       <c r="I3" t="n">
-        <v>0.59875</v>
+        <v>0.4125</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -767,13 +767,13 @@
         <v>750</v>
       </c>
       <c r="G4" t="n">
-        <v>18.5</v>
+        <v>12.95</v>
       </c>
       <c r="H4" t="n">
-        <v>24.66666666666667</v>
+        <v>17.26666666666667</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.4316666666666666</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -799,30 +799,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
+          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G5" t="n">
-        <v>24.99</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>24.99</v>
+        <v>17.9</v>
       </c>
       <c r="I5" t="n">
-        <v>0.62475</v>
+        <v>0.4475</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -862,32 +862,32 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G6" t="n">
-        <v>12.95</v>
+        <v>5.5</v>
       </c>
       <c r="H6" t="n">
-        <v>25.9</v>
+        <v>22</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6475</v>
+        <v>0.55</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -897,30 +897,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 1kg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G7" t="n">
-        <v>12.95</v>
+        <v>24.99</v>
       </c>
       <c r="H7" t="n">
-        <v>25.9</v>
+        <v>24.99</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6475</v>
+        <v>0.62475</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -929,14 +929,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -946,46 +946,46 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>500</v>
       </c>
       <c r="G8" t="n">
-        <v>12.99</v>
+        <v>12.95</v>
       </c>
       <c r="H8" t="n">
-        <v>25.98</v>
+        <v>25.9</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6495</v>
+        <v>0.6475</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -995,30 +995,30 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 500g</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="G9" t="n">
-        <v>10.95</v>
+        <v>12.99</v>
       </c>
       <c r="H9" t="n">
-        <v>27.375</v>
+        <v>25.98</v>
       </c>
       <c r="I9" t="n">
-        <v>0.684375</v>
+        <v>0.6495</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1027,14 +1027,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bulk</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1044,30 +1044,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="G10" t="n">
-        <v>7.49</v>
+        <v>10.95</v>
       </c>
       <c r="H10" t="n">
-        <v>29.96</v>
+        <v>27.375</v>
       </c>
       <c r="I10" t="n">
-        <v>0.749</v>
+        <v>0.684375</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1107,25 +1107,25 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="G11" t="n">
-        <v>7.5</v>
+        <v>12.5</v>
       </c>
       <c r="H11" t="n">
-        <v>30</v>
+        <v>31.25</v>
       </c>
       <c r="I11" t="n">
-        <v>0.75</v>
+        <v>0.78125</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1156,32 +1156,32 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="G12" t="n">
-        <v>12.5</v>
+        <v>33.95</v>
       </c>
       <c r="H12" t="n">
-        <v>31.25</v>
+        <v>33.95</v>
       </c>
       <c r="I12" t="n">
-        <v>0.78125</v>
+        <v>0.84875</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>bulk</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1191,30 +1191,30 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine Monohydrate Powder - Unflavoured 250g</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>Bulk</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="G13" t="n">
-        <v>33.95</v>
+        <v>8.99</v>
       </c>
       <c r="H13" t="n">
-        <v>33.95</v>
+        <v>35.96</v>
       </c>
       <c r="I13" t="n">
-        <v>0.84875</v>
+        <v>0.899</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://www.bulk.com/uk/products/creatine-monohydrate/bpb-cmon-0000</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P143"/>
+  <dimension ref="A1:P144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2284,13 +2284,13 @@
         <v>500</v>
       </c>
       <c r="G14" t="n">
-        <v>16.99</v>
+        <v>19.99</v>
       </c>
       <c r="H14" t="n">
-        <v>33.98</v>
+        <v>39.98</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8495</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -2333,13 +2333,13 @@
         <v>1000</v>
       </c>
       <c r="G15" t="n">
-        <v>31.99</v>
+        <v>38.99</v>
       </c>
       <c r="H15" t="n">
-        <v>31.99</v>
+        <v>38.99</v>
       </c>
       <c r="I15" t="n">
-        <v>0.79975</v>
+        <v>0.97475</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -2382,13 +2382,13 @@
         <v>2500</v>
       </c>
       <c r="G16" t="n">
-        <v>74.98999999999999</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>29.996</v>
+        <v>35.996</v>
       </c>
       <c r="I16" t="n">
-        <v>0.7499</v>
+        <v>0.8999</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -2431,13 +2431,13 @@
         <v>5000</v>
       </c>
       <c r="G17" t="n">
-        <v>139.99</v>
+        <v>174.99</v>
       </c>
       <c r="H17" t="n">
-        <v>27.998</v>
+        <v>34.998</v>
       </c>
       <c r="I17" t="n">
-        <v>0.69995</v>
+        <v>0.87495</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -3803,13 +3803,13 @@
         <v>250</v>
       </c>
       <c r="G45" t="n">
-        <v>7.49</v>
+        <v>8.99</v>
       </c>
       <c r="H45" t="n">
-        <v>29.96</v>
+        <v>35.96</v>
       </c>
       <c r="I45" t="n">
-        <v>0.749</v>
+        <v>0.899</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 3000 g - vanilka</t>
+          <t>Whey Proteín - Mammut Nutrition 3000 g - čokoláda</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,25 +6789,25 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G106" t="n">
-        <v>16.5</v>
+        <v>28.95</v>
       </c>
       <c r="H106" t="n">
-        <v>16.5</v>
+        <v>57.9</v>
       </c>
       <c r="I106" t="n">
-        <v>0.4125</v>
+        <v>1.4475</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G107" t="n">
-        <v>31.95</v>
+        <v>16.5</v>
       </c>
       <c r="H107" t="n">
-        <v>12.78</v>
+        <v>16.5</v>
       </c>
       <c r="I107" t="n">
-        <v>0.3195</v>
+        <v>0.4125</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="G108" t="n">
-        <v>11.95</v>
+        <v>31.95</v>
       </c>
       <c r="H108" t="n">
-        <v>23.9</v>
+        <v>12.78</v>
       </c>
       <c r="I108" t="n">
-        <v>0.5975</v>
+        <v>0.3195</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6936,16 +6936,16 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>1450</v>
+        <v>500</v>
       </c>
       <c r="G109" t="n">
-        <v>29.95</v>
+        <v>11.95</v>
       </c>
       <c r="H109" t="n">
-        <v>20.6551724137931</v>
+        <v>23.9</v>
       </c>
       <c r="I109" t="n">
-        <v>0.5163793103448275</v>
+        <v>0.5975</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6966,12 +6966,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6985,25 +6985,25 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>400</v>
+        <v>1450</v>
       </c>
       <c r="G110" t="n">
-        <v>10.95</v>
+        <v>39.95</v>
       </c>
       <c r="H110" t="n">
-        <v>27.375</v>
+        <v>27.55172413793104</v>
       </c>
       <c r="I110" t="n">
-        <v>0.684375</v>
+        <v>0.6887931034482758</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7034,16 +7034,16 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="G111" t="n">
-        <v>33.95</v>
+        <v>10.95</v>
       </c>
       <c r="H111" t="n">
-        <v>33.95</v>
+        <v>27.375</v>
       </c>
       <c r="I111" t="n">
-        <v>0.84875</v>
+        <v>0.684375</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7083,16 +7083,16 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="G112" t="n">
-        <v>14.95</v>
+        <v>33.95</v>
       </c>
       <c r="H112" t="n">
-        <v>49.83333333333334</v>
+        <v>33.95</v>
       </c>
       <c r="I112" t="n">
-        <v>1.245833333333333</v>
+        <v>0.84875</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7132,16 +7132,16 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G113" t="n">
-        <v>18.5</v>
+        <v>14.95</v>
       </c>
       <c r="H113" t="n">
-        <v>37</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I113" t="n">
-        <v>0.925</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7184,22 +7184,22 @@
         <v>500</v>
       </c>
       <c r="G114" t="n">
-        <v>12.95</v>
+        <v>18.5</v>
       </c>
       <c r="H114" t="n">
-        <v>25.9</v>
+        <v>37</v>
       </c>
       <c r="I114" t="n">
-        <v>0.6475</v>
+        <v>0.925</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7230,25 +7230,25 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G115" t="n">
-        <v>23.95</v>
+        <v>12.95</v>
       </c>
       <c r="H115" t="n">
-        <v>23.95</v>
+        <v>25.9</v>
       </c>
       <c r="I115" t="n">
-        <v>0.59875</v>
+        <v>0.6475</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7279,16 +7279,16 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="G116" t="n">
-        <v>33.95</v>
+        <v>16.5</v>
       </c>
       <c r="H116" t="n">
-        <v>22.63333333333333</v>
+        <v>16.5</v>
       </c>
       <c r="I116" t="n">
-        <v>0.5658333333333333</v>
+        <v>0.4125</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7328,16 +7328,16 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>250</v>
+        <v>1500</v>
       </c>
       <c r="G117" t="n">
-        <v>7.5</v>
+        <v>23.5</v>
       </c>
       <c r="H117" t="n">
-        <v>30</v>
+        <v>15.66666666666667</v>
       </c>
       <c r="I117" t="n">
-        <v>0.75</v>
+        <v>0.3916666666666667</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7377,16 +7377,16 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G118" t="n">
-        <v>12.95</v>
+        <v>5.5</v>
       </c>
       <c r="H118" t="n">
-        <v>25.9</v>
+        <v>22</v>
       </c>
       <c r="I118" t="n">
-        <v>0.6475</v>
+        <v>0.55</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="G119" t="n">
-        <v>18.5</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="H119" t="n">
-        <v>24.66666666666667</v>
+        <v>17.9</v>
       </c>
       <c r="I119" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.4475</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7475,25 +7475,25 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="G120" t="n">
-        <v>13.95</v>
+        <v>12.95</v>
       </c>
       <c r="H120" t="n">
-        <v>46.5</v>
+        <v>17.26666666666667</v>
       </c>
       <c r="I120" t="n">
-        <v>1.1625</v>
+        <v>0.4316666666666666</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7524,16 +7524,16 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G121" t="n">
-        <v>12.5</v>
+        <v>13.95</v>
       </c>
       <c r="H121" t="n">
-        <v>31.25</v>
+        <v>46.5</v>
       </c>
       <c r="I121" t="n">
-        <v>0.78125</v>
+        <v>1.1625</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -7542,56 +7542,56 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>protein_works</t>
+          <t>gymbeam</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>The Protein Works</t>
+          <t>GymBeam</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="G122" t="n">
-        <v>34.99</v>
+        <v>12.5</v>
       </c>
       <c r="H122" t="n">
-        <v>69.98</v>
+        <v>31.25</v>
       </c>
       <c r="I122" t="n">
-        <v>1.7495</v>
+        <v>0.78125</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -7622,16 +7622,16 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G123" t="n">
-        <v>58.99</v>
+        <v>23.99</v>
       </c>
       <c r="H123" t="n">
-        <v>58.99</v>
+        <v>47.98</v>
       </c>
       <c r="I123" t="n">
-        <v>1.47475</v>
+        <v>1.1995</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7657,7 +7657,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7671,16 +7671,16 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G124" t="n">
-        <v>109.99</v>
+        <v>44.99</v>
       </c>
       <c r="H124" t="n">
-        <v>54.995</v>
+        <v>44.99</v>
       </c>
       <c r="I124" t="n">
-        <v>1.374875</v>
+        <v>1.12475</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7689,7 +7689,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7720,20 +7720,20 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>4000</v>
+        <v>500</v>
       </c>
       <c r="G125" t="n">
-        <v>208.49</v>
+        <v>34.99</v>
       </c>
       <c r="H125" t="n">
-        <v>52.1225</v>
+        <v>69.98</v>
       </c>
       <c r="I125" t="n">
-        <v>1.3030625</v>
+        <v>1.7495</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7769,16 +7769,16 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G126" t="n">
-        <v>23.99</v>
+        <v>58.99</v>
       </c>
       <c r="H126" t="n">
-        <v>47.98</v>
+        <v>58.99</v>
       </c>
       <c r="I126" t="n">
-        <v>1.1995</v>
+        <v>1.47475</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7818,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G127" t="n">
-        <v>44.99</v>
+        <v>109.99</v>
       </c>
       <c r="H127" t="n">
-        <v>44.99</v>
+        <v>54.995</v>
       </c>
       <c r="I127" t="n">
-        <v>1.12475</v>
+        <v>1.374875</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7867,25 +7867,25 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>600</v>
+        <v>4000</v>
       </c>
       <c r="G128" t="n">
-        <v>16.99</v>
+        <v>208.49</v>
       </c>
       <c r="H128" t="n">
-        <v>28.31666666666667</v>
+        <v>52.1225</v>
       </c>
       <c r="I128" t="n">
-        <v>0.7079166666666666</v>
+        <v>1.3030625</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="G129" t="n">
-        <v>26.99</v>
+        <v>14.99</v>
       </c>
       <c r="H129" t="n">
-        <v>22.49166666666667</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I129" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>2400</v>
+        <v>1200</v>
       </c>
       <c r="G130" t="n">
-        <v>49.99</v>
+        <v>23.99</v>
       </c>
       <c r="H130" t="n">
-        <v>20.82916666666667</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.5207291666666667</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>4800</v>
+        <v>2400</v>
       </c>
       <c r="G131" t="n">
-        <v>95.98999999999999</v>
+        <v>44.49</v>
       </c>
       <c r="H131" t="n">
-        <v>19.99791666666667</v>
+        <v>18.5375</v>
       </c>
       <c r="I131" t="n">
-        <v>0.4999479166666667</v>
+        <v>0.4634375</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8049,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -8063,16 +8063,16 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>500</v>
+        <v>4800</v>
       </c>
       <c r="G132" t="n">
-        <v>19.99</v>
+        <v>85.48999999999999</v>
       </c>
       <c r="H132" t="n">
-        <v>39.98</v>
+        <v>17.81041666666667</v>
       </c>
       <c r="I132" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.4452604166666667</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8098,7 +8098,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -8112,16 +8112,16 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="G133" t="n">
-        <v>33.99</v>
+        <v>16.99</v>
       </c>
       <c r="H133" t="n">
-        <v>33.99</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I133" t="n">
-        <v>0.84975</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8147,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -8161,16 +8161,16 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="G134" t="n">
-        <v>63.49</v>
+        <v>26.99</v>
       </c>
       <c r="H134" t="n">
-        <v>31.745</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I134" t="n">
-        <v>0.793625</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8196,7 +8196,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8210,16 +8210,16 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>4000</v>
+        <v>2400</v>
       </c>
       <c r="G135" t="n">
-        <v>122.99</v>
+        <v>49.99</v>
       </c>
       <c r="H135" t="n">
-        <v>30.7475</v>
+        <v>20.82916666666667</v>
       </c>
       <c r="I135" t="n">
-        <v>0.7686875</v>
+        <v>0.5207291666666667</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8259,16 +8259,16 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>600</v>
+        <v>4800</v>
       </c>
       <c r="G136" t="n">
-        <v>14.99</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="H136" t="n">
-        <v>24.98333333333333</v>
+        <v>19.99791666666667</v>
       </c>
       <c r="I136" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.4999479166666667</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -8308,16 +8308,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="G137" t="n">
-        <v>23.99</v>
+        <v>17.99</v>
       </c>
       <c r="H137" t="n">
-        <v>19.99166666666667</v>
+        <v>35.98</v>
       </c>
       <c r="I137" t="n">
-        <v>0.4997916666666667</v>
+        <v>0.8995</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8357,16 +8357,16 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>2400</v>
+        <v>1000</v>
       </c>
       <c r="G138" t="n">
-        <v>44.49</v>
+        <v>33.99</v>
       </c>
       <c r="H138" t="n">
-        <v>18.5375</v>
+        <v>33.99</v>
       </c>
       <c r="I138" t="n">
-        <v>0.4634375</v>
+        <v>0.84975</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8406,16 +8406,16 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>4800</v>
+        <v>2000</v>
       </c>
       <c r="G139" t="n">
-        <v>85.48999999999999</v>
+        <v>63.49</v>
       </c>
       <c r="H139" t="n">
-        <v>17.81041666666667</v>
+        <v>31.745</v>
       </c>
       <c r="I139" t="n">
-        <v>0.4452604166666667</v>
+        <v>0.793625</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Whey Protein 360 - Vanilla</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8455,16 +8455,16 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>600</v>
+        <v>4000</v>
       </c>
       <c r="G140" t="n">
-        <v>11.49</v>
+        <v>122.99</v>
       </c>
       <c r="H140" t="n">
-        <v>19.15</v>
+        <v>30.7475</v>
       </c>
       <c r="I140" t="n">
-        <v>0.47875</v>
+        <v>0.7686875</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8504,16 +8504,16 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="G141" t="n">
-        <v>21.19</v>
+        <v>11.49</v>
       </c>
       <c r="H141" t="n">
-        <v>17.65833333333333</v>
+        <v>19.15</v>
       </c>
       <c r="I141" t="n">
-        <v>0.4414583333333333</v>
+        <v>0.47875</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8553,16 +8553,16 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>2400</v>
+        <v>1200</v>
       </c>
       <c r="G142" t="n">
-        <v>39.99</v>
+        <v>21.19</v>
       </c>
       <c r="H142" t="n">
-        <v>16.6625</v>
+        <v>17.65833333333333</v>
       </c>
       <c r="I142" t="n">
-        <v>0.4165625</v>
+        <v>0.4414583333333333</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8602,23 +8602,72 @@
         </is>
       </c>
       <c r="F143" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G143" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="H143" t="n">
+        <v>16.6625</v>
+      </c>
+      <c r="I143" t="n">
+        <v>0.4165625</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>protein_works</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>whey_protein</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Whey Protein 360 - Vanilla</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>The Protein Works</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
         <v>4800</v>
       </c>
-      <c r="G143" t="n">
+      <c r="G144" t="n">
         <v>77.48999999999999</v>
       </c>
-      <c r="H143" t="n">
+      <c r="H144" t="n">
         <v>16.14375</v>
       </c>
-      <c r="I143" t="n">
+      <c r="I144" t="n">
         <v>0.40359375</v>
       </c>
-      <c r="O143" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P143" t="inlineStr">
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
         <is>
           <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-10
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G34" t="n">
-        <v>15.99</v>
+        <v>18.99</v>
       </c>
       <c r="H34" t="n">
-        <v>31.98</v>
+        <v>15.192</v>
       </c>
       <c r="I34" t="n">
-        <v>0.7995</v>
+        <v>0.3798</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3310,16 +3310,16 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G35" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H35" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I35" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3359,16 +3359,16 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G36" t="n">
-        <v>18.99</v>
+        <v>15.99</v>
       </c>
       <c r="H36" t="n">
-        <v>15.192</v>
+        <v>31.98</v>
       </c>
       <c r="I36" t="n">
-        <v>0.3798</v>
+        <v>0.7995</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3408,16 +3408,16 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G37" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H37" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I37" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,25 +6789,25 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G106" t="n">
-        <v>28.95</v>
+        <v>16.5</v>
       </c>
       <c r="H106" t="n">
-        <v>57.9</v>
+        <v>16.5</v>
       </c>
       <c r="I106" t="n">
-        <v>1.4475</v>
+        <v>0.4125</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G107" t="n">
-        <v>16.5</v>
+        <v>31.95</v>
       </c>
       <c r="H107" t="n">
-        <v>16.5</v>
+        <v>12.78</v>
       </c>
       <c r="I107" t="n">
-        <v>0.4125</v>
+        <v>0.3195</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6887,16 +6887,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="G108" t="n">
-        <v>31.95</v>
+        <v>11.95</v>
       </c>
       <c r="H108" t="n">
-        <v>12.78</v>
+        <v>23.9</v>
       </c>
       <c r="I108" t="n">
-        <v>0.3195</v>
+        <v>0.5975</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6939,22 +6939,22 @@
         <v>500</v>
       </c>
       <c r="G109" t="n">
-        <v>11.95</v>
+        <v>22.95</v>
       </c>
       <c r="H109" t="n">
-        <v>23.9</v>
+        <v>45.9</v>
       </c>
       <c r="I109" t="n">
-        <v>0.5975</v>
+        <v>1.1475</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -7625,13 +7625,13 @@
         <v>500</v>
       </c>
       <c r="G123" t="n">
-        <v>23.99</v>
+        <v>35.99</v>
       </c>
       <c r="H123" t="n">
-        <v>47.98</v>
+        <v>71.98</v>
       </c>
       <c r="I123" t="n">
-        <v>1.1995</v>
+        <v>1.7995</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7657,7 +7657,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7674,13 +7674,13 @@
         <v>1000</v>
       </c>
       <c r="G124" t="n">
-        <v>44.99</v>
+        <v>58.99</v>
       </c>
       <c r="H124" t="n">
-        <v>44.99</v>
+        <v>58.99</v>
       </c>
       <c r="I124" t="n">
-        <v>1.12475</v>
+        <v>1.47475</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7689,7 +7689,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7720,16 +7720,16 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G125" t="n">
-        <v>34.99</v>
+        <v>109.99</v>
       </c>
       <c r="H125" t="n">
-        <v>69.98</v>
+        <v>54.995</v>
       </c>
       <c r="I125" t="n">
-        <v>1.7495</v>
+        <v>1.374875</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -7769,20 +7769,20 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="G126" t="n">
-        <v>58.99</v>
+        <v>208.49</v>
       </c>
       <c r="H126" t="n">
-        <v>58.99</v>
+        <v>52.1225</v>
       </c>
       <c r="I126" t="n">
-        <v>1.47475</v>
+        <v>1.3030625</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -7804,7 +7804,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7818,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G127" t="n">
-        <v>109.99</v>
+        <v>23.99</v>
       </c>
       <c r="H127" t="n">
-        <v>54.995</v>
+        <v>47.98</v>
       </c>
       <c r="I127" t="n">
-        <v>1.374875</v>
+        <v>1.1995</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7867,25 +7867,25 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="G128" t="n">
-        <v>208.49</v>
+        <v>44.99</v>
       </c>
       <c r="H128" t="n">
-        <v>52.1225</v>
+        <v>44.99</v>
       </c>
       <c r="I128" t="n">
-        <v>1.3030625</v>
+        <v>1.12475</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7919,13 +7919,13 @@
         <v>600</v>
       </c>
       <c r="G129" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="H129" t="n">
-        <v>24.98333333333333</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I129" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7968,13 +7968,13 @@
         <v>1200</v>
       </c>
       <c r="G130" t="n">
-        <v>23.99</v>
+        <v>26.99</v>
       </c>
       <c r="H130" t="n">
-        <v>19.99166666666667</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.4997916666666667</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8017,13 +8017,13 @@
         <v>2400</v>
       </c>
       <c r="G131" t="n">
-        <v>44.49</v>
+        <v>49.99</v>
       </c>
       <c r="H131" t="n">
-        <v>18.5375</v>
+        <v>20.82916666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.4634375</v>
+        <v>0.5207291666666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8066,13 +8066,13 @@
         <v>4800</v>
       </c>
       <c r="G132" t="n">
-        <v>85.48999999999999</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="H132" t="n">
-        <v>17.81041666666667</v>
+        <v>19.99791666666667</v>
       </c>
       <c r="I132" t="n">
-        <v>0.4452604166666667</v>
+        <v>0.4999479166666667</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8115,13 +8115,13 @@
         <v>600</v>
       </c>
       <c r="G133" t="n">
-        <v>16.99</v>
+        <v>14.99</v>
       </c>
       <c r="H133" t="n">
-        <v>28.31666666666667</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I133" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8164,13 +8164,13 @@
         <v>1200</v>
       </c>
       <c r="G134" t="n">
-        <v>26.99</v>
+        <v>23.99</v>
       </c>
       <c r="H134" t="n">
-        <v>22.49166666666667</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I134" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8213,13 +8213,13 @@
         <v>2400</v>
       </c>
       <c r="G135" t="n">
-        <v>49.99</v>
+        <v>44.49</v>
       </c>
       <c r="H135" t="n">
-        <v>20.82916666666667</v>
+        <v>18.5375</v>
       </c>
       <c r="I135" t="n">
-        <v>0.5207291666666667</v>
+        <v>0.4634375</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8262,13 +8262,13 @@
         <v>4800</v>
       </c>
       <c r="G136" t="n">
-        <v>95.98999999999999</v>
+        <v>85.48999999999999</v>
       </c>
       <c r="H136" t="n">
-        <v>19.99791666666667</v>
+        <v>17.81041666666667</v>
       </c>
       <c r="I136" t="n">
-        <v>0.4999479166666667</v>
+        <v>0.4452604166666667</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-11
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P144"/>
+  <dimension ref="A1:P143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Vanilla 1.25kg</t>
+          <t>Diet Whey Protein - Chocolate 500g</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3261,16 +3261,16 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="G34" t="n">
-        <v>18.99</v>
+        <v>15.99</v>
       </c>
       <c r="H34" t="n">
-        <v>15.192</v>
+        <v>31.98</v>
       </c>
       <c r="I34" t="n">
-        <v>0.3798</v>
+        <v>0.7995</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Basic Whey Protein - Strawberry 2.5kg</t>
+          <t>Diet Whey Protein - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3310,16 +3310,16 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G35" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="H35" t="n">
-        <v>14.396</v>
+        <v>39.99</v>
       </c>
       <c r="I35" t="n">
-        <v>0.3599</v>
+        <v>0.99975</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
+          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 500g</t>
+          <t>Basic Whey Protein - Vanilla 1.25kg</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3359,16 +3359,16 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="G36" t="n">
-        <v>15.99</v>
+        <v>18.99</v>
       </c>
       <c r="H36" t="n">
-        <v>31.98</v>
+        <v>15.192</v>
       </c>
       <c r="I36" t="n">
-        <v>0.7995</v>
+        <v>0.3798</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Diet Whey Protein - Chocolate 1kg</t>
+          <t>Basic Whey Protein - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3408,16 +3408,16 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G37" t="n">
-        <v>39.99</v>
+        <v>35.99</v>
       </c>
       <c r="H37" t="n">
-        <v>39.99</v>
+        <v>14.396</v>
       </c>
       <c r="I37" t="n">
-        <v>0.99975</v>
+        <v>0.3599</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/diet-whey-protein/bble-dwpr</t>
+          <t>https://www.bulk.com/uk/products/basic-whey-protein/bpb-vwhe</t>
         </is>
       </c>
     </row>
@@ -5746,7 +5746,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Protein Gold Whey - Weider 500 g - jahoda</t>
+          <t>BIO Whey Protein - GymBeam 900 g - kakao</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5760,25 +5760,25 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="G85" t="n">
-        <v>19.95</v>
+        <v>45.95</v>
       </c>
       <c r="H85" t="n">
-        <v>39.9</v>
+        <v>51.05555555555556</v>
       </c>
       <c r="I85" t="n">
-        <v>0.9975000000000001</v>
+        <v>1.276388888888889</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-gold-whey-weider.html</t>
+          <t>https://gymbeam.sk/bio-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>BIO Whey Protein - GymBeam 900 g - kakao</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5809,16 +5809,16 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="G86" t="n">
-        <v>45.95</v>
+        <v>37.95</v>
       </c>
       <c r="H86" t="n">
-        <v>51.05555555555556</v>
+        <v>37.95</v>
       </c>
       <c r="I86" t="n">
-        <v>1.276388888888889</v>
+        <v>0.94875</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -5827,7 +5827,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/bio-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 1000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5858,16 +5858,16 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G87" t="n">
-        <v>37.95</v>
+        <v>67.95</v>
       </c>
       <c r="H87" t="n">
-        <v>37.95</v>
+        <v>33.975</v>
       </c>
       <c r="I87" t="n">
-        <v>0.94875</v>
+        <v>0.849375</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 2000 g - bez príchute - 01</t>
+          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5907,16 +5907,16 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G88" t="n">
-        <v>67.95</v>
+        <v>24.95</v>
       </c>
       <c r="H88" t="n">
-        <v>33.975</v>
+        <v>49.9</v>
       </c>
       <c r="I88" t="n">
-        <v>0.849375</v>
+        <v>1.2475</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Just Whey Grass-Fed Protein – GymBeam 500 g - banán - 01</t>
+          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5956,16 +5956,16 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G89" t="n">
-        <v>24.95</v>
+        <v>37.95</v>
       </c>
       <c r="H89" t="n">
-        <v>49.9</v>
+        <v>37.95</v>
       </c>
       <c r="I89" t="n">
-        <v>1.2475</v>
+        <v>0.94875</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -5974,7 +5974,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/just-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 1000 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6005,16 +6005,16 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="G90" t="n">
-        <v>37.95</v>
+        <v>24.95</v>
       </c>
       <c r="H90" t="n">
-        <v>37.95</v>
+        <v>49.9</v>
       </c>
       <c r="I90" t="n">
-        <v>0.94875</v>
+        <v>1.2475</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Proteín Yum Yum Whey - BeastPink 500 g - čokoláda lieskový oriešok</t>
+          <t>Proteín Anabolic Whey - GymBeam 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6054,16 +6054,16 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G91" t="n">
-        <v>24.95</v>
+        <v>21.95</v>
       </c>
       <c r="H91" t="n">
-        <v>49.9</v>
+        <v>21.95</v>
       </c>
       <c r="I91" t="n">
-        <v>1.2475</v>
+        <v>0.54875</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -6072,7 +6072,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/yum-yum-whey-beastpink-darceky.html</t>
+          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Proteín Anabolic Whey - GymBeam 1000 g - čokoláda</t>
+          <t>Proteín Anabolic Whey - GymBeam 2500 g - čokoláda</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6103,16 +6103,16 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G92" t="n">
-        <v>21.95</v>
+        <v>52.95</v>
       </c>
       <c r="H92" t="n">
-        <v>21.95</v>
+        <v>21.18</v>
       </c>
       <c r="I92" t="n">
-        <v>0.54875</v>
+        <v>0.5295</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Proteín Anabolic Whey - GymBeam 2500 g - čokoláda</t>
+          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6152,16 +6152,16 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="G93" t="n">
-        <v>52.95</v>
+        <v>31.95</v>
       </c>
       <c r="H93" t="n">
-        <v>21.18</v>
+        <v>31.95</v>
       </c>
       <c r="I93" t="n">
-        <v>0.5295</v>
+        <v>0.79875</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -6170,7 +6170,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/protein-anabolic-whey-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 1000 g - čokoláda</t>
+          <t>Whey Proteín - Mammut Nutrition 3000 g - čokoláda</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6201,16 +6201,16 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="G94" t="n">
-        <v>31.95</v>
+        <v>93.95</v>
       </c>
       <c r="H94" t="n">
-        <v>31.95</v>
+        <v>31.31666666666667</v>
       </c>
       <c r="I94" t="n">
-        <v>0.79875</v>
+        <v>0.7829166666666667</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whey Proteín - Mammut Nutrition 3000 g - čokoláda</t>
+          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6250,25 +6250,25 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G95" t="n">
-        <v>93.95</v>
+        <v>21.95</v>
       </c>
       <c r="H95" t="n">
-        <v>31.31666666666667</v>
+        <v>43.9</v>
       </c>
       <c r="I95" t="n">
-        <v>0.7829166666666667</v>
+        <v>1.0975</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-mammut-nutrition.html</t>
+          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
         </is>
       </c>
     </row>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Whey Proteín - GYMQUEEN banán - 500 g</t>
+          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6299,16 +6299,16 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G96" t="n">
-        <v>21.95</v>
+        <v>34.95</v>
       </c>
       <c r="H96" t="n">
-        <v>43.9</v>
+        <v>34.95</v>
       </c>
       <c r="I96" t="n">
-        <v>1.0975</v>
+        <v>0.87375</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6317,7 +6317,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-gymqueen.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 1000 g - karamelové macchiato</t>
+          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6348,16 +6348,16 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G97" t="n">
-        <v>34.95</v>
+        <v>62.95</v>
       </c>
       <c r="H97" t="n">
-        <v>34.95</v>
+        <v>31.475</v>
       </c>
       <c r="I97" t="n">
-        <v>0.87375</v>
+        <v>0.786875</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 2000 g - karamelové macchiato</t>
+          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6397,16 +6397,16 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G98" t="n">
-        <v>62.95</v>
+        <v>19.5</v>
       </c>
       <c r="H98" t="n">
-        <v>31.475</v>
+        <v>39</v>
       </c>
       <c r="I98" t="n">
-        <v>0.786875</v>
+        <v>0.975</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - The Protein Works 500 g - karamelové macchiato</t>
+          <t>Whey Protein - Bodylab24 1000 g - banán</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6446,16 +6446,16 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G99" t="n">
-        <v>19.5</v>
+        <v>39.95</v>
       </c>
       <c r="H99" t="n">
-        <v>39</v>
+        <v>39.95</v>
       </c>
       <c r="I99" t="n">
-        <v>0.975</v>
+        <v>0.99875</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-the-protein-works.html</t>
+          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 1000 g - banán</t>
+          <t>Whey Protein - Bodylab24 2000 g - banán</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6495,16 +6495,16 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G100" t="n">
-        <v>39.95</v>
+        <v>64.95</v>
       </c>
       <c r="H100" t="n">
-        <v>39.95</v>
+        <v>32.475</v>
       </c>
       <c r="I100" t="n">
-        <v>0.99875</v>
+        <v>0.811875</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Whey Protein - Bodylab24 2000 g - banán</t>
+          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6544,16 +6544,16 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>2000</v>
+        <v>400</v>
       </c>
       <c r="G101" t="n">
-        <v>64.95</v>
+        <v>42.95</v>
       </c>
       <c r="H101" t="n">
-        <v>32.475</v>
+        <v>107.375</v>
       </c>
       <c r="I101" t="n">
-        <v>0.811875</v>
+        <v>2.684375</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-bodylab24.html</t>
+          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>BIO Whey Protein Lactose Free - Purasana čokoláda - 400 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6593,16 +6593,16 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>400</v>
+        <v>1200</v>
       </c>
       <c r="G102" t="n">
-        <v>42.95</v>
+        <v>34.95</v>
       </c>
       <c r="H102" t="n">
-        <v>107.375</v>
+        <v>29.125</v>
       </c>
       <c r="I102" t="n">
-        <v>2.684375</v>
+        <v>0.728125</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -6611,7 +6611,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/bio-whey-protein-lactose-free-purasana.html</t>
+          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 1200 g</t>
+          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6642,16 +6642,16 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G103" t="n">
-        <v>34.95</v>
+        <v>62.95</v>
       </c>
       <c r="H103" t="n">
-        <v>29.125</v>
+        <v>26.22916666666667</v>
       </c>
       <c r="I103" t="n">
-        <v>0.728125</v>
+        <v>0.6557291666666667</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -6677,7 +6677,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works narodeninová torta - 2400 g</t>
+          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6691,20 +6691,20 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>2400</v>
+        <v>600</v>
       </c>
       <c r="G104" t="n">
-        <v>62.95</v>
+        <v>19.5</v>
       </c>
       <c r="H104" t="n">
-        <v>26.22916666666667</v>
+        <v>32.5</v>
       </c>
       <c r="I104" t="n">
-        <v>0.6557291666666667</v>
+        <v>0.8125</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Whey Protein 360 ® - The Protein Works jahoda &amp; krém - 600 g</t>
+          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,16 +6740,16 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="G105" t="n">
-        <v>19.5</v>
+        <v>22.95</v>
       </c>
       <c r="H105" t="n">
-        <v>32.5</v>
+        <v>45.9</v>
       </c>
       <c r="I105" t="n">
-        <v>0.8125</v>
+        <v>1.1475</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-360-r-the-protein-works.html</t>
+          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6922,7 +6922,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
+          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6936,16 +6936,16 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>500</v>
+        <v>1450</v>
       </c>
       <c r="G109" t="n">
-        <v>22.95</v>
+        <v>39.95</v>
       </c>
       <c r="H109" t="n">
-        <v>45.9</v>
+        <v>27.55172413793104</v>
       </c>
       <c r="I109" t="n">
-        <v>1.1475</v>
+        <v>0.6887931034482758</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -6966,12 +6966,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>whey_protein</t>
+          <t>creatine_monohydrate</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ReFuel Whey Protein - GymBeam 1450 g - čokoláda</t>
+          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6985,16 +6985,16 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1450</v>
+        <v>400</v>
       </c>
       <c r="G110" t="n">
-        <v>39.95</v>
+        <v>10.95</v>
       </c>
       <c r="H110" t="n">
-        <v>27.55172413793104</v>
+        <v>27.375</v>
       </c>
       <c r="I110" t="n">
-        <v>0.6887931034482758</v>
+        <v>0.684375</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/refuel-whey-protein-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Creatine monohydrate+ - GymBeam 400 g - zelené jablko</t>
+          <t>Creatine Monohydrate - Amix 1000 g</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7034,16 +7034,16 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="G111" t="n">
-        <v>10.95</v>
+        <v>33.95</v>
       </c>
       <c r="H111" t="n">
-        <v>27.375</v>
+        <v>33.95</v>
       </c>
       <c r="I111" t="n">
-        <v>0.684375</v>
+        <v>0.84875</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-performance-gymbeam.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 1000 g</t>
+          <t>Creatine Monohydrate - Amix 300 g</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7083,16 +7083,16 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="G112" t="n">
-        <v>33.95</v>
+        <v>14.95</v>
       </c>
       <c r="H112" t="n">
-        <v>33.95</v>
+        <v>49.83333333333334</v>
       </c>
       <c r="I112" t="n">
-        <v>0.84875</v>
+        <v>1.245833333333333</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 300 g</t>
+          <t>Creatine Monohydrate - Amix 500 g</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7132,16 +7132,16 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G113" t="n">
-        <v>14.95</v>
+        <v>18.5</v>
       </c>
       <c r="H113" t="n">
-        <v>49.83333333333334</v>
+        <v>37</v>
       </c>
       <c r="I113" t="n">
-        <v>1.245833333333333</v>
+        <v>0.925</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - Amix 500 g</t>
+          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7184,22 +7184,22 @@
         <v>500</v>
       </c>
       <c r="G114" t="n">
-        <v>18.5</v>
+        <v>12.95</v>
       </c>
       <c r="H114" t="n">
-        <v>37</v>
+        <v>25.9</v>
       </c>
       <c r="I114" t="n">
-        <v>0.925</v>
+        <v>0.6475</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-amix.html</t>
+          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Creatine Monohydrate - GoNutrition bez príchute - 500 g</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7230,25 +7230,25 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G115" t="n">
-        <v>12.95</v>
+        <v>16.5</v>
       </c>
       <c r="H115" t="n">
-        <v>25.9</v>
+        <v>16.5</v>
       </c>
       <c r="I115" t="n">
-        <v>0.6475</v>
+        <v>0.4125</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-monohydrate-gonutrition.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1000 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7279,16 +7279,16 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G116" t="n">
-        <v>16.5</v>
+        <v>23.5</v>
       </c>
       <c r="H116" t="n">
-        <v>16.5</v>
+        <v>15.66666666666667</v>
       </c>
       <c r="I116" t="n">
-        <v>0.4125</v>
+        <v>0.3916666666666667</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 1500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7328,16 +7328,16 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>1500</v>
+        <v>250</v>
       </c>
       <c r="G117" t="n">
-        <v>23.5</v>
+        <v>5.5</v>
       </c>
       <c r="H117" t="n">
-        <v>15.66666666666667</v>
+        <v>22</v>
       </c>
       <c r="I117" t="n">
-        <v>0.3916666666666667</v>
+        <v>0.55</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 250 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7377,16 +7377,16 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="G118" t="n">
-        <v>5.5</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="H118" t="n">
-        <v>22</v>
+        <v>17.9</v>
       </c>
       <c r="I118" t="n">
-        <v>0.55</v>
+        <v>0.4475</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 500 g - zelené jablko - 01</t>
+          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="G119" t="n">
-        <v>8.949999999999999</v>
+        <v>12.95</v>
       </c>
       <c r="H119" t="n">
-        <v>17.9</v>
+        <v>17.26666666666667</v>
       </c>
       <c r="I119" t="n">
-        <v>0.4475</v>
+        <v>0.4316666666666666</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>100 % Kreatín monohydrát - GymBeam 750 g - zelené jablko - 01</t>
+          <t>Kreatín monohydrát - Redcon1 300 g</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7475,25 +7475,25 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>750</v>
+        <v>300</v>
       </c>
       <c r="G120" t="n">
-        <v>12.95</v>
+        <v>13.95</v>
       </c>
       <c r="H120" t="n">
-        <v>17.26666666666667</v>
+        <v>46.5</v>
       </c>
       <c r="I120" t="n">
-        <v>0.4316666666666666</v>
+        <v>1.1625</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Kreatín monohydrát - Redcon1 300 g</t>
+          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7524,16 +7524,16 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="G121" t="n">
-        <v>13.95</v>
+        <v>12.5</v>
       </c>
       <c r="H121" t="n">
-        <v>46.5</v>
+        <v>31.25</v>
       </c>
       <c r="I121" t="n">
-        <v>1.1625</v>
+        <v>0.78125</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -7542,56 +7542,56 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/kreatin-monohydrat-redcon1.html</t>
+          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>gymbeam</t>
+          <t>protein_works</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>creatine_monohydrate</t>
+          <t>whey_protein</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Kreatín Pure monohydrát - Bodylab 400 g</t>
+          <t>Diet Whey Protein Isolate</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>GymBeam</t>
+          <t>The Protein Works</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="G122" t="n">
-        <v>12.5</v>
+        <v>34.99</v>
       </c>
       <c r="H122" t="n">
-        <v>31.25</v>
+        <v>69.98</v>
       </c>
       <c r="I122" t="n">
-        <v>0.78125</v>
+        <v>1.7495</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/creatine-pure-monohydrate-bodylab.html</t>
+          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
         </is>
       </c>
     </row>
@@ -7622,16 +7622,16 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G123" t="n">
-        <v>35.99</v>
+        <v>58.99</v>
       </c>
       <c r="H123" t="n">
-        <v>71.98</v>
+        <v>58.99</v>
       </c>
       <c r="I123" t="n">
-        <v>1.7995</v>
+        <v>1.47475</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -7671,16 +7671,16 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G124" t="n">
-        <v>58.99</v>
+        <v>109.99</v>
       </c>
       <c r="H124" t="n">
-        <v>58.99</v>
+        <v>54.995</v>
       </c>
       <c r="I124" t="n">
-        <v>1.47475</v>
+        <v>1.374875</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -7720,20 +7720,20 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="G125" t="n">
-        <v>109.99</v>
+        <v>208.49</v>
       </c>
       <c r="H125" t="n">
-        <v>54.995</v>
+        <v>52.1225</v>
       </c>
       <c r="I125" t="n">
-        <v>1.374875</v>
+        <v>1.3030625</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Diet Whey Protein Isolate</t>
+          <t>Clear Diet Whey Protein Protein</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7769,25 +7769,25 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>4000</v>
+        <v>500</v>
       </c>
       <c r="G126" t="n">
-        <v>208.49</v>
+        <v>23.99</v>
       </c>
       <c r="H126" t="n">
-        <v>52.1225</v>
+        <v>47.98</v>
       </c>
       <c r="I126" t="n">
-        <v>1.3030625</v>
+        <v>1.1995</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-90-isolate-january</t>
+          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
         </is>
       </c>
     </row>
@@ -7818,16 +7818,16 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G127" t="n">
-        <v>23.99</v>
+        <v>44.99</v>
       </c>
       <c r="H127" t="n">
-        <v>47.98</v>
+        <v>44.99</v>
       </c>
       <c r="I127" t="n">
-        <v>1.1995</v>
+        <v>1.12475</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Clear Diet Whey Protein Protein</t>
+          <t>Whey Protein 360</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7867,16 +7867,16 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="G128" t="n">
-        <v>44.99</v>
+        <v>14.99</v>
       </c>
       <c r="H128" t="n">
-        <v>44.99</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I128" t="n">
-        <v>1.12475</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/clear-diet-whey-protein</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7916,16 +7916,16 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G129" t="n">
-        <v>16.99</v>
+        <v>23.99</v>
       </c>
       <c r="H129" t="n">
-        <v>28.31666666666667</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I129" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -7965,16 +7965,16 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G130" t="n">
-        <v>26.99</v>
+        <v>44.49</v>
       </c>
       <c r="H130" t="n">
-        <v>22.49166666666667</v>
+        <v>18.5375</v>
       </c>
       <c r="I130" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.4634375</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8014,16 +8014,16 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G131" t="n">
-        <v>49.99</v>
+        <v>85.48999999999999</v>
       </c>
       <c r="H131" t="n">
-        <v>20.82916666666667</v>
+        <v>17.81041666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.5207291666666667</v>
+        <v>0.4452604166666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8063,16 +8063,16 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>4800</v>
+        <v>600</v>
       </c>
       <c r="G132" t="n">
-        <v>95.98999999999999</v>
+        <v>16.99</v>
       </c>
       <c r="H132" t="n">
-        <v>19.99791666666667</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I132" t="n">
-        <v>0.4999479166666667</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8112,16 +8112,16 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G133" t="n">
-        <v>14.99</v>
+        <v>26.99</v>
       </c>
       <c r="H133" t="n">
-        <v>24.98333333333333</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I133" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8161,16 +8161,16 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G134" t="n">
-        <v>23.99</v>
+        <v>49.99</v>
       </c>
       <c r="H134" t="n">
-        <v>19.99166666666667</v>
+        <v>20.82916666666667</v>
       </c>
       <c r="I134" t="n">
-        <v>0.4997916666666667</v>
+        <v>0.5207291666666667</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8210,16 +8210,16 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G135" t="n">
-        <v>44.49</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="H135" t="n">
-        <v>18.5375</v>
+        <v>19.99791666666667</v>
       </c>
       <c r="I135" t="n">
-        <v>0.4634375</v>
+        <v>0.4999479166666667</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8245,7 +8245,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Whey Protein 360</t>
+          <t>Whey Protein 80</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -8259,16 +8259,16 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>4800</v>
+        <v>500</v>
       </c>
       <c r="G136" t="n">
-        <v>85.48999999999999</v>
+        <v>17.99</v>
       </c>
       <c r="H136" t="n">
-        <v>17.81041666666667</v>
+        <v>35.98</v>
       </c>
       <c r="I136" t="n">
-        <v>0.4452604166666667</v>
+        <v>0.8995</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
         </is>
       </c>
     </row>
@@ -8308,16 +8308,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G137" t="n">
-        <v>17.99</v>
+        <v>33.99</v>
       </c>
       <c r="H137" t="n">
-        <v>35.98</v>
+        <v>33.99</v>
       </c>
       <c r="I137" t="n">
-        <v>0.8995</v>
+        <v>0.84975</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -8357,16 +8357,16 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G138" t="n">
-        <v>33.99</v>
+        <v>63.49</v>
       </c>
       <c r="H138" t="n">
-        <v>33.99</v>
+        <v>31.745</v>
       </c>
       <c r="I138" t="n">
-        <v>0.84975</v>
+        <v>0.793625</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -8406,16 +8406,16 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="G139" t="n">
-        <v>63.49</v>
+        <v>122.99</v>
       </c>
       <c r="H139" t="n">
-        <v>31.745</v>
+        <v>30.7475</v>
       </c>
       <c r="I139" t="n">
-        <v>0.793625</v>
+        <v>0.7686875</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Whey Protein 80</t>
+          <t>Whey Protein 360 - Vanilla</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8455,16 +8455,16 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>4000</v>
+        <v>600</v>
       </c>
       <c r="G140" t="n">
-        <v>122.99</v>
+        <v>11.49</v>
       </c>
       <c r="H140" t="n">
-        <v>30.7475</v>
+        <v>19.15</v>
       </c>
       <c r="I140" t="n">
-        <v>0.7686875</v>
+        <v>0.47875</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-80-concentrate</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>
       </c>
     </row>
@@ -8504,16 +8504,16 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G141" t="n">
-        <v>11.49</v>
+        <v>21.19</v>
       </c>
       <c r="H141" t="n">
-        <v>19.15</v>
+        <v>17.65833333333333</v>
       </c>
       <c r="I141" t="n">
-        <v>0.47875</v>
+        <v>0.4414583333333333</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -8553,16 +8553,16 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="G142" t="n">
-        <v>21.19</v>
+        <v>39.99</v>
       </c>
       <c r="H142" t="n">
-        <v>17.65833333333333</v>
+        <v>16.6625</v>
       </c>
       <c r="I142" t="n">
-        <v>0.4414583333333333</v>
+        <v>0.4165625</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8602,16 +8602,16 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="G143" t="n">
-        <v>39.99</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="H143" t="n">
-        <v>16.6625</v>
+        <v>16.14375</v>
       </c>
       <c r="I143" t="n">
-        <v>0.4165625</v>
+        <v>0.40359375</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -8619,55 +8619,6 @@
         </is>
       </c>
       <c r="P143" t="inlineStr">
-        <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>protein_works</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>whey_protein</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Whey Protein 360 - Vanilla</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>The Protein Works</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="F144" t="n">
-        <v>4800</v>
-      </c>
-      <c r="G144" t="n">
-        <v>77.48999999999999</v>
-      </c>
-      <c r="H144" t="n">
-        <v>16.14375</v>
-      </c>
-      <c r="I144" t="n">
-        <v>0.40359375</v>
-      </c>
-      <c r="O144" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="P144" t="inlineStr">
         <is>
           <t>https://www.theproteinworks.com/whey-protein-360-black-innovation</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): nightly refresh 2026-09-12
</commit_message>
<xml_diff>
--- a/artifacts/reports/report.xlsx
+++ b/artifacts/reports/report.xlsx
@@ -1875,7 +1875,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pure Whey Isolate™ - Chocolate 500g</t>
+          <t>Pure Whey Isolate™ - Strawberry 500g</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pure Whey Isolate™ - Chocolate 2.5kg</t>
+          <t>Pure Whey Isolate™ - Strawberry 2.5kg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pure Whey Isolate™ - Chocolate 5kg</t>
+          <t>Pure Whey Isolate™ - Strawberry 5kg</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
+          <t>Natural Pure Whey Isolate™ - Chocolate 500g</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2477,25 +2477,25 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2270</v>
+        <v>500</v>
       </c>
       <c r="G18" t="n">
-        <v>79.98999999999999</v>
+        <v>25.99</v>
       </c>
       <c r="H18" t="n">
-        <v>35.23788546255506</v>
+        <v>51.98</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8809471365638767</v>
+        <v>1.2995</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
+          <t>https://www.bulk.com/uk/products/natural-pure-whey-isolate-90/bpb-npwi</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Isolate™ - Chocolate 500g</t>
+          <t>Natural Pure Whey Isolate™ - Chocolate 1kg</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2526,16 +2526,16 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G19" t="n">
-        <v>25.99</v>
+        <v>49.99</v>
       </c>
       <c r="H19" t="n">
-        <v>51.98</v>
+        <v>49.99</v>
       </c>
       <c r="I19" t="n">
-        <v>1.2995</v>
+        <v>1.24975</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Isolate™ - Chocolate 1kg</t>
+          <t>Natural Pure Whey Isolate™ - Chocolate 2.5kg</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2575,16 +2575,16 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G20" t="n">
-        <v>49.99</v>
+        <v>111.99</v>
       </c>
       <c r="H20" t="n">
-        <v>49.99</v>
+        <v>44.796</v>
       </c>
       <c r="I20" t="n">
-        <v>1.24975</v>
+        <v>1.1199</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Isolate™ - Chocolate 2.5kg</t>
+          <t>Natural Pure Whey Isolate™ - Chocolate 5kg</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2624,20 +2624,20 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="G21" t="n">
-        <v>111.99</v>
+        <v>209.99</v>
       </c>
       <c r="H21" t="n">
-        <v>44.796</v>
+        <v>41.998</v>
       </c>
       <c r="I21" t="n">
-        <v>1.1199</v>
+        <v>1.04995</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Natural Pure Whey Isolate™ - Chocolate 5kg</t>
+          <t>Informed Whey Protein - Double Chocolate 2.27kg</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2673,16 +2673,16 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5000</v>
+        <v>2270</v>
       </c>
       <c r="G22" t="n">
-        <v>209.99</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>41.998</v>
+        <v>35.23788546255506</v>
       </c>
       <c r="I22" t="n">
-        <v>1.04995</v>
+        <v>0.8809471365638767</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>https://www.bulk.com/uk/products/natural-pure-whey-isolate-90/bpb-npwi</t>
+          <t>https://www.bulk.com/uk/products/informed-whey/bpps-iwhe</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Proteín Pure IsoWhey - GymBeam 2500 g - čokoláda - 00</t>
+          <t>Proteín Pure IsoWhey - GymBeam 2500 g - slaný karamel - 00</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
+          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6740,25 +6740,25 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G105" t="n">
-        <v>22.95</v>
+        <v>16.5</v>
       </c>
       <c r="H105" t="n">
-        <v>45.9</v>
+        <v>16.5</v>
       </c>
       <c r="I105" t="n">
-        <v>1.1475</v>
+        <v>0.4125</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>in_stock</t>
+          <t>out_of_stock</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
+          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition caffe latte - 1000 g</t>
+          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6789,16 +6789,16 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G106" t="n">
-        <v>16.5</v>
+        <v>31.95</v>
       </c>
       <c r="H106" t="n">
-        <v>16.5</v>
+        <v>12.78</v>
       </c>
       <c r="I106" t="n">
-        <v>0.4125</v>
+        <v>0.3195</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition čokoláda banán - 2500 g</t>
+          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="G107" t="n">
-        <v>31.95</v>
+        <v>11.95</v>
       </c>
       <c r="H107" t="n">
-        <v>12.78</v>
+        <v>23.9</v>
       </c>
       <c r="I107" t="n">
-        <v>0.3195</v>
+        <v>0.5975</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Whey Protein 80 - GoNutrition trojitá čokoláda - 500 g</t>
+          <t>Proteín Clear Whey Hydrate - GymBeam 500 g - zelené jablko</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6890,22 +6890,22 @@
         <v>500</v>
       </c>
       <c r="G108" t="n">
-        <v>11.95</v>
+        <v>22.95</v>
       </c>
       <c r="H108" t="n">
-        <v>23.9</v>
+        <v>45.9</v>
       </c>
       <c r="I108" t="n">
-        <v>0.5975</v>
+        <v>1.1475</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>out_of_stock</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>https://gymbeam.sk/whey-protein-80-gonutrition.html</t>
+          <t>https://gymbeam.sk/clear-whey-hydrate-gymbeam.html</t>
         </is>
       </c>
     </row>
@@ -7870,13 +7870,13 @@
         <v>600</v>
       </c>
       <c r="G128" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="H128" t="n">
-        <v>24.98333333333333</v>
+        <v>28.31666666666667</v>
       </c>
       <c r="I128" t="n">
-        <v>0.6245833333333334</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7919,13 +7919,13 @@
         <v>1200</v>
       </c>
       <c r="G129" t="n">
-        <v>23.99</v>
+        <v>26.99</v>
       </c>
       <c r="H129" t="n">
-        <v>19.99166666666667</v>
+        <v>22.49166666666667</v>
       </c>
       <c r="I129" t="n">
-        <v>0.4997916666666667</v>
+        <v>0.5622916666666666</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -7968,13 +7968,13 @@
         <v>2400</v>
       </c>
       <c r="G130" t="n">
-        <v>44.49</v>
+        <v>49.99</v>
       </c>
       <c r="H130" t="n">
-        <v>18.5375</v>
+        <v>20.82916666666667</v>
       </c>
       <c r="I130" t="n">
-        <v>0.4634375</v>
+        <v>0.5207291666666667</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8017,13 +8017,13 @@
         <v>4800</v>
       </c>
       <c r="G131" t="n">
-        <v>85.48999999999999</v>
+        <v>95.98999999999999</v>
       </c>
       <c r="H131" t="n">
-        <v>17.81041666666667</v>
+        <v>19.99791666666667</v>
       </c>
       <c r="I131" t="n">
-        <v>0.4452604166666667</v>
+        <v>0.4999479166666667</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360</t>
+          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
         </is>
       </c>
     </row>
@@ -8066,13 +8066,13 @@
         <v>600</v>
       </c>
       <c r="G132" t="n">
-        <v>16.99</v>
+        <v>14.99</v>
       </c>
       <c r="H132" t="n">
-        <v>28.31666666666667</v>
+        <v>24.98333333333333</v>
       </c>
       <c r="I132" t="n">
-        <v>0.7079166666666666</v>
+        <v>0.6245833333333334</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8115,13 +8115,13 @@
         <v>1200</v>
       </c>
       <c r="G133" t="n">
-        <v>26.99</v>
+        <v>23.99</v>
       </c>
       <c r="H133" t="n">
-        <v>22.49166666666667</v>
+        <v>19.99166666666667</v>
       </c>
       <c r="I133" t="n">
-        <v>0.5622916666666666</v>
+        <v>0.4997916666666667</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8164,13 +8164,13 @@
         <v>2400</v>
       </c>
       <c r="G134" t="n">
-        <v>49.99</v>
+        <v>44.49</v>
       </c>
       <c r="H134" t="n">
-        <v>20.82916666666667</v>
+        <v>18.5375</v>
       </c>
       <c r="I134" t="n">
-        <v>0.5207291666666667</v>
+        <v>0.4634375</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>
@@ -8213,13 +8213,13 @@
         <v>4800</v>
       </c>
       <c r="G135" t="n">
-        <v>95.98999999999999</v>
+        <v>85.48999999999999</v>
       </c>
       <c r="H135" t="n">
-        <v>19.99791666666667</v>
+        <v>17.81041666666667</v>
       </c>
       <c r="I135" t="n">
-        <v>0.4999479166666667</v>
+        <v>0.4452604166666667</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>https://www.theproteinworks.com/whey-protein-360-extreme</t>
+          <t>https://www.theproteinworks.com/whey-protein-360</t>
         </is>
       </c>
     </row>

</xml_diff>